<commit_message>
Data files appended for lower RAM
</commit_message>
<xml_diff>
--- a/5-SentenceTransformerResultsforCalls.xlsx
+++ b/5-SentenceTransformerResultsforCalls.xlsx
@@ -498,7 +498,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['support smes', 'social development', 'agile green', 'small medium enterprises', 'software development processes', 'social media support', 'performance arts', 'green building technologies', 'environmental sustainability', 'migration', 'transition csa', 'community development', 'parenting', 'sustainable development', 'green finance', 'programme sustainable', 'transition programme', 'sustainability', 'transform support', 'sustainable transition', 'green enterprise', 'software development', 'policy analysis', 'change innovation.', 'sustainability transition', 'digital transformation', 'stage sustainability', 'transition agile', 'social media support tools', 'child development', 'smes sustainability', 'csa stage', 'green consensus', 'accreditation', 'innovate transform', 'leadership', 'green technologies', 'design sustainability', 'ngo', 'data transformation']</t>
+          <t>['support smes', 'sustainability', 'green building technologies', 'design sustainability', 'innovate transform', 'software development processes', 'green technologies', 'transition programme', 'environmental sustainability', 'green enterprise', 'sustainability transition', 'social media support', 'migration', 'small medium enterprises', 'change innovation.', 'data transformation', 'policy analysis', 'child development', 'smes sustainability', 'community development', 'programme sustainable', 'sustainable development', 'transform support', 'accreditation', 'leadership', 'agile green', 'social development', 'digital transformation', 'stage sustainability', 'performance arts', 'parenting', 'transition agile', 'transition csa', 'csa stage', 'sustainable transition', 'software development', 'green consensus', 'social media support tools', 'green finance', 'ngo']</t>
         </is>
       </c>
     </row>
@@ -535,7 +535,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>['plan innovation', 'permanently open', 'strategic business management', 'urbanization', 'urban planning', 'planning design', 'biotechnology innovation', 'mobility business', 'targeted innovation', 'city', 'entrepreneurship', 'eit urban', 'durability', 'victimology', 'open data', 'open call', 'software development', 'change innovation.', 'urban design', 'teleworking', 'call targeted', 'biotech innovation', 'open banking', 'social entrepreneurship', 'victimization harm', 'plan permanently', 'software project management', 'innovation projects', 'business plan', 'projects eit', 'eco-design', 'business model studies', 'urban mobility', 'business history']</t>
+          <t>['biotech innovation', 'business history', 'call targeted', 'business model studies', 'durability', 'urban mobility', 'eit urban', 'change innovation.', 'open call', 'city', 'software project management', 'urbanization', 'urban design', 'mobility business', 'teleworking', 'social entrepreneurship', 'business plan', 'plan permanently', 'projects eit', 'entrepreneurship', 'eco-design', 'strategic business management', 'biotechnology innovation', 'urban planning', 'victimization harm', 'victimology', 'plan innovation', 'software development', 'open data', 'innovation projects', 'planning design', 'permanently open', 'open banking', 'targeted innovation']</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>['system dynamics', 'planet climate', 'reshaping food', 'choices european', 'food innovations', 'biological systems', 'fostering food', 'political systems', 'local food', 'environmental sustainability', 'control systems', 'parenting', 'sustainable development', 'food systems', 'future food', 'climate change', 'climate adaptation', 'systems reshaping', 'sustainability', 'human behavior', 'social media innovation', 'climate', 'information systems', 'european union', 'food system', 'people planet', 'space collaboration', 'multidimensional scaling', 'change innovation.', 'food waste', 'interactions fostering', 'alternative organizations', 'communication', 'systems people', 'transforming food', 'space colonization', 'european integration', 'system interactions', 'empowering sustainable', 'sustainable future', 'climate transforming', 'nutritional biotechnology', 'europeanization', 'sustainable agriculture', 'food choices', 'food chemistry', 'food heritage', 'innovations empowering', 'european partnership', 'social cohesion', 'system design', 'sustainable food', 'partnership sustainable', 'systems theory', 'functional foods', 'sustainable consumption', 'planetary science']</t>
+          <t>['multidimensional scaling', 'food heritage', 'space colonization', 'information systems', 'functional foods', 'sustainability', 'climate adaptation', 'human behavior', 'environmental sustainability', 'future food', 'europeanization', 'nutritional biotechnology', 'food chemistry', 'change innovation.', 'innovations empowering', 'planetary science', 'european integration', 'food waste', 'sustainable development', 'food choices', 'people planet', 'food system', 'sustainable consumption', 'biological systems', 'systems theory', 'climate', 'social media innovation', 'transforming food', 'reshaping food', 'communication', 'food innovations', 'planet climate', 'european partnership', 'space collaboration', 'sustainable agriculture', 'parenting', 'fostering food', 'empowering sustainable', 'systems people', 'food systems', 'choices european', 'climate change', 'local food', 'climate transforming', 'sustainable food', 'systems reshaping', 'control systems', 'sustainable future', 'system design', 'partnership sustainable', 'european union', 'political systems', 'system dynamics', 'social cohesion', 'interactions fostering', 'alternative organizations', 'system interactions']</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>['small medium enterprises', 'call startups', 'strategic business management', 'biodegradable materials', 'urban planning', 'biomaterials', 'raw materials', 'eit raw', 'scandinavian cinema', 'entrepreneurship', 'telemedicine', 'rawmaterials booster', 'actuary', 'teleworking', 'd esign education', 'booster call', 'startups smes', 'materials business', 'rewarding', 'plan eit', 'eit rawmaterials', 'materials science', 'material design behavior', 'd esign management', 'eit rawmatrials', 'smes eit', 'tissue engineering regenerative medicine', 'composite materials', 'rawmatrials business', 'biotech startups', 'business plan', 'renewable materials', 'evaluation', 'transmedia', 'material based design', 'business model studies', 'technical textiles', 'business history']</t>
+          <t>['evaluation', 'rawmaterials booster', 'business history', 'business model studies', 'biotech startups', 'scandinavian cinema', 'materials business', 'rawmatrials business', 'biodegradable materials', 'rewarding', 'material based design', 'telemedicine', 'small medium enterprises', 'd esign education', 'd esign management', 'booster call', 'actuary', 'eit rawmatrials', 'eit rawmaterials', 'eit raw', 'call startups', 'transmedia', 'materials science', 'material design behavior', 'business plan', 'teleworking', 'biomaterials', 'tissue engineering regenerative medicine', 'entrepreneurship', 'strategic business management', 'urban planning', 'renewable materials', 'technical textiles', 'plan eit', 'composite materials', 'raw materials', 'startups smes', 'smes eit']</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>['strategic business management', 'biodegradable materials', 'urban planning', 'biomaterials', 'raw materials', 'eit raw', 'scandinavian cinema', 'upscaling eit', 'kava call', 'multidimensional scaling', 'actuary', 'teleworking', 'd esign education', 'preoperative measurement', 'call upscaling', 'materials business', 'plan eit', 'eit rawmaterials', 'materials science', 'material design behavior', 'europeanization', 'eit rawmatrials', 'digitization', 'composite materials', 'rawmatrials business', 'business plan', 'renewable materials', 'rawmaterials kava', 'evaluation', 'transmedia', 'form', 'material based design', 'business model studies', 'technical textiles', 'business history']</t>
+          <t>['multidimensional scaling', 'call upscaling', 'evaluation', 'business history', 'business model studies', 'scandinavian cinema', 'materials business', 'rawmatrials business', 'biodegradable materials', 'europeanization', 'material based design', 'd esign education', 'form', 'preoperative measurement', 'actuary', 'eit rawmatrials', 'kava call', 'eit rawmaterials', 'upscaling eit', 'eit raw', 'transmedia', 'materials science', 'material design behavior', 'teleworking', 'business plan', 'biomaterials', 'strategic business management', 'urban planning', 'renewable materials', 'technical textiles', 'plan eit', 'composite materials', 'digitization', 'raw materials', 'rawmaterials kava']</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>['biological systems', 'food safety', 'fermented food', 'processors euau', 'euafrica union', 'robotic safety', 'local food', 'occupational health safety', 'inclusion', 'employee safety', 'euau partnership', 'food systems', 'microbiology', 'uprise open', 'open data', 'european union', 'inclusive safe', 'open call', 'ecological resilience', 'patient safety', 'teleworking', 'food waste', 'healthcare systems', 'safety uprise', 'bioprocessing', 'conflict resolution', 'open banking', 'european integration', 'safe food', 'food processors', 'partnership resilient', 'resilient inclusive', 'bioenergy', 'food chemistry', 'social inclusion.', 'food heritage', 'call fermented', 'system design', 'microprocessors', 'world trade organization', 'functional foods', 'resilience', 'educational buildings', 'systems theory', 'systems everyone', 'union food']</t>
+          <t>['call fermented', 'conflict resolution', 'food heritage', 'functional foods', 'euau partnership', 'social inclusion.', 'bioprocessing', 'union food', 'microprocessors', 'partnership resilient', 'resilient inclusive', 'food chemistry', 'open call', 'processors euau', 'inclusion', 'healthcare systems', 'bioenergy', 'inclusive safe', 'european integration', 'food waste', 'world trade organization', 'systems everyone', 'biological systems', 'systems theory', 'food processors', 'food safety', 'safe food', 'teleworking', 'occupational health safety', 'uprise open', 'fermented food', 'ecological resilience', 'food systems', 'local food', 'robotic safety', 'microbiology', 'educational buildings', 'euafrica union', 'open data', 'system design', 'patient safety', 'european union', 'safety uprise', 'open banking', 'resilience', 'employee safety']</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>['support smes', 'poverty studies', 'grant programme', 'agile green', 'small medium enterprises', 'software development processes', 'social media support', 'performance arts', 'green building technologies', 'financial grant', 'environmental sustainability', 'transition csa', 'stage financial', 'migration', 'financial reporting', 'parenting', 'community development', 'sustainable development', 'green finance', 'sustainability', 'transform support', 'sustainable transition', 'green enterprise', 'biosimilars', 'software development', 'change innovation.', 'teleworking', 'sustainability transition', 'digital transformation', 'transition agile', 'social media support tools', 'bioprocessing', 'smes sustainability', 'csa stage', 'call sustainable', 'financial analysis', 'international finance', 'green consensus', 'accreditation', 'sponsorship management', 'innovate transform', 'banking', 'software', 'leadership', 'programme call', 'green technologies', 'ngo', 'data transformation']</t>
+          <t>['support smes', 'financial reporting', 'sustainability', 'bioprocessing', 'green building technologies', 'poverty studies', 'innovate transform', 'software development processes', 'green technologies', 'financial grant', 'environmental sustainability', 'green enterprise', 'sustainability transition', 'social media support', 'migration', 'small medium enterprises', 'change innovation.', 'grant programme', 'programme call', 'data transformation', 'smes sustainability', 'community development', 'sustainable development', 'financial analysis', 'transform support', 'accreditation', 'leadership', 'stage financial', 'call sustainable', 'agile green', 'teleworking', 'digital transformation', 'international finance', 'performance arts', 'parenting', 'transition agile', 'transition csa', 'csa stage', 'software', 'sustainable transition', 'software development', 'banking', 'green consensus', 'sponsorship management', 'biosimilars', 'social media support tools', 'green finance', 'ngo']</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>['strategic business management', 'local food', 'urban planning', 'eit food', 'sustainable finance', 'food impact', 'enterprise software systems', 'impact funding', 'food waste', 'corporate marketing', 'framework eit', 'plan eit', 'stabilization programs banking', 'food heritage', 'crowdfunding', 'food business', 'sponsorship management', 'business plan', 'funding framework', 'functional foods', 'eco-design', 'business model studies', 'use design contexts', 'business history']</t>
+          <t>['food heritage', 'functional foods', 'business history', 'business model studies', 'stabilization programs banking', 'enterprise software systems', 'crowdfunding', 'food impact', 'food waste', 'framework eit', 'food business', 'business plan', 'eit food', 'sustainable finance', 'eco-design', 'strategic business management', 'corporate marketing', 'urban planning', 'local food', 'plan eit', 'use design contexts', 'sponsorship management', 'impact funding', 'funding framework']</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>['medical research', 'area health', 'modern urban history', 'effectrial fostering', 'disease prevention', 'visual effect', 'research methods', 'comparative law', 'european research', 'research fostering', 'experimental economics', 'clinical applications', 'africa health', 'european union', 'era health', 'mediation', 'european studies', 'economic history', 'public health research', 'immunology', 'partnership fostering', 'research area', 'psycholinguistics', 'victimoffender mediation', 'area era', 'european integration', 'community studies', 'immunotherapy', 'europeanization', 'fostering pragmatic', 'community health', 'biomedical research', 'noncommunicable diseases', 'trials noncommunicable', 'european partnership', 'therapeutic alliance', 'public health', 'health research', 'clinical trials', 'infectious diseases', 'global collaboration', 'comparativeeffectiveness trials', 'diseases effectrial', 'mentalization', 'cognitive linguistics', 'research performance', 'clinical research', 'fostering european', 'pragmatic comparativeeffectiveness', 'comparative politics', 'social research']</t>
+          <t>['public health', 'biomedical research', 'effectrial fostering', 'social research', 'comparative politics', 'clinical trials', 'visual effect', 'comparative law', 'research performance', 'victimoffender mediation', 'mediation', 'research methods', 'area era', 'global collaboration', 'partnership fostering', 'fostering pragmatic', 'europeanization', 'public health research', 'noncommunicable diseases', 'community health', 'european research', 'research area', 'infectious diseases', 'european integration', 'community studies', 'mentalization', 'therapeutic alliance', 'pragmatic comparativeeffectiveness', 'africa health', 'psycholinguistics', 'economic history', 'comparativeeffectiveness trials', 'european partnership', 'trials noncommunicable', 'research fostering', 'clinical research', 'immunotherapy', 'immunology', 'health research', 'area health', 'clinical applications', 'cognitive linguistics', 'experimental economics', 'european union', 'fostering european', 'medical research', 'modern urban history', 'disease prevention', 'diseases effectrial', 'era health', 'european studies']</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>['aesthetics architecture', 'urban sprawl', 'better care', 'community development', 'economic transformation', 'intelligent systems', 'care european', 'care systems', 'healthcare technology', 'city', 'disabled care)', 'home culture', 'european union', 'elderly care', 'right city', 'health management', 'global health', 'community care', 'healthcare systems', 'digital transformation', 'closer home', 'growth', 'enhancing primary', 'home enhancing', 'european integration', 'primary community', 'community health', 'europeanization', 'partnership transforming', 'comfort', 'regeneration', 'interior design', 'european partnership', 'care closer', 'public health', 'transforming health', 'system design', 'health care', 'systems theory', 'systems better', 'healthcare policy']</t>
+          <t>['public health', 'healthcare policy', 'care closer', 'closer home', 'economic transformation', 'elderly care', 'health management', 'urban sprawl', 'regeneration', 'home enhancing', 'intelligent systems', 'home culture', 'europeanization', 'community health', 'healthcare systems', 'european integration', 'city', 'care european', 'community development', 'transforming health', 'systems theory', 'primary community', 'interior design', 'care systems', 'disabled care)', 'comfort', 'european partnership', 'digital transformation', 'health care', 'growth', 'partnership transforming', 'better care', 'healthcare technology', 'enhancing primary', 'aesthetics architecture', 'system design', 'global health', 'european union', 'community care', 'systems better', 'right city']</t>
         </is>
       </c>
     </row>
@@ -868,7 +868,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>['transnational adaptations', 'medical research', 'small medium enterprises', 'biological systems', 'european rare', 'urbanization', 'disease prevention', 'transnational call', 'diseases erdera', 'preclinical therapy', 'development validation', 'validity reliability', 'infectious disease control', 'child health diseases', 'small moleculesnand', 'partnership rare', 'research alliance', 'call preclinical', 'diseases using', 'mechanical engineering validation', 'fit', 'pharmacological treatments', 'studies rare', 'european union', 'clinical psychology', 'human development', ' validity', 'european studies', 'moleculesnand biologicals', 'biologicals development', 'erogenic aids', 'tempormandibular disorders', 'therapy studies', 'molecular modeling', 'joint transnational', 'european integration', 'using small', 'diseases research', 'europeanization', 'globalization', 'micromobility', 'psychodynamic psychotherapy', 'european partnership', 'therapeutic alliance', 'infectious diseases', 'genetic disorders', 'erdera joint', 'internationalization', 'clinical trials', 'global collaboration', 'molecular biology', 'rheumatologic rehabilitation', 'research performance', 'rare diseases', 'clinical research', 'drug development', 'transnational politics', 'sharing economy', 'validation european']</t>
+          <t>['micromobility', 'child health diseases', 'development validation', 'clinical trials', 'tempormandibular disorders', 'joint transnational', 'studies rare', 'research performance', 'erdera joint', 'clinical psychology', 'transnational call', 'molecular modeling', 'global collaboration', 'europeanization', 'research alliance', 'diseases erdera', 'small medium enterprises', 'infectious disease control', 'molecular biology', 'fit', ' validity', 'infectious diseases', 'rare diseases', 'european integration', 'transnational politics', 'mechanical engineering validation', 'globalization', 'biological systems', 'urbanization', 'therapeutic alliance', 'diseases research', 'psychodynamic psychotherapy', 'therapy studies', 'preclinical therapy', 'sharing economy', 'biologicals development', 'human development', 'diseases using', 'european partnership', 'erogenic aids', 'clinical research', 'validation european', 'moleculesnand biologicals', 'drug development', 'transnational adaptations', 'call preclinical', 'european rare', 'small moleculesnand', 'pharmacological treatments', 'partnership rare', 'validity reliability', 'european union', 'internationalization', 'using small', 'rheumatologic rehabilitation', 'genetic disorders', 'medical research', 'disease prevention', 'european studies']</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>['interest representation', 'tumor growth', 'erc proof', 'medical research', 'positron emission tomography', 'studies access justice', 'ercpoc ercpoc', 'council frontier', 'electronic commerce', 'convergence hypothesis', 'land reclamation', 'wages', 'right be forgotten', 'proposals erc', 'global studies', 'research horizonerc', 'european research', 'proof concept', 'public law', 'free associations', 'urban communication', 'enterprise software systems', 'quantitative research', 'city', 'social services', 'space settlement', 'lump sum', 'research council', 'european union', 'biosimilars', 'european studies', 'teleworking', 'conceptual design', 'social theory law', 'erogenic aids', 'black hole physics', 'grants call', 'political theory', 'frontier research', 'theory', 'conflict resolution', 'european integration', 'poc poc', 'concept lump', 'identity', 'sum ercpoc', 'coalition politics', 'reputation', 'erc ercpoc', 'sponsorship management', 'public economic law', 'therapeutic alliance', 'european education area', 'computational studies', 'mathematical finance', 'breast cancer', 'morphology', 'horizonerc lump', 'social research', 'public administration', 'dark matter', 'research performance', 'ngo', 'call proposals', 'concept proof', 'concept grant', 'poc proof', 'evaluation', 'grant erc', 'space debris', 'ercpoc european', 'concept grants', 'sum poc', 'economic analysis law', 'space research']</t>
+          <t>['proof concept', 'conflict resolution', 'evaluation', 'identity', 'social research', 'space debris', 'ercpoc ercpoc', 'sum poc', 'erc ercpoc', 'research performance', 'dark matter', 'enterprise software systems', 'concept proof', 'interest representation', 'reputation', 'free associations', 'wages', 'public law', 'grant erc', 'frontier research', 'european research', 'conceptual design', 'concept grants', 'european integration', 'city', 'convergence hypothesis', 'land reclamation', 'morphology', 'electronic commerce', 'economic analysis law', 'urban communication', 'therapeutic alliance', 'breast cancer', 'computational studies', 'erc proof', 'grants call', 'political theory', 'public economic law', 'teleworking', 'proposals erc', 'social services', 'space settlement', 'erogenic aids', 'tumor growth', 'global studies', 'space research', 'sum ercpoc', 'positron emission tomography', 'lump sum', 'right be forgotten', 'horizonerc lump', 'ercpoc european', 'concept grant', 'council frontier', 'poc proof', 'concept lump', 'research council', 'theory', 'sponsorship management', 'coalition politics', 'mathematical finance', 'call proposals', 'research horizonerc', 'biosimilars', 'european education area', 'european union', 'quantitative research', 'medical research', 'public administration', 'social theory law', 'poc poc', 'studies access justice', 'european studies', 'ngo', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -942,7 +942,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>['marine technology', 'biodiversity monitoring', 'data acquisition', 'call marine', 'data digital', 'environmental monitoring', 'ocean energy', 'monitoring data', 'twin ocean', 'ecology', 'integration biodiversity', 'data architecture', 'ecosystem', 'data analytics', 'data wrangling', 'marine ecosystem', 'seas', 'ocean call', 'marine biodiversity', 'data engineering', 'digitalization', 'digital twin', 'oceanography', 'digital systems', 'data integration', 'biodiversity conservation', 'marine discharges', 'digital', 'marine law']</t>
+          <t>['call marine', 'environmental monitoring', 'seas', 'marine ecosystem', 'integration biodiversity', 'marine discharges', 'marine technology', 'data acquisition', 'data wrangling', 'ocean energy', 'oceanography', 'data architecture', 'marine law', 'data digital', 'data analytics', 'data integration', 'ocean call', 'marine biodiversity', 'twin ocean', 'biodiversity monitoring', 'digital', 'data engineering', 'biodiversity conservation', 'ecology', 'digital twin', 'ecosystem', 'digitalization', 'digital systems', 'monitoring data']</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>['communication research', 'short film', 'medical research', 'biological systems', 'company law', 'culture, identity, body', 'serious games', 'exchange focussing', 'manufacturing systems', 'strategic communication', 'piloting new', 'bioremediation', 'new industryacademia', 'business capabilities', 'industryacademia collaborations', 'aviation', 'cocreation mechanism', 'indusac open', 'open data', 'human development', 'open call', 'call students', 'public relations', 'knowledge exchange', 'adaptation', 'child studies', 'biotechnology companies', 'teleworking', 'space industry', 'industrial engineering', 'needs csa', 'corporate marketing', 'communication', 'youth studies', 'restructuring companies', 'open banking', 'knowledge discovery', 'new ways working', 'community studies', 'commodification', '(integrative) system biology', 'csa indusac', 'quick challengedriven', 'mechanism industryacademia', 'biomedical research', 'developmental needs', 'industrial data', 'researchers quick', 'human rights', 'students researchers', 'humancentered cocreation', 'challengedriven humancentered', 'industryacademia knowledge', 'biotech industry', 'focussing companies', 'companies needs', 'ngo', 'research performance', 'educational buildings', 'aviation management', 'classroom climate', 'pharmaceutical industry', 'care policies (childcare', 'industrial design']</t>
+          <t>['biomedical research', 'call students', 'industrial design', 'strategic communication', 'developmental needs', 'research performance', 'humancentered cocreation', 'industrial data', 'cocreation mechanism', 'industryacademia knowledge', 'human rights', 'aviation', 'care policies (childcare', 'new ways working', 'open call', 'indusac open', 'industryacademia collaborations', 'companies needs', 'bioremediation', '(integrative) system biology', 'community studies', 'manufacturing systems', 'knowledge exchange', 'biological systems', 'mechanism industryacademia', 'exchange focussing', 'company law', 'communication', 'commodification', 'space industry', 'short film', 'adaptation', 'teleworking', 'human development', 'piloting new', 'public relations', 'csa indusac', 'pharmaceutical industry', 'corporate marketing', 'needs csa', 'communication research', 'culture, identity, body', 'new industryacademia', 'business capabilities', 'industrial engineering', 'knowledge discovery', 'classroom climate', 'biotech industry', 'students researchers', 'aviation management', 'restructuring companies', 'serious games', 'open data', 'child studies', 'quick challengedriven', 'researchers quick', 'medical research', 'biotechnology companies', 'challengedriven humancentered', 'educational buildings', 'open banking', 'focussing companies', 'ngo', 'youth studies']</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>['understanding interactions', 'medical research', 'molecular therapeutics', 'area health', 'modern urban history', 'parenting', 'therapeutic proteins', 'research methods', 'european research', 'human behavior', 'cardiovascular disorders', 'quantitative research', 'africa health', 'pharmacological treatments', 'european union', 'contact mechanics', 'era health', 'mediation', 'european studies', 'disorders comorbidities', 'economic history', 'public health research', 'mental health diseases', 'partnership fostering', 'anxiety', 'research area', 'area era', 'european integration', 'vascularization', 'therapeutic treatments', 'interactions cardiovascular', 'treatments interheart', 'europeanization', 'community studies', 'interheart fostering', 'immunotherapy', 'community health', 'cardiovascular nursing', 'biomolecular interactions', 'social inclusion.', 'european partnership', 'research understanding', 'therapeutic alliance', 'health research', 'public health', 'genetic disorders', 'global collaboration', 'mental health', 'research performance', 'comorbidities andor', 'bipolar disorders', 'fostering european', 'psychosocial problems chronic diseases (especially cancer patients)', 'social research', 'andor therapeutic']</t>
+          <t>['molecular therapeutics', 'public health', 'disorders comorbidities', 'therapeutic treatments', 'social research', 'contact mechanics', 'research performance', 'biomolecular interactions', 'social inclusion.', 'understanding interactions', 'mediation', 'human behavior', 'research methods', 'cardiovascular nursing', 'interactions cardiovascular', 'area era', 'bipolar disorders', 'vascularization', 'global collaboration', 'partnership fostering', 'europeanization', 'public health research', 'treatments interheart', 'community health', 'european research', 'research area', 'european integration', 'community studies', 'therapeutic alliance', 'interheart fostering', 'therapeutic proteins', 'africa health', 'economic history', 'psychosocial problems chronic diseases (especially cancer patients)', 'european partnership', 'research understanding', 'comorbidities andor', 'parenting', 'immunotherapy', 'health research', 'area health', 'pharmacological treatments', 'mental health diseases', 'cardiovascular disorders', 'anxiety', 'mental health', 'quantitative research', 'european union', 'fostering european', 'medical research', 'modern urban history', 'genetic disorders', 'era health', 'european studies', 'andor therapeutic']</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>['eu missions', 'image recognition', 'civil society', 'urban society', 'ecosystem services', 'environmental sustainability', 'area european', 'prize citizen', 'image recognition algorithms', 'sustainable eco', 'urban ecology', 'research methods', 'citizen science', 'european research', 'science impetus', 'climate change', 'citizenship', 'society climate', 'sustainability', 'climate', 'eco ecosystem', 'supporting giving', 'volunteering', 'ecosystem', 'european union', 'european studies', 'eu law', 'urban design', 'society', 'giving recognition', 'recognition citizen', 'research area', 'biometric recognition', 'ecosystem urban', 'european integration', 'rewarding', 'science european', 'environmental science', 'identity', 'community studies', 'reputation', 'change eu', 'european education area', 'impetus sustainable', 'sustainable cities', 'physics', 'collective bargaining models', 'artificial ecosystems', 'union prize', 'political science', 'sustainable consumption', 'planetary science']</t>
+          <t>['society', 'giving recognition', 'identity', 'sustainability', 'change eu', 'political science', 'area european', 'urban society', 'research methods', 'supporting giving', 'rewarding', 'image recognition', 'eu law', 'physics', 'environmental sustainability', 'union prize', 'impetus sustainable', 'reputation', 'urban ecology', 'science european', 'european studies', 'collective bargaining models', 'planetary science', 'european research', 'research area', 'european integration', 'community studies', 'volunteering', 'climate', 'sustainable cities', 'sustainable consumption', 'urban design', 'citizenship', 'artificial ecosystems', 'sustainable eco', 'image recognition algorithms', 'eu missions', 'society climate', 'civil society', 'climate change', 'eco ecosystem', 'recognition citizen', 'ecosystem urban', 'ecosystem', 'citizen science', 'european education area', 'european union', 'prize citizen', 'environmental science', 'biometric recognition', 'ecosystem services', 'science impetus']</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>['short film', 'innovation partnership', 'african economy', 'renewable energy', 'environmental sustainability', 'africa', 'sustainable development', 'green finance', 'biotechnology innovation', 'energy innovation', 'energy longterm', 'action europeafrica', 'investor behavior', 'sustainability', 'euau research', 'european union', 'energy', 'european studies', 'change innovation.', 'welding', 'africaeu cofund', 'tempormandibular disorders', 'african development', 'europeafrica research', 'biotech innovation', 'energy efficiency', 'european integration', 'call sustainable', 'research innovation', 'crowdfunding', 'cofund action', 'sustainable technology', 'sustainable energy', 'longterm joint', 'joint euau', 'partnership sustainable', 'research performance', 'innovation call', 'energy policy']</t>
+          <t>['biotech innovation', 'sustainable technology', 'investor behavior', 'longterm joint', 'sustainability', 'tempormandibular disorders', 'welding', 'research performance', 'africa', 'innovation call', 'energy', 'environmental sustainability', 'crowdfunding', 'change innovation.', 'african development', 'energy longterm', 'renewable energy', 'euau research', 'european integration', 'energy policy', 'african economy', 'sustainable development', 'europeafrica research', 'call sustainable', 'innovation partnership', 'action europeafrica', 'biotechnology innovation', 'cofund action', 'sustainable energy', 'research innovation', 'joint euau', 'africaeu cofund', 'partnership sustainable', 'european union', 'green finance', 'short film', 'energy efficiency', 'european studies', 'energy innovation']</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>['production planning', 'call companies', 'eit manufacturing', 'higher education', 'manufacturing systems', 'strategic business management', 'urban planning', 'companies students', 'labor markets', 'competition law', 'child studies', 'teleworking', 'd esign education', 'eit manufacturings', 'industrial engineering', 'corporate marketing', 'students eit', 'educational technologies', 'industrial design', 'competitive strategies', 'teaching factories', 'manufacturing business', 'plan eit', 'competition call', 'factories competition', 'manufacturings teaching', 'corporate communication', 'electronics manufacturing', 'business plan', 'competition law policy', 'education', 'business model studies', 'mechanical engineering manufacturing', 'business history']</t>
+          <t>['mechanical engineering manufacturing', 'companies students', 'business model studies', 'business history', 'industrial design', 'educational technologies', 'higher education', 'call companies', 'corporate communication', 'labor markets', 'competition law', 'd esign education', 'eit manufacturings', 'eit manufacturing', 'manufacturings teaching', 'competition call', 'manufacturing systems', 'competition law policy', 'students eit', 'teleworking', 'business plan', 'strategic business management', 'production planning', 'urban planning', 'corporate marketing', 'education', 'industrial engineering', 'plan eit', 'electronics manufacturing', 'competitive strategies', 'manufacturing business', 'factories competition', 'child studies', 'teaching factories']</t>
         </is>
       </c>
     </row>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>['hinfinity control', 'fashion supply chain', 'local food', 'sustainable fashion', 'open data', 'european union', 'open call', 'european studies', 'mechanical engineering support', 'creativity', 'open banking', 'beautiful sustainably', 'urban manufacturing', 'prisons', 'technical textiles', 'localised urban', 'operations research', 'urbanization', 'sustainably designed', 'new media technologies', 'community development', 'textile history', 'spina bifida', 'regenerative textile', 'scandinavian cinema', 'fstp open', 'fostering local', 'ecological resilience', 'bauhaus ria', 'teleworking', 'regenerative medicine', 'technology fashion products', 'social media systems', 'urban studies', 'regeneration', 'athens rotterdam', 'balkans', 'cultural landscapes', 'clothing industry', 'using fstp', 'facilitators athens', 'clothing ecosystems', 'african music', 'industry facilitators', 'sustainability', 'city', 'rotterdam fostering', 'call textile', 'sustainable design planning', 'urban design', 'european bauhaus', 'sustainable fashion practices', 'ria using', 'europeanization', 'software', 'leadership', 'transmedia', 'supporting creativity', 'design sustainability', 'mechanical engineering manufacturing', 'fashion retail', 'local beautiful', 'manufacturing systems', 'creativity new', 'designed regenerative', ' housing studies', 'ecological design', 'textile art', 'aesthetics place', 'ecosystem', 'manufacturing supporting', 'new european', 'press history', 'creative industry', 'creative labor', 'textile clothing', 'tissue engineering regenerative medicine', 'european education area']</t>
+          <t>['scandinavian cinema', 'sustainable fashion practices', 'fashion supply chain', 'community development', 'mechanical engineering support', 'african music', 'european bauhaus', 'transmedia', 'call textile', 'using fstp', 'localised urban', 'urban manufacturing', 'regenerative medicine', 'open data', 'creative industry', 'sustainable design planning', ' housing studies', 'fostering local', 'mechanical engineering manufacturing', 'operations research', 'cultural landscapes', 'sustainable fashion', 'manufacturing supporting', 'open call', 'regenerative textile', 'urban design', 'hinfinity control', 'technology fashion products', 'tissue engineering regenerative medicine', 'ecological resilience', 'local food', 'creativity new', 'software', 'rotterdam fostering', 'european union', 'open banking', 'designed regenerative', 'creative labor', 'fstp open', 'urban studies', 'sustainability', 'supporting creativity', 'textile art', 'regeneration', 'new european', 'clothing industry', 'new media technologies', 'facilitators athens', 'textile history', 'leadership', 'ecological design', 'aesthetics place', 'bauhaus ria', 'local beautiful', 'social media systems', 'ecosystem', 'european studies', 'spina bifida', 'press history', 'design sustainability', 'textile clothing', 'europeanization', 'fashion retail', 'city', 'manufacturing systems', 'urbanization', 'balkans', 'teleworking', 'beautiful sustainably', 'technical textiles', 'prisons', 'ria using', 'european education area', 'creativity', 'athens rotterdam', 'sustainably designed', 'industry facilitators', 'clothing ecosystems']</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>['', 'penology', 'actor training', 'planetary science', 'fellowship residencies', 'immigration', 'journalism initiative', ' housing studies', 'earth science', 'space reporting', 'initiative call', 'citizenship', 'round n', 'training independent', 'fit', 'call applications', 'frontiers science', 'ethics', 'space consulting', 'journalism', 'teleworking', 'erc science', 'program round', 'independent ethical', 'mobile applications', 'n fellowship', 'science journalism', 'bioengineering applications', 'applications mathematical physics', 'environmental science', 'applications frontiers', 'robotic training', 'professionals tools', 'tools training', 'mechanical engineering training', 'reporting science', 'ethical reporting', 'parallel programming', 'reputation', 'accreditation', 'space training', 'news analysis', 'science news', 'therapeutic alliance', 'space exploration', 'tool design', 'mechanical engineering tools', 'software', 'physics', 'journalism media studies', 'egovernment', 'news professionals', 'journalism residency', 'residency program', 'ngo', 'automation', 'residencies offering', 'offering science']</t>
+          <t>['', 'penology', 'applications frontiers', 'science journalism', ' housing studies', 'space exploration', 'tool design', 'ethics', 'journalism', 'mobile applications', 'offering science', 'bioengineering applications', 'n fellowship', 'journalism initiative', 'round n', 'physics', 'parallel programming', 'robotic training', 'space consulting', 'reputation', 'mechanical engineering tools', 'journalism residency', 'reporting science', 'planetary science', 'fit', 'earth science', 'initiative call', 'training independent', 'mechanical engineering training', 'space training', 'accreditation', 'news professionals', 'therapeutic alliance', 'news analysis', 'frontiers science', 'citizenship', 'independent ethical', 'teleworking', 'professionals tools', 'space reporting', 'tools training', 'applications mathematical physics', 'erc science', 'fellowship residencies', 'program round', 'residencies offering', 'residency program', 'actor training', 'egovernment', 'software', 'journalism media studies', 'ethical reporting', 'immigration', 'automation', 'science news', 'environmental science', 'ngo', 'call applications']</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>['plan innovation', 'ris innovation', 'strategic business management', 'capacity building', 'green building technologies', 'space services', 'robotic innovation', 'biodegradable materials', 'urban planning', 'biomaterials', 'raw materials', 'planning design', 'biotechnology innovation', 'business capabilities', 'eit raw', 'scandinavian cinema', 'civil society capacity strengthening', 'kava call', 'change innovation.', 'actuary', 'teleworking', 'd esign education', 'materials business', 'growth', 'electronic engineering design', 'innovation capacity', 'plan eit', 'eit rawmaterials', 'materials science', 'material design behavior', 'eit rawmatrials', 'building eit', 'rawmatrials business', 'composite materials', 'business plan', 'renewable materials', 'rawmaterials kava', 'evaluation', 'transmedia', 'form', 'eco-design', 'material based design', 'business model studies', 'call ris', 'technical textiles', 'business history']</t>
+          <t>['ris innovation', 'evaluation', 'robotic innovation', 'electronic engineering design', 'business history', 'business model studies', 'scandinavian cinema', 'materials business', 'capacity building', 'rawmatrials business', 'green building technologies', 'biodegradable materials', 'material based design', 'innovation capacity', 'd esign education', 'change innovation.', 'call ris', 'form', 'civil society capacity strengthening', 'actuary', 'eit rawmatrials', 'kava call', 'eit rawmaterials', 'eit raw', 'transmedia', 'materials science', 'material design behavior', 'teleworking', 'business plan', 'biomaterials', 'growth', 'eco-design', 'strategic business management', 'biotechnology innovation', 'urban planning', 'building eit', 'renewable materials', 'business capabilities', 'plan eit', 'composite materials', 'technical textiles', 'plan innovation', 'raw materials', 'space services', 'planning design', 'rawmaterials kava']</t>
         </is>
       </c>
     </row>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>['strategic business management', 'biodegradable materials', 'urban planning', 'biomaterials', 'call eit', 'raw materials', 'eit raw', 'scandinavian cinema', 'actuary', 'teleworking', 'd esign education', 'erogenic aids', 'booster call', 'erma booster', 'materials business', 'rewarding', 'plan eit', 'eit rawmaterials', 'materials science', 'material design behavior', 'd esign management', 'eit rawmatrials', 'electronic payment services', 'composite materials', 'rawmatrials business', 'concordat', 'performance', 'business plan', 'renewable materials', 'evaluation', 'transmedia', 'rawmaterials erma', 'material based design', 'business model studies', 'technical textiles', 'business history']</t>
+          <t>['evaluation', 'electronic payment services', 'business history', 'business model studies', 'scandinavian cinema', 'materials business', 'erma booster', 'rawmatrials business', 'biodegradable materials', 'rewarding', 'material based design', 'performance', 'd esign education', 'd esign management', 'booster call', 'actuary', 'eit rawmatrials', 'eit rawmaterials', 'eit raw', 'transmedia', 'materials science', 'material design behavior', 'teleworking', 'business plan', 'rawmaterials erma', 'erogenic aids', 'biomaterials', 'strategic business management', 'urban planning', 'renewable materials', 'technical textiles', 'plan eit', 'composite materials', 'raw materials', 'concordat', 'call eit']</t>
         </is>
       </c>
     </row>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>['transnational adaptations', 'strategic business management', 'strategic communication', 'economic transformation', 'robotic innovation', 'jumpstarter crosskic', 'rocket propulsion', 'crosskic regional', 'social media innovation tools', 'social media innovation', 'entrepreneurship', 'sports', 'change innovation.', 'immigrant athletes', 'd esign education', 'eit crosskic', 'strategic regional', 'regional innovation', 'russia', 'competitive strategies', 'regional innovations', 'football', 'd esign management', 'innovation eit', 'strategic management', 'concordat', 'innovations cluster', 'crosskic strategic', 'electric vehicles', 'economic development', 'eco-design', 'strategy', 'eit jumpstarter']</t>
+          <t>['robotic innovation', 'regional innovation', 'strategic management', 'economic transformation', 'strategic communication', 'immigrant athletes', 'economic development', 'crosskic strategic', 'social media innovation tools', 'football', 'regional innovations', 'd esign education', 'change innovation.', 'd esign management', 'rocket propulsion', 'social media innovation', 'strategy', 'innovations cluster', 'eit jumpstarter', 'jumpstarter crosskic', 'electric vehicles', 'entrepreneurship', 'eco-design', 'eit crosskic', 'strategic business management', 'transnational adaptations', 'innovation eit', 'competitive strategies', 'strategic regional', 'crosskic regional', 'sports', 'russia', 'concordat']</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1349,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>['online child abuse', 'open sharing', 'business intelligence', 'sharing fair', 'open data', 'call adoption', 'performance based design', 'initiatives helping', 'alliance facilitation', 'creativity', 'open banking', 'crowdfunding', 'detector rd', 'data journalism', 'system design', 'research solutions', 'fair research', 'care policies (childcare', 'biosecurity', 'hurricane', 'deep ecology', 'research methods', 'defense mechanisms', 'quantitative research', 'space standards', 'recommendation systems', 'specifications recommendations', 'rda tiger', 'eoscrelated research', 'cascade grant', 'biomedical research', 'internationalization', 'design research methods', 'global collaboration', 'research performance', 'group theory', 'support initiatives', 'facilitation targeted', 'mechanical engineering standards', 'social research', 'international working', 'signal generators', 'youth work', 'medical research', 'social media support', 'data analysis', 'data collection', 'software rda', 'global value chains', 'free associations', 'enterprise software systems', 'disadvantaged groups', 'family studies', 'volunteering', 'biosimilars', 'alternative organizations', 'international organizations', 'groups eoscrelated', 'reputation', 'software design', 'therapeutic alliance', 'software', 'collective identities', 'global standards', 'strategy', 'recommendations open', 'grant call', 'mobilization', 'parenting', 'land reclamation', 'research data', 'international relations', 'grandparenting', 'targeted international', 'grants research', 'ecosystem', 'generative algorithms', 'data publications', 'adaptation', 'data alliance', 'fairness', 'tiger cascade', 'social media support tools', 'working groups', 'group dynamics', 'generate global', 'publications software', 'globalization', 'coalition politics', 'data governance', 'adoption grants', 'international development', 'privacy', 'helping generate', 'standards specifications', 'data science', 'sharing economy']</t>
+          <t>['data analysis', 'eoscrelated research', 'social research', 'data alliance', 'grant call', 'global collaboration', 'reputation', 'helping generate', 'research solutions', 'care policies (childcare', 'group dynamics', 'land reclamation', 'data science', 'disadvantaged groups', 'sharing economy', 'software rda', 'parenting', 'online child abuse', 'data publications', 'recommendation systems', 'publications software', 'collective identities', 'open data', 'biosimilars', 'quantitative research', 'youth work', 'sharing fair', 'family studies', 'social media support', 'free associations', 'international organizations', 'standards specifications', 'space standards', 'performance based design', 'global value chains', 'biosecurity', 'design research methods', 'group theory', 'rda tiger', 'fair research', 'software', 'system design', 'defense mechanisms', 'open banking', 'mechanical engineering standards', 'biomedical research', 'working groups', 'generate global', 'research performance', 'research methods', 'groups eoscrelated', 'research data', 'crowdfunding', 'specifications recommendations', 'detector rd', 'grandparenting', 'adoption grants', 'volunteering', 'globalization', 'strategy', 'mobilization', 'data journalism', 'tiger cascade', 'deep ecology', 'cascade grant', 'data governance', 'ecosystem', 'coalition politics', 'alternative organizations', 'alliance facilitation', 'international relations', 'software design', 'support initiatives', 'recommendations open', 'enterprise software systems', 'initiatives helping', 'privacy', 'hurricane', 'signal generators', 'international working', 'data collection', 'international development', 'therapeutic alliance', 'open sharing', 'adaptation', 'grants research', 'targeted international', 'generative algorithms', 'business intelligence', 'fairness', 'global standards', 'facilitation targeted', 'internationalization', 'creativity', 'social media support tools', 'medical research', 'call adoption']</t>
         </is>
       </c>
     </row>
@@ -1386,7 +1386,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>['towards sustainable', 'actor training', 'robotic maintenance', 'performance arts', 'biological networks', 'cascade grants', 'upskilling towards', 'deconstruction', 'environmental sustainability', 'ecosystem open', 'international construction law', 'ecosystem services', 'distribution agreements', 'africa', 'cbe ju', 'sustainable development', 'alliance new', 'academy alliance', 'free associations', 'sustainability', 'cybersecurity', 'physical activity', 'african education', 'bauhaus academy', 'volunteering', 'supporting activities', 'european union', 'ecosystem', 'open call', 'open data', 'robotic support', 'method architectural design', 'biosimilars', 'new european', 'grants neba', 'reskilling upskilling', 'european bauhaus', 'd esign education', 'supporters', 'academy network', 'network analysis', 'sustainable construction', 'teleworking', 'theater', 'bioprocessing', 'neba alliance', 'open banking', 'african refugees', 'law education', 'new ways working', 'europeanization', 'construction management', 'accreditation', 'activities new', 'space training', 'construction ecosystem', 'ju supporting', 'waste management', 'therapeutic alliance', 'supporter behavior', 'global collaboration', 'evliyâ çelebi studies', 'network reskilling', 'ngo', 'strategy', 'design sustainability', 'artificial ecosystems', 'call cascade', 'new media']</t>
+          <t>['supporters', 'new media', 'waste management', 'sustainability', 'international construction law', 'sustainable construction', 'bioprocessing', 'africa', 'supporting activities', 'design sustainability', 'environmental sustainability', 'global collaboration', 'evliyâ çelebi studies', 'new european', 'europeanization', 'free associations', 'academy alliance', 'd esign education', 'new ways working', 'open call', 'method architectural design', 'law education', 'biological networks', 'activities new', 'cbe ju', 'physical activity', 'ju supporting', 'reskilling upskilling', 'volunteering', 'space training', 'accreditation', 'robotic maintenance', 'network reskilling', 'call cascade', 'supporter behavior', 'cybersecurity', 'strategy', 'therapeutic alliance', 'african education', 'european bauhaus', 'cascade grants', 'artificial ecosystems', 'robotic support', 'teleworking', 'construction ecosystem', 'grants neba', 'alliance new', 'ecosystem open', 'performance arts', 'ngo', 'construction management', 'sustainable development', 'neba alliance', 'actor training', 'academy network', 'theater', 'bauhaus academy', 'deconstruction', 'ecosystem', 'african refugees', 'network analysis', 'open data', 'distribution agreements', 'biosimilars', 'upskilling towards', 'european union', 'towards sustainable', 'open banking', 'ecosystem services']</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>['computation based design', 'youth work', 'implementation support', 'ottoman institutions civilization', 'making western', 'performance arts', 'ri policy', 'policy implementation', 'making implementation', 'youth campaign', 'history middle east.', 'method architectural design', 'robotic support', 'policy analysis', 'mechanical engineering support', 'social media campaign tools', 'supporters', 'support western', 'youth awards', 'support ri', 'youth studies', 'algorithm design', 'rewarding', 'ottoman constitutional history modern balkans abilities albanians (luke) history', 'policy making', 'western balkans', 'coalition politics', 'social media campaigns', 'western blotting', 'balkans ri', 'youth cultures', 'balkans western', 'turkish', 'space support', 'balkans', 'ri youth', 'awards western', 'public policy', 'cultural landscapes', 'campaign ri']</t>
+          <t>['supporters', 'making western', 'cultural landscapes', 'balkans western', 'support western', 'rewarding', 'social media campaigns', 'balkans ri', 'method architectural design', 'space support', 'policy analysis', 'turkish', 'ri policy', 'mechanical engineering support', 'social media campaign tools', 'computation based design', 'balkans', 'ottoman institutions civilization', 'ottoman constitutional history modern balkans abilities albanians (luke) history', 'western balkans', 'public policy', 'robotic support', 'ri youth', 'awards western', 'youth awards', 'implementation support', 'policy implementation', 'performance arts', 'support ri', 'youth cultures', 'history middle east.', 'algorithm design', 'policy making', 'campaign ri', 'making implementation', 'coalition politics', 'youth campaign', 'western blotting', 'youth work', 'youth studies']</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>['interest representation', 'transnational adaptations', 'strategic business management', 'strategic communication', 'economic transformation', 'robotic innovation', 'next call', 'crosskic regional', 'urban communication', 'social media innovation tools', 'social media innovation', 'entrepreneurship', 'change innovation.', 'teleworking', 'd esign education', 'eit crosskic', 'strategic regional', 'regional innovation', 'sexuality gender football', 'russia', 'competitive strategies', 'regional innovations', 'football', 'proposals crosskic', 'd esign management', 'innovation eit', 'crowdfunding', 'strategic management', 'space exploration', 'concordat', 'directing', ' future work', 'innovations cluster', 'crosskic strategic', 'electric vehicles', 'jumpstarter next', 'economic development', 'eco-design', 'strategy', 'call proposals', 'eit jumpstarter']</t>
+          <t>['robotic innovation', 'regional innovation', 'space exploration', 'strategic management', 'economic transformation', 'strategic communication', 'economic development', 'crosskic strategic', 'social media innovation tools', 'interest representation', 'football', 'crowdfunding', 'directing', 'regional innovations', 'd esign education', 'change innovation.', 'd esign management', 'next call', 'social media innovation', 'strategy', 'urban communication', 'innovations cluster', 'eit jumpstarter', 'electric vehicles', 'teleworking', 'entrepreneurship', 'eit crosskic', 'eco-design', 'strategic business management', 'transnational adaptations', 'innovation eit', 'competitive strategies', 'strategic regional', 'crosskic regional', 'jumpstarter next', 'proposals crosskic', 'call proposals', 'russia', 'concordat', 'sexuality gender football', ' future work']</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>['interest representation', 'grant scheme', 'distribution agreements', 'booster grant', 'financial reporting', 'social welfare', 'land reclamation', 'sports sponsorship', 'robotic research', 'sustainable finance', 'biotechnology innovation', 'eic booster', 'urban communication', 'investor behavior', 'impact eicsupported', 'social media innovation', 'proposals bringing', 'physical activity', 'dynamic portfolio theory', 'bringing financial', 'mode choice', 'robotic support', 'change innovation.', 'decision tree', 'financial support', 'teleworking', 'increasing impact', 'biotech innovation', 'growth', 'rewarding', 'financial analysis', 'scheme boost', 'portfolio activities', 'support innovation', 'electronic devices', 'electronic payment services', 'parallel programming', 'sponsorship management', 'biomedical research', 'algorithm optimization', 'innovation portfolio', 'performance', 'banking', 'biomechanics', 'activities increasing', 'electric vehicles', 'policy studies', 'research performance', 'boost call', 'support eic', 'financial crises', 'giftgiving', 'call proposals', 'eicsupported research']</t>
+          <t>['biotech innovation', 'bringing financial', 'boost call', 'biomedical research', 'financial reporting', 'electronic payment services', 'financial crises', 'investor behavior', 'increasing impact', 'booster grant', 'research performance', 'rewarding', 'scheme boost', 'parallel programming', 'biomechanics', 'algorithm optimization', 'interest representation', 'policy studies', 'electronic devices', 'performance', 'giftgiving', 'change innovation.', 'mode choice', 'physical activity', 'land reclamation', 'financial analysis', 'social media innovation', 'grant scheme', 'urban communication', 'sports sponsorship', 'eicsupported research', 'dynamic portfolio theory', 'support innovation', 'robotic support', 'electric vehicles', 'teleworking', 'social welfare', 'sustainable finance', 'growth', 'impact eicsupported', 'support eic', 'biotechnology innovation', 'portfolio activities', 'banking', 'financial support', 'sponsorship management', 'proposals bringing', 'call proposals', 'distribution agreements', 'innovation portfolio', 'eic booster', 'activities increasing', 'robotic research', 'decision tree']</t>
         </is>
       </c>
     </row>
@@ -1534,7 +1534,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>['composition', 'startups access', 'space infrastructure', 'small medium enterprises', 'signal generators', 'network pilot', 'euwide network', 'generation platform', 'growth development', 'aircraft systems', 'facilities improving', 'electronic testing', 'robotic testing', 'operations research', 'faster innovation', 'strategic business management', 'plants testing', 'calltravelvouchers cocreating', 'trust service provider', 'ecosystem services', 'data security', 'pilot plants', 'memory', 'business capabilities', 'unlocking faster', 'cocreating next', 'biotechnology innovation', 'testing facilities', 'entrepreneurship', 'aviation', 'children', 'infrastructures unlocking', 'documentary', 'european union', 'smes startups', 'multidimensional scaling', 'change innovation.', 'european studies', 'network analysis', 'digital media children', 'internal entrepreneurship', 'biotech innovation', 'access scaleup', 'genetic testing', 'growth', 'decarbonization', 'improving smes', 'pilot demo', 'airport access', 'platform pilot', 'rewarding', 'genetic engineering', 'eu bioeconomy', 'platform employees', 'europeanization', 'stabilization programs banking', 'innovation eu', 'commodification', 'electronic payment services', 'scaleup calltravelvouchers', 'digital services', 'smart infrastructure', 'european education area', 'performance', 'biotech startups', 'demo infrastructures', 'bioengineering', 'consumer ethics', 'genetic programming', 'bioeconomy growth', 'automated testing', 'educational buildings', 'aviation management', 'demographic change', 'next generation']</t>
+          <t>['biotech innovation', 'multidimensional scaling', 'trust service provider', 'electronic payment services', 'genetic testing', 'stabilization programs banking', 'consumer ethics', 'biotech startups', 'innovation eu', 'bioeconomy growth', 'operations research', 'genetic engineering', 'airport access', 'cocreating next', 'euwide network', 'decarbonization', 'rewarding', 'pilot plants', 'memory', 'electronic testing', 'improving smes', 'faster innovation', 'internal entrepreneurship', 'facilities improving', 'platform pilot', 'smart infrastructure', 'performance', 'aircraft systems', 'small medium enterprises', 'aviation', 'signal generators', 'change innovation.', 'smes startups', 'eu bioeconomy', 'european studies', 'europeanization', 'access scaleup', 'infrastructures unlocking', 'demographic change', 'bioengineering', 'commodification', 'generation platform', 'scaleup calltravelvouchers', 'documentary', 'growth', 'growth development', 'entrepreneurship', 'automated testing', 'testing facilities', 'strategic business management', 'biotechnology innovation', 'pilot demo', 'business capabilities', 'genetic programming', 'network pilot', 'next generation', 'robotic testing', 'plants testing', 'demo infrastructures', 'aviation management', 'platform employees', 'network analysis', 'startups access', 'space infrastructure', 'unlocking faster', 'european education area', 'digital services', 'composition', 'european union', 'data security', 'educational buildings', 'calltravelvouchers cocreating', 'digital media children', 'ecosystem services', 'children']</t>
         </is>
       </c>
     </row>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>['women entrepreneurs', 'speech synthesis', 'renewable energy', 'werise open', 'sustainable development', 'renewable energy systems', 'sustainability', 'entrepreneurship', 'aesthetics place', 'renewable energy engineering', 'open data', 'entrepreneurs renewable', 'european union', 'open call', 'mode choice', 'sustainable enterprises', 'teleworking', 'innovative sustainable', 'phase women', 'open banking', 'womens entrepreneurship', 'call phase', 'europe werise', 'gender psychology', 'feminist theory', 'sustainable technology', 'european education area', 'startup europe', 'renewable innovative', 'women']</t>
+          <t>['sustainable technology', 'innovative sustainable', 'sustainability', 'startup europe', 'renewable innovative', 'renewable energy engineering', 'call phase', 'europe werise', 'phase women', 'open call', 'renewable energy', 'mode choice', 'women entrepreneurs', 'renewable energy systems', 'sustainable development', 'gender psychology', 'teleworking', 'womens entrepreneurship', 'entrepreneurship', 'aesthetics place', 'werise open', 'women', 'speech synthesis', 'open data', 'european education area', 'feminist theory', 'european union', 'sustainable enterprises', 'open banking', 'entrepreneurs renewable']</t>
         </is>
       </c>
     </row>
@@ -1608,7 +1608,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>['transnational adaptations', 'turkish cuisine', 'strategic business management', 'strategic communication', 'economic transformation', 'robotic innovation', 'electronic commerce', 'crosskic regional', 'social media innovation tools', 'social media innovation', 'turkish music', 'eit red', 'change innovation.', 'immigrant athletes', 'd esign education', 'erogenic aids', 'eit crosskic', 'strategic regional', 'regional innovation', 'russia', 'competitive strategies', 'regional innovations', 'football', 'd esign management', 'red kalyna', 'green consensus', 'kalyna crosskic', 'innovation eit', 'strategic management', 'turkish', 'concordat', 'womens sports', 'innovations cluster', 'crosskic strategic', 'economic development', 'eco-design', 'strategy']</t>
+          <t>['robotic innovation', 'turkish cuisine', 'regional innovation', 'strategic management', 'economic transformation', 'strategic communication', 'immigrant athletes', 'economic development', 'crosskic strategic', 'social media innovation tools', 'red kalyna', 'football', 'regional innovations', 'd esign education', 'change innovation.', 'd esign management', 'turkish', 'electronic commerce', 'social media innovation', 'strategy', 'turkish music', 'innovations cluster', 'erogenic aids', 'eit crosskic', 'eco-design', 'strategic business management', 'transnational adaptations', 'innovation eit', 'eit red', 'strategic regional', 'competitive strategies', 'green consensus', 'crosskic regional', 'womens sports', 'russia', 'concordat', 'kalyna crosskic']</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>['composition', 'support smes', 'boosting uptake', 'small medium enterprises', 'production planning', 'software development processes', 'social media support', 'strategic business management', 'environmental sustainability', 'business model', 'transition csa', 'migration', 'upcirc second', 'inclusion', 'manufacturing systems', 'robotic innovation', 'product process', 'sustainability', 'call boosting', 'transform support', 'second open', 'open data', 'data mining', 'open call', 'change innovation.', 'decision tree', 'teleworking', 'd esign education', 'sustainability transition', 'dyscalculia', 'corporate marketing', 'digital transformation', 'social media support tools', 'bioprocessing', 'circular business', 'open banking', 'sediment transport', 'smes sustainability', 'rewarding', 'process innovation', 'transport engineering', 'business models social enterprises', 'accreditation', 'model evaluation', 'literary translation', 'innovate transform', 'model product', 'business ethics', 'modeling', 'csa upcirc', 'models theory', 'transportation planning', 'uptake circular', 'business model studies', 'ngo', 'data transformation']</t>
+          <t>['uptake circular', 'support smes', 'robotic innovation', 'business model studies', 'sustainability', 'business models social enterprises', 'dyscalculia', 'bioprocessing', 'csa upcirc', 'business model', 'innovate transform', 'rewarding', 'software development processes', 'environmental sustainability', 'sediment transport', 'sustainability transition', 'call boosting', 'social media support', 'transportation planning', 'migration', 'small medium enterprises', 'literary translation', 'd esign education', 'second open', 'change innovation.', 'open call', 'boosting uptake', 'inclusion', 'process innovation', 'data transformation', 'models theory', 'manufacturing systems', 'smes sustainability', 'circular business', 'transform support', 'accreditation', 'teleworking', 'digital transformation', 'transport engineering', 'upcirc second', 'model product', 'transition csa', 'data mining', 'business ethics', 'corporate marketing', 'strategic business management', 'production planning', 'modeling', 'open data', 'composition', 'model evaluation', 'decision tree', 'social media support tools', 'open banking', 'product process', 'ngo']</t>
         </is>
       </c>
     </row>
@@ -1682,7 +1682,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>['sustainability st', 'call european', 'eu missions', 'st open', 'excellence centres', 'civil society', 'growth development', 'urban society', 'ecosystem services', 'environmental sustainability', 'sustainability sustainable', 'sustainable eco', 'urban ecology', 'expanding european', 'quality management system', 'elias european', 'lighthouse ria', 'climate change', 'european network', 'network ai', 'society climate', 'city', 'sustainability', 'eco ecosystem', 'climate', 'aesthetics place', 'ai lighthouse', 'ecosystem', 'open data', 'european union', 'open call', 'european studies', 'management organization', 'eu law', 'urban design', 'teleworking', 'ria elias', 'centres expanding', 'lighthouse ai', 'society', 'cyber intelligence', 'growth', 'european ai', 'ecosystem urban', 'european integration', 'open banking', 'european lighthouse', 'europeanization', 'accreditation', 'artificial intelligence', 'change eu', 'european education area', 'sustainable cities', 'ai sustainability', 'coastal structures', 'mythology', 'artificial ecosystems', 'ai excellence', 'ngo', 'sustainable consumption']</t>
+          <t>['society', 'network ai', 'european network', 'sustainability', 'change eu', 'urban society', 'ria elias', 'eu law', 'european ai', 'sustainability sustainable', 'environmental sustainability', 'europeanization', 'urban ecology', 'expanding european', 'ai lighthouse', 'open call', 'european integration', 'city', 'ecosystem services', 'artificial intelligence', 'climate', 'sustainable cities', 'accreditation', 'sustainable consumption', 'urban design', 'quality management system', 'ai excellence', 'lighthouse ria', 'call european', 'artificial ecosystems', 'teleworking', 'sustainable eco', 'sustainability st', 'centres expanding', 'eu missions', 'growth', 'growth development', 'society climate', 'cyber intelligence', 'aesthetics place', 'coastal structures', 'ai sustainability', 'civil society', 'climate change', 'eco ecosystem', 'elias european', 'ecosystem urban', 'ecosystem', 'excellence centres', 'lighthouse ai', 'management organization', 'open data', 'european education area', 'st open', 'mythology', 'european union', 'open banking', 'european studies', 'ngo', 'european lighthouse']</t>
         </is>
       </c>
     </row>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>['ai data', 'intercultural communication', 'intersubjective aidriven', 'graphic representation', 'advanced motion control', 'robotics', 'inclusion', 'human robot', 'visual effect', 'business capabilities', 'social media presence', 'human behavior', 'interaction ai', 'advanced human', 'space perception', 'multimodal interaction', 'robotics advanced', 'industrial leadership', 'call intersubjective', 'jarvis open', 'advanced usercentric', 'open call', 'human development', 'open data', 'virtual/augmented reality', 'usercentric human', 'robotic collaboration', 'teleworking', 'artifical intelligence', 'robotic communication', 'erogenic aids', 'mobile applications', 'partnership ia', 'data robotics', 'robot interaction', 'robot collaborative', 'international organizations', 'open banking', 'psychosocial intervention', 'aidriven multimodal', 'animation', 'augmented reality', 'robotic coordination', 'software design', 'accreditation', 'artificial intelligence', 'social inclusion.', 'ia jarvis', 'multi-object recognition', 'software', 'leadership', 'interaction advanced', 'leadership ai', 'robotics partnership', 'collaborative applications', 'shakespeare', 'convergans clubs', 'audiovisual production', 'automation']</t>
+          <t>['robot collaborative', 'robotic collaboration', 'software design', 'visual effect', 'ia jarvis', 'industrial leadership', 'social inclusion.', 'leadership ai', 'interaction advanced', 'augmented reality', 'call intersubjective', 'human behavior', 'intersubjective aidriven', 'advanced usercentric', 'animation', 'aidriven multimodal', 'virtual/augmented reality', 'human robot', 'artifical intelligence', 'data robotics', 'international organizations', 'shakespeare', 'multi-object recognition', 'advanced human', 'open call', 'inclusion', 'intercultural communication', 'space perception', 'ai data', 'robotics advanced', 'advanced motion control', 'social media presence', 'artificial intelligence', 'accreditation', 'jarvis open', 'audiovisual production', 'leadership', 'usercentric human', 'human development', 'teleworking', 'erogenic aids', 'robotics', 'robotic coordination', 'psychosocial intervention', 'robotic communication', 'interaction ai', 'business capabilities', 'partnership ia', 'software', 'collaborative applications', 'robot interaction', 'open data', 'multimodal interaction', 'automation', 'robotics partnership', 'open banking', 'graphic representation', 'convergans clubs', 'mobile applications']</t>
         </is>
       </c>
     </row>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>['living labs', 'penology', 'labs livingsoill', 'space solutions', 'laboratory studies', 'soil health', 'solutions soil', 'livingsoill open', 'microbiology', 'aesthetics place', 'open data', 'open call', 'right city', 'health management', 'quality life', 'teleworking', 'health living', 'precision agriculture', 'biomedical', 'open banking', 'soil architecture', 'sustainable agriculture', 'poor soil characterization', 'crops living', 'public health', 'call healthy', 'seasonal agricultural work', 'healthy soil', 'cocreating solutions', 'permanent crops', 'family health', 'health law', 'soil permanent']</t>
+          <t>['penology', 'family health', 'public health', 'soil permanent', 'right city', 'livingsoill open', 'living labs', 'health management', 'health living', 'labs livingsoill', 'call healthy', 'open call', 'solutions soil', 'space solutions', 'soil health', 'open banking', 'soil architecture', 'teleworking', 'cocreating solutions', 'sustainable agriculture', 'poor soil characterization', 'aesthetics place', 'quality life', 'crops living', 'microbiology', 'healthy soil', 'permanent crops', 'open data', 'precision agriculture', 'biomedical', 'laboratory studies', 'seasonal agricultural work', 'health law']</t>
         </is>
       </c>
     </row>
@@ -1793,7 +1793,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>['plan fast', 'track market', 'mobilization', 'strategic business management', 'local food', 'urban planning', 'eit food', 'fit', 'volunteering', 'music', 'mechanical', 'market initiative', 'food waste', 'fast track', 'corporate marketing', 'marketing strategy', 'market policies', 'food heritage', 'food business', 'spring eit', 'performance', 'seasonal agricultural work', 'business plan', 'electric vehicles', 'functional foods', 'economics', 'business model studies', 'initiative spring', 'business history']</t>
+          <t>['market initiative', 'market policies', 'food heritage', 'functional foods', 'business history', 'business model studies', 'economics', 'fast track', 'initiative spring', 'performance', 'plan fast', 'fit', 'music', 'food waste', 'volunteering', 'spring eit', 'food business', 'mobilization', 'electric vehicles', 'business plan', 'eit food', 'track market', 'strategic business management', 'corporate marketing', 'urban planning', 'local food', 'marketing strategy', 'seasonal agricultural work', 'mechanical']</t>
         </is>
       </c>
     </row>
@@ -1830,7 +1830,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>['space infrastructure', 'cluster approach', 'services oscars', 'performance arts', 'electronic testing', 'eosc research', 'policy implementation', 'community development', 'laboratory studies', 'electronic commerce', 'build science', 'cinema', 'infrastructures research', 'open science', 'research methods', 'communities oscars', 'earth science', 'research communities', 'service marketing', 'open data', 'data mining', 'robotic validation', 'open call', 'call open', 'research society', 'teleworking', 'oscars nd', 'society', 'science projects', 'bioinformatics', 'engineering', 'education urban space / traffic)', 'electronic engineering design', 'theater', 'group dynamics', 'space coordination', 'open banking', 'clusters action', 'projects services', 'action research', 'environmental science', 'community studies', 'social media research', 'science cluster', 'accreditation', 'electronic payment services', 'biomedical research', 'uptake eosc', 'film', 'smart infrastructure', 'software project management', 'oscars open', 'nd open', 'transportation planning', 'research performance', 'convergans clubs', 'research infrastructures', 'science clusters', 'approach ensure', 'ensure uptake', 'technology society', 'social research', 'planetary science', 'highways railways infrastructure design construction']</t>
+          <t>['society', 'biomedical research', 'robotic validation', 'electronic payment services', 'electronic engineering design', 'science clusters', 'build science', 'social research', 'space coordination', 'research performance', 'nd open', 'services oscars', 'eosc research', 'research methods', 'bioinformatics', 'electronic testing', 'film', 'research infrastructures', 'science cluster', 'smart infrastructure', 'social media research', 'transportation planning', 'cinema', 'infrastructures research', 'oscars nd', 'open call', 'planetary science', 'projects services', 'earth science', 'approach ensure', 'uptake eosc', 'technology society', 'software project management', 'community studies', 'group dynamics', 'highways railways infrastructure design construction', 'community development', 'action research', 'electronic commerce', 'clusters action', 'accreditation', 'service marketing', 'laboratory studies', 'ensure uptake', 'oscars open', 'teleworking', 'communities oscars', 'policy implementation', 'performance arts', 'data mining', 'open science', 'research society', 'call open', 'education urban space / traffic)', 'theater', 'space infrastructure', 'open data', 'cluster approach', 'research communities', 'open banking', 'science projects', 'environmental science', 'convergans clubs', 'engineering']</t>
         </is>
       </c>
     </row>
@@ -1867,7 +1867,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>['performance arts', 'ui/ux', 'talents innonext', 'biotechnology innovation', 'initiative innovation', 'social media innovation', 'children', 'performing arts', 'change innovation.', 'performance improvisation', 'digital media children', 'initiative next', 'biotech innovation', 'cyber intelligence', 'creativity', 'creative industry', 'innonext next', 'film', 'artificial intelligence', 'talents initiative', 'generation innovation', 'demographic change', 'strategy', 'next generation', 'innovation talents', 'mems']</t>
+          <t>['biotech innovation', 'initiative next', 'innovation talents', 'generation innovation', 'innonext next', 'initiative innovation', 'film', 'change innovation.', 'artificial intelligence', 'talents initiative', 'strategy', 'social media innovation', 'demographic change', 'performance arts', 'cyber intelligence', 'biotechnology innovation', 'mems', 'ui/ux', 'next generation', 'performing arts', 'creative industry', 'creativity', 'performance improvisation', 'talents innonext', 'digital media children', 'children']</t>
         </is>
       </c>
     </row>
@@ -1904,7 +1904,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>['ria ngi', 'fund z', 'digital craft', 'growth development', 'zero emission', 'internet governance', 'digital culture', 'internet commons', 'fund ria', 'zero commons', 'green finance', 'spina bifida', 'zero emissions', 'generation internet', 'grow internet', 'ngi zero', 'children', 'aging', 'z create', 'commons fund', 'internet of things', 'digital media children', 'mature grow', 'growth', 'internet fund', 'international finance', 'coalition politics', 'lgbti', 'social media', 'electronic payment services', 'crowdfunding', 'developmental needs', 'macro', 'create mature', 'form', 'demographic change', 'next generation', 'ngo']</t>
+          <t>['electronic payment services', 'zero commons', 'developmental needs', 'macro', 'ngi zero', 'crowdfunding', 'zero emission', 'z create', 'social media', 'fund ria', 'form', 'fund z', 'spina bifida', 'zero emissions', 'mature grow', 'internet fund', 'commons fund', 'demographic change', 'aging', 'digital culture', 'international finance', 'growth development', 'growth', 'lgbti', 'generation internet', 'ria ngi', 'digital craft', 'next generation', 'grow internet', 'internet of things', 'coalition politics', 'create mature', 'internet commons', 'green finance', 'internet governance', 'digital media children', 'ngo', 'children']</t>
         </is>
       </c>
     </row>
@@ -1941,7 +1941,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>['freedom expression', 'freedom mobifree', 'call mobile', 'aircraft systems', 'internet governance', 'ia ngi', 'africa', 'digital culture', 'spina bifida', 'freedom association', 'generation internet', 'mobile freedom', 'ngi mobifree', 'internet things', 'aviation', 'children', 'mobile multimedia communication', 'open data', 'open call', 'internet of things', 'freedom art', 'mobile applications', 'teleworking', 'digital media children', 'pilots next', 'open banking', 'social media', 'lgbti', 'complex data analysis', 'internet ia', 'mobifree open', 'aviation management', 'demographic change', 'next generation', 'ngo']</t>
+          <t>['freedom mobifree', 'africa', 'call mobile', 'ngi mobifree', 'aircraft systems', 'aviation', 'open call', 'social media', 'internet things', 'pilots next', 'spina bifida', 'mobile multimedia communication', 'demographic change', 'internet ia', 'mobifree open', 'digital culture', 'teleworking', 'freedom art', 'ia ngi', 'complex data analysis', 'lgbti', 'generation internet', 'freedom association', 'next generation', 'freedom expression', 'aviation management', 'mobile freedom', 'internet of things', 'open data', 'open banking', 'internet governance', 'digital media children', 'ngo', 'children', 'mobile applications']</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>['play', 'composites', 'aircraft systems', 'internet governance', 'ia ngi', 'f fediversity', 'africa', 'digital humanities', 'digital culture', 'generation internet', 'african education', 'internet things', 'aviation', 'children', 'open data', 'open call', 'internet of things', 'teleworking', 'd esign education', 'digital media children', 'pilots next', 'open banking', 'fediversity open', 'vote', 'social media', 'lgbti', 'internet ia', 'nursing education', 'call f', 'ngi fediversity', 'educational buildings', 'aviation management', 'demographic change', 'next generation', 'ngo']</t>
+          <t>['play', 'fediversity open', 'africa', 'vote', 'ngi fediversity', 'f fediversity', 'aircraft systems', 'aviation', 'd esign education', 'open call', 'social media', 'internet things', 'pilots next', 'demographic change', 'composites', 'african education', 'internet ia', 'teleworking', 'digital culture', 'nursing education', 'ia ngi', 'call f', 'lgbti', 'generation internet', 'digital humanities', 'next generation', 'aviation management', 'internet of things', 'open data', 'educational buildings', 'open banking', 'internet governance', 'digital media children', 'ngo', 'children']</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>['living labs', 'mobilization', 'carbon footprint', 'carbon farming', 'laboratory studies', 'european soils', 'professional quality life', 'practices living', 'farming living', 'social constructionism', 'microbiology', 'labs open', 'mediterranean southern', 'home culture', 'healthy future', 'open data', 'call farmers', 'volunteering', 'open call', 'european union', 'project fostering', 'european studies', 'carbon capture', 'quality life', 'teleworking', 'global health', 'traditional mediterranean architecture', 'labs mediterranean', 'seas', 'farmers contribute', 'precision agriculture', 'biomedical', 'open banking', 'sustainable agriculture', 'soil architecture', 'construction management', 'poor soil characterization', 'lilassoils project', 'european education area', 'concordat', 'geopolymers', ' future work', 'school books', 'seasonal agricultural work', 'balkans', 'southern eu', 'farming practices', 'contribute lilassoils', 'fostering carbon', 'educational buildings', 'family health', 'eu healthy', 'future european', 'carbon reduction', 'carbon tax']</t>
+          <t>['healthy future', 'family health', 'eu healthy', 'seas', 'living labs', 'southern eu', 'future european', 'geopolymers', 'home culture', 'contribute lilassoils', 'european studies', 'open call', 'call farmers', 'fostering carbon', 'farming practices', 'european soils', 'volunteering', 'traditional mediterranean architecture', 'balkans', 'open banking', 'lilassoils project', 'mediterranean southern', 'mobilization', 'carbon farming', 'soil architecture', 'labs open', 'labs mediterranean', 'teleworking', 'carbon footprint', 'carbon capture', 'carbon tax', 'sustainable agriculture', 'construction management', 'poor soil characterization', 'farming living', 'farmers contribute', 'quality life', 'school books', 'microbiology', 'carbon reduction', 'educational buildings', 'open data', 'social constructionism', 'european education area', 'practices living', 'precision agriculture', 'concordat', 'european union', 'professional quality life', 'global health', 'biomedical', 'laboratory studies', ' future work', 'project fostering', 'seasonal agricultural work']</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2052,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>['cryptography framework', 'applied macro', 'framework energy', 'data security', 'call implement', 'policy implementation', 'pqreact open', 'cultural context', 'robotic implementation', 'towards quantumresistant', 'energy harvesting', 'method architectural design', 'quantum cryptography', 'open data', 'open call', 'quantum electronics', 'energy', 'change innovation.', 'teleworking', 'social change', 'cryptocurrencies', 'energy efficiency', 'transition towards', 'quantumresistant cryptography', 'post quantum', 'open banking', 'quantum computing algorithms', 'energy policy', 'implement post', 'cryptography pqreact', 'energy aware', 'quantum computing', 'bioreactors', 'contextual mapping', 'aware contexts', 'quantum mechanics', 'use design contexts']</t>
+          <t>['quantum computing algorithms', 'quantumresistant cryptography', 'towards quantumresistant', 'quantum electronics', 'post quantum', 'energy harvesting', 'cultural context', 'energy aware', 'applied macro', 'quantum computing', 'energy', 'aware contexts', 'change innovation.', 'open call', 'implement post', 'bioreactors', 'method architectural design', 'energy policy', 'cryptocurrencies', 'quantum mechanics', 'energy efficiency', 'teleworking', 'cryptography pqreact', 'cryptography framework', 'framework energy', 'policy implementation', 'robotic implementation', 'quantum cryptography', 'pqreact open', 'contextual mapping', 'use design contexts', 'call implement', 'open data', 'transition towards', 'data security', 'open banking', 'social change']</t>
         </is>
       </c>
     </row>
@@ -2089,7 +2089,7 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>['development economics', 'ai data', 'software development processes', 'ia fortis', 'fortis solution', 'growth development', 'space solutions', 'robotics', 'turkish military', 'human robot', 'visual effect', 'business capabilities', 'interaction ai', 'advanced human', 'call boosting', 'syria', 'robotics advanced', 'industrial leadership', 'open data', 'human development', 'open call', 'software development', 'decision tree', 'robotic collaboration', 'teleworking', 'artifical intelligence', 'multiaspect holistic', 'partnership ia', 'fortis open', 'data robotics', 'robot interaction', 'international organizations', 'open banking', 'multimodal multiaspect', 'rewarding', 'metaheuristic approaches', 'humanrobot interaction', 'boosting development', 'biological agents', 'lgbti', 'accreditation', 'artificial intelligence', 'multisensory design', 'solution multimodal', 'multi-object recognition', 'new buildins historical environments', 'leadership', 'robotic evaluation', 'leadership ai', 'robotics partnership', 'development fortis', 'holistic humanrobot', 'multicriteria decision making', 'contextual mapping', 'robotic solutions']</t>
+          <t>['robotic collaboration', 'visual effect', 'industrial leadership', 'biological agents', 'leadership ai', 'turkish military', 'rewarding', 'software development processes', 'humanrobot interaction', 'human robot', 'call boosting', 'artifical intelligence', 'data robotics', 'international organizations', 'development economics', 'multi-object recognition', 'advanced human', 'open call', 'ai data', 'robotics advanced', 'new buildins historical environments', 'robotic solutions', 'robotic evaluation', 'solution multimodal', 'artificial intelligence', 'fortis open', 'multiaspect holistic', 'accreditation', 'space solutions', 'leadership', 'syria', 'human development', 'teleworking', 'robotics', 'growth development', 'lgbti', 'multimodal multiaspect', 'interaction ai', 'boosting development', 'business capabilities', 'metaheuristic approaches', 'multisensory design', 'contextual mapping', 'partnership ia', 'development fortis', 'software development', 'open data', 'robot interaction', 'multicriteria decision making', 'fortis solution', 'robotics partnership', 'decision tree', 'open banking', 'holistic humanrobot', 'ia fortis']</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>['drones ecosystem', 'mechanical devices', 'physicalcyber agriforest', 'ecosystem services', 'environmental sustainability', 'drones multipurpose', 'environmental monitoring', 'robotics', 'inclusion', 'self-driving cars', 'values spade', 'multipurpose vehicle', 'mechanical components', 'mechanical equipment', 'call multipurpose', 'spade open', 'moral values', 'ecology', 'ecosystem', 'added values', 'open data', 'multipurpose physicalcyber', 'risks added', 'open call', 'teleworking', 'aerospace robotics', 'multicriteria decision making', 'governance environmental', 'transportation engineering', 'global environmental governance', 'precision agriculture', 'potential drones', 'open banking', 'stroke', 'environmental science', 'vehicle risks', 'sustainable agriculture', 'autonomous drones', 'ecosystem governance', 'multisensory design', 'solid mechanics', 'electric vehicles', 'environmental observation', 'risk assessment', 'values', 'multi-agent systems', 'bioreactors', 'environmental policy', 'agriforest drones', 'artificial ecosystems', 'risk management', 'robotic deployment']</t>
+          <t>['environmental science', 'environmental monitoring', 'spade open', 'multipurpose physicalcyber', 'risks added', 'potential drones', 'agriforest drones', 'environmental sustainability', 'call multipurpose', 'ecosystem governance', 'stroke', 'open call', 'inclusion', 'bioreactors', 'global environmental governance', 'governance environmental', 'solid mechanics', 'autonomous drones', 'ecosystem services', 'mechanical equipment', 'drones ecosystem', 'open banking', 'environmental policy', 'drones multipurpose', 'artificial ecosystems', 'environmental observation', 'electric vehicles', 'transportation engineering', 'teleworking', 'risk assessment', 'robotics', 'sustainable agriculture', 'ecology', 'robotic deployment', 'risk management', 'aerospace robotics', 'multisensory design', 'moral values', 'physicalcyber agriforest', 'ecosystem', 'values spade', 'mechanical devices', 'open data', 'values', 'mechanical components', 'multicriteria decision making', 'precision agriculture', 'self-driving cars', 'added values', 'multi-agent systems', 'vehicle risks', 'multipurpose vehicle']</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>['interact ia', 'cognitive learning', 'intercultural communication', 'reality ecosystem', 'higher education', 'ecosystem services', 'teaching robotics', 'robotics', 'extended reality', 'reality learning', 'ecology', 'nursing', 'virtual/augmented reality', 'open data', 'ecosystem', 'hybrid', 'open call', 'robotic fabrication processes', 'learning engage', 'robotic engineering', 'fairness', 'teleworking', 'communication', 'social media engagement', 'open banking', 'digital game', 'industrial robotics', 'call mixed', 'social media engagement tools', 'nuclear engineering', 'augmented reality', 'virtual reality', 'accreditation', 'mixed reality', 'master nd', 'nd open', 'robotics manufacturing', 'convergans clubs', 'engage interact', 'robotic education', 'ecosystem teaching', 'artificial ecosystems', 'automation', 'ia master', 'education']</t>
+          <t>['robotic engineering', 'ia master', 'digital game', 'engage interact', 'nd open', 'augmented reality', 'higher education', 'robotic education', 'virtual/augmented reality', 'industrial robotics', 'cognitive learning', 'intercultural communication', 'open call', 'mixed reality', 'reality ecosystem', 'robotic fabrication processes', 'accreditation', 'master nd', 'open banking', 'communication', 'nursing', 'artificial ecosystems', 'teleworking', 'social media engagement tools', 'robotics manufacturing', 'robotics', 'hybrid', 'virtual reality', 'ecology', 'education', 'extended reality', 'teaching robotics', 'learning engage', 'interact ia', 'ecosystem', 'ecosystem teaching', 'open data', 'fairness', 'nuclear engineering', 'reality learning', 'automation', 'social media engagement', 'call mixed', 'convergans clubs', 'ecosystem services']</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>['interest representation', 'deconstruction', 'chemical engineering', 'robotic assessment', 'durability', 'aging', 'fit', 'sea basin', 'open data', 'open call', 'associated regions', 'minimise remediate', 'open banking', 'electromagnetism', 'sustainable technology', 'actions prevent', 'oceanography', 'green technologies', 'optimization algorithms', 'theoretical physics', 'human geography', 'aiming assessing', 'algorithm optimization', 'marine technology', 'remediate chemical', 'air pollution control', 'call associated', 'responsive hub', 'cosmology', 'basin lighthouse', 'teleworking', 'geology', 'statistical physics', 'space support', 'balkans', 'preventive police powers', 'risk management', 'carbon reduction', 'space', 'lighthouse actions', 'destress mediterranean', 'inclusion', 'bioremediation', 'validity reliability', 'memory', 'free associations', 'pollution open', 'sea chemical', 'control', 'mediterranean sea', 'water purification', 'environmental economics', 'performance studies', 'quality life', 'hub long', 'optimization techniques', 'assessing replicability', 'remote sensing', 'rhemediation technologies', 'replicability exploitability', 'psychological assessment', 'european politics governance', 'signal integrity', 'performance', 'technologies rhemediation', 'african geography', 'term governance', 'coastal structures', 'strategy', 'recycling technologies', 'estuaries rivers (wave', 'internet governance', 'prevent minimise', 'technology', 'reliability', 'space governance', 'law sea', 'regions aiming', 'chemical pollution', 'human behavior', 'aesthetics place', 'exploitability potentials', 'governance destress', 'traditional mediterranean architecture', 'seas', 'corporate governance', 'distributed computing', 'environmental science', 'theory restoration', 'micromobility', 'potentials rhemediation', 'egovernment', 'long term', 'rhemediation responsive', 'environmental policy']</t>
+          <t>['sustainable technology', 'water purification', 'human behavior', 'law sea', 'distributed computing', 'inclusion', 'space', 'minimise remediate', 'traditional mediterranean architecture', 'destress mediterranean', 'potentials rhemediation', 'chemical pollution', 'aging', 'hub long', 'coastal structures', 'carbon reduction', 'geology', 'open data', 'validity reliability', 'estuaries rivers (wave', 'european politics governance', 'chemical engineering', 'seas', 'recycling technologies', 'oceanography', 'interest representation', 'free associations', 'long term', 'lighthouse actions', 'preventive police powers', 'open call', 'sea basin', 'control', 'governance destress', 'space governance', 'risk management', 'prevent minimise', 'technology', 'open banking', 'statistical physics', 'signal integrity', 'theoretical physics', 'air pollution control', 'green technologies', 'algorithm optimization', 'replicability exploitability', 'actions prevent', 'robotic assessment', 'mediterranean sea', 'pollution open', 'african geography', 'rhemediation technologies', 'theory restoration', 'strategy', 'basin lighthouse', 'rhemediation responsive', 'corporate governance', 'environmental economics', 'aesthetics place', 'quality life', 'egovernment', 'call associated', 'reliability', 'performance studies', 'sea chemical', 'micromobility', 'responsive hub', 'durability', 'remote sensing', 'memory', 'marine technology', 'cosmology', 'associated regions', 'performance', 'optimization techniques', 'fit', 'bioremediation', 'space support', 'technologies rhemediation', 'electromagnetism', 'remediate chemical', 'balkans', 'environmental policy', 'aiming assessing', 'optimization algorithms', 'teleworking', 'human geography', 'assessing replicability', 'deconstruction', 'psychological assessment', 'exploitability potentials', 'regions aiming', 'internet governance', 'term governance', 'environmental science']</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2237,7 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>['eu missions', 'civil society', 'urban society', 'ecosystem services', 'environmental sustainability', 'missions innovation', 'sustainable eco', 'urban ecology', 'critical mapping', 'biotechnology innovation', 'climate change', 'icapital horizoneicprize', 'society climate', 'sustainability', 'climate', 'eco ecosystem', 'ecosystem', 'european union', 'capital markets law', 'change innovation.', 'eu law', 'urban design', 'black hole physics', 'optimization techniques', 'capital innovation', 'society', 'biotech innovation', 'european integration', 'ecosystem urban', 'rewarding', 'europeanization', 'award icapital', 'accreditation', 'change eu', 'innovation award', 'european capital', 'space innovation', 'european education area', 'sustainable cities', 'horizoneicprize horizoneicprize', 'horizoneicprize sustainable', 'evaluation', 'optimization algorithms', 'artificial ecosystems', 'icapital european', 'einstein finsler metrics', 'sustainable consumption']</t>
+          <t>['biotech innovation', 'society', 'evaluation', 'sustainability', 'change eu', 'capital markets law', 'urban society', 'critical mapping', 'missions innovation', 'eu law', 'rewarding', 'environmental sustainability', 'europeanization', 'innovation award', 'urban ecology', 'optimization techniques', 'change innovation.', 'einstein finsler metrics', 'european integration', 'space innovation', 'climate', 'sustainable cities', 'accreditation', 'sustainable consumption', 'capital innovation', 'urban design', 'optimization algorithms', 'artificial ecosystems', 'sustainable eco', 'icapital horizoneicprize', 'eu missions', 'society climate', 'award icapital', 'biotechnology innovation', 'civil society', 'climate change', 'eco ecosystem', 'ecosystem urban', 'ecosystem', 'horizoneicprize horizoneicprize', 'icapital european', 'european education area', 'horizoneicprize sustainable', 'european union', 'european capital', 'ecosystem services', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2274,7 @@
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>['eu missions', 'civil society', 'urban society', 'performance arts', 'ecosystem services', 'environmental sustainability', 'missions innovation', 'sustainable eco', 'urban ecology', 'critical mapping', 'biotechnology innovation', 'climate change', 'icapital horizoneicprize', 'society climate', 'sustainability', 'climate', 'eco ecosystem', 'ecosystem', 'european union', 'capital markets law', 'rising european', 'change innovation.', 'urban design', 'black hole physics', 'eu law', 'optimization techniques', 'capital innovation', 'society', 'biotech innovation', 'european integration', 'ecosystem urban', 'rewarding', 'europeanization', 'award icapital', 'reputation', 'awards rising', 'accreditation', 'change eu', 'innovation award', 'european capital', 'space innovation', 'european education area', 'sustainable cities', 'horizoneicprize horizoneicprize', 'innovation awards', 'horizoneicprize sustainable', 'evaluation', 'optimization algorithms', 'artificial ecosystems', 'einstein finsler metrics', 'sustainable consumption']</t>
+          <t>['awards rising', 'biotech innovation', 'society', 'evaluation', 'sustainability', 'change eu', 'capital markets law', 'urban society', 'critical mapping', 'missions innovation', 'eu law', 'rewarding', 'environmental sustainability', 'reputation', 'innovation award', 'europeanization', 'urban ecology', 'optimization techniques', 'change innovation.', 'einstein finsler metrics', 'innovation awards', 'european integration', 'space innovation', 'climate', 'sustainable cities', 'accreditation', 'sustainable consumption', 'capital innovation', 'urban design', 'optimization algorithms', 'artificial ecosystems', 'sustainable eco', 'icapital horizoneicprize', 'eu missions', 'performance arts', 'society climate', 'award icapital', 'biotechnology innovation', 'civil society', 'climate change', 'eco ecosystem', 'ecosystem urban', 'ecosystem', 'horizoneicprize horizoneicprize', 'rising european', 'european education area', 'horizoneicprize sustainable', 'european union', 'european capital', 'ecosystem services', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -2311,7 +2311,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>['related regional', 'interest representation', 'community water', 'support related', 'business model', 'urban planning', 'ocean energy', 'sustainable innovation', 'biotechnology innovation', 'marine ocean', 'challenges integrated', 'african education', 'integrated circuits', 'entrepreneurship', 'maritime security', 'european union', 'strategies sustainable', 'european studies', 'mechanical engineering support', 'maritime sectors', 'technological innovation', 'open banking', 'competitive strategies', 'robotic training', 'd esign management', 'support services', 'social media services', 'innovation management', 'solutions maritime', 'sme startup', 'sustainable technology', 'institute innovation', 'model innovation', 'regional development', 'related industrial', 'models theory', 'oceanography', 'system design', 'sectors ecosystems', 'maritime challenges', 'management innovation', 'human geography', 'smart electronics', 'call proposals', 'smart specialisation', 'small medium enterprises', 'marine technology', 'freshwater hydrosphere', 'operations research', 'higher education', 'deep ecology', 'innovation support', 'community development', 'smart systems', 'innovation smart', 'specialisation strategies', 'management marketcreating', 'social media innovation', 'water technology', 'marketcreating innovation', 'robotic support', 'policy analysis', 'software development', 'teleworking', 'product innovation', 'ecosystems horizoneit', 'information technology', 'biotech innovation', 'disruptive innovation', 'water management', 'horizoneitkicwater business', 'geology', 'mechanical engineering integration', 'innovation technology', 'marine maritime', 'horizoneit horizoneitkicwater', 'community studies', 'community health', 'management water', 'innovation technological', 'electronic devices', 'hydropower', 'training water', 'industrial data', 'hydrosphere freshwater', 'smart infrastructure', 'biotech startups', 'balkans', 'european institute', 'knowledge innovation', 'innovative solutions', 'service innovation', 'innovation related', 'social media platforms', 'technology knowledge', 'business model studies', 'policy related', 'marketing strategy', 'education', 'consortium eit', 'education hydrosphere', 'innovation vocational', 'social media support', 'systems engineering', 'community eit', 'ecosystem services', 'robotic innovation', 'electronic commerce', 'green finance', 'systems innovative', 'strategies innovation', 'related sme', 'urban communication', 'sustainability', 'open innovation', 'innovation disruptive', 'water purification', 'service marketing', 'water marine', 'health management', 'change innovation.', 'management organization', 'd esign education', 'marine ecosystem', 'industrial engineering', 'mechanical engineering innovation', 'water resources engineering', 'international organizations', 'social networks', 'europeanization', 'business models social enterprises', 'innovation open', 'hydrosphere marine', 'african geography', 'innovation strategies', 'innovation product', 'proposals consortium', 'economic development', 'space education', 'artificial ecosystems', 'strategy', 'irregular maritime migration', 'industrial design', 'startup support', 'software development processes', 'innovation systems', 'technology', 'ocean innovation', 'policy implementation', 'sustainable development', 'digital marketing', 'social services', 'eit kics', 'kics european', 'ecosystem', 'eit call', 'development service', 'eit community', 'ocean management', 'natural resource management', 'educational technologies', 'corporate marketing', 'seas', 'integrated management', 'european integration', 'innovation higher', 'mechanical engineering training', 'coalition politics', 'industrial policy', 'vocational training', 'electronic payment services', 'services innovation', 'innovation community', 'economic policy', 'european education area', 'strategic management', 'international development', 'water eit', 'maritime delimitation']</t>
+          <t>['sustainable technology', 'water purification', 'strategic management', 'hydrosphere marine', 'solutions maritime', 'innovation smart', 'digital marketing', 'ocean innovation', 'open innovation', 'sectors ecosystems', 'economic development', 'social media services', 'higher education', 'robotic training', 'eit community', 'horizoneitkicwater business', 'change innovation.', 'management marketcreating', 'policy analysis', 'community development', 'innovation product', 'mechanical engineering support', 'urban communication', 'development service', 'african education', 'artificial ecosystems', 'water eit', 'water marine', 'geology', 'management organization', 'strategies innovation', 'systems engineering', 'green finance', 'maritime delimitation', 'information technology', 'regional development', 'ecosystem services', 'innovation related', 'electronic payment services', 'freshwater hydrosphere', 'educational technologies', 'smart systems', 'biotech startups', 'seas', 'operations research', 'consortium eit', 'european institute', 'health management', 'software development processes', 'ocean energy', 'oceanography', 'interest representation', 'social media support', 'electronic devices', 'international organizations', 'd esign education', 'disruptive innovation', 'european integration', 'sustainable development', 'proposals consortium', 'ocean management', 'service marketing', 'water technology', 'natural resource management', 'management water', 'innovation technology', 'institute innovation', 'entrepreneurship', 'biotechnology innovation', 'education', 'competitive strategies', 'vocational training', 'service innovation', 'related industrial', 'strategies sustainable', 'sustainable innovation', 'innovation vocational', 'marketcreating innovation', 'eit kics', 'technology', 'european union', 'system design', 'space education', 'open banking', 'innovation technological', 'robotic innovation', 'industrial design', 'innovation management', 'sme startup', 'business models social enterprises', 'sustainability', 'marine ecosystem', 'marine ocean', 'industrial data', 'smart infrastructure', 'innovation community', 'water management', 'education hydrosphere', 'innovation support', 'support related', 'integrated circuits', 'management innovation', 'african geography', 'community studies', 'mechanical engineering training', 'systems innovative', 'electronic commerce', 'social media innovation', 'community water', 'strategy', 'related sme', 'robotic support', 'support services', 'social services', 'industrial policy', 'deep ecology', 'water resources engineering', 'integrated management', 'corporate marketing', 'model innovation', 'innovation open', 'technological innovation', 'industrial engineering', 'ecosystem', 'software development', 'smart electronics', 'coalition politics', 'innovation higher', 'hydropower', 'social networks', 'policy related', 'innovation systems', 'european studies', 'biotech innovation', 'business model studies', 'mechanical engineering innovation', 'community eit', 'business model', 'marine technology', 'technology knowledge', 'challenges integrated', 'maritime challenges', 'innovation disruptive', 'europeanization', 'small medium enterprises', 'community health', 'horizoneit horizoneitkicwater', 'marketing strategy', 'startup support', 'models theory', 'eit call', 'marine maritime', 'smart specialisation', 'knowledge innovation', 'd esign management', 'international development', 'balkans', 'services innovation', 'economic policy', 'kics european', 'maritime security', 'teleworking', 'maritime sectors', 'ecosystems horizoneit', 'mechanical engineering integration', 'policy implementation', 'product innovation', 'training water', 'innovative solutions', 'urban planning', 'related regional', 'innovation strategies', 'social media platforms', 'human geography', 'call proposals', 'european education area', 'specialisation strategies', 'irregular maritime migration', 'hydrosphere freshwater']</t>
         </is>
       </c>
     </row>
@@ -2348,7 +2348,7 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>['atm impact', 'arbitration', 'galactic astronomy', 'change digital', 'impact climate', 'research methods', 'climate change', 'climate', 'digital european', 'sky exploratory', 'european union', 'quantitative finance', 'exploratory research', 'digital transformation', 'qualitative research', 'european sky', 'research horizonsesardeserwa', 'digitalization', 'banking', 'horizonsesardeserwa horizonsesardeser', 'astrophysics', 'digital', 'social research', 'planetary science', 'space research']</t>
+          <t>['social research', 'quantitative finance', 'digital european', 'research methods', 'horizonsesardeserwa horizonsesardeser', 'planetary science', 'exploratory research', 'sky exploratory', 'climate', 'european sky', 'arbitration', 'change digital', 'digital', 'qualitative research', 'digital transformation', 'astrophysics', 'galactic astronomy', 'climate change', 'impact climate', 'banking', 'digitalization', 'atm impact', 'european union', 'research horizonsesardeserwa', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2385,7 +2385,7 @@
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'digital humanities', 'research methods', 'quantitative research', 'digital european', 'sky exploratory', 'european union', 'exploratory research', 'digital media', 'topics digital', 'qualitative research', 'european sky', 'research horizonsesardeserwa', 'digitalization', 'research topics', 'fundamental research', 'horizonsesardeserwa horizonsesardeser', 'astrophysics', 'digital', 'social research', 'planetary science', 'space research']</t>
+          <t>['social research', 'digital european', 'research methods', 'horizonsesardeserwa horizonsesardeser', 'planetary science', 'exploratory research', 'sky exploratory', 'topics digital', 'european sky', 'research topics', 'digital', 'qualitative research', 'astrophysics', 'galactic astronomy', 'digital media', 'digital humanities', 'fundamental research', 'digitalization', 'quantitative research', 'european union', 'research horizonsesardeserwa', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>['research help', 'galactic astronomy', 'regulatory biotechnology', 'physical modeling', 'framework des', '3d design', 'regulatory framework', 'shape future', 'research methods', 'cae methodology development', 'digital european', 'sky exploratory', 'data protection regulation', 'european union', 'fractal geometry', 'exploratory research', 'd esign education', 'help shape', 'des digital', 'future regulatory', 'biotechnology policy', 'qualitative research', 'european sky', 'digital', 'd esign management', 'digital company', 'research horizonsesardeserwa', 'government regulations', 'digitalization', 'modeling', 'horizonsesardeserwa horizonsesardeser', 'astrophysics', ' future work', 'social research', 'planetary science', 'space research']</t>
+          <t>['des digital', 'social research', 'data protection regulation', 'digital european', 'research methods', 'regulatory framework', 'horizonsesardeserwa horizonsesardeser', 'biotechnology policy', 'cae methodology development', 'd esign education', 'planetary science', 'exploratory research', 'sky exploratory', 'd esign management', 'physical modeling', 'european sky', 'research help', 'help shape', 'framework des', 'digital', 'government regulations', 'qualitative research', 'astrophysics', 'galactic astronomy', 'space research', 'fractal geometry', 'digital company', '3d design', 'future regulatory', 'modeling', 'digitalization', 'shape future', 'regulatory biotechnology', 'european union', 'research horizonsesardeserwa', ' future work']</t>
         </is>
       </c>
     </row>
@@ -2459,7 +2459,7 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'aircraft systems', 'zero emission', 'generation aircraft', 'space integration', 'zero emissions', 'research methods', 'aviation', 'digital european', 'children', 'sky exploratory', 'european union', 'exploratory research', 'digital media children', 'emission aviation', 'aerospace engineering', 'radiation physics', 'qualitative research', 'aircraft zerolow', 'aviation digital', 'european sky', 'research horizonsesardeserwa', 'digitalization', 'horizonsesardeserwa horizonsesardeser', 'aviation management', 'astrophysics', 'integration next', 'zerolow emission', 'demographic change', 'next generation', 'digital', 'social research', 'planetary science', 'space research']</t>
+          <t>['emission aviation', 'social research', 'digital european', 'integration next', 'radiation physics', 'research methods', 'horizonsesardeserwa horizonsesardeser', 'zero emission', 'aircraft systems', 'aircraft zerolow', 'space integration', 'aviation', 'planetary science', 'exploratory research', 'zerolow emission', 'sky exploratory', 'european sky', 'generation aircraft', 'zero emissions', 'demographic change', 'aerospace engineering', 'aviation digital', 'digital', 'qualitative research', 'astrophysics', 'galactic astronomy', 'next generation', 'aviation management', 'digitalization', 'european union', 'research horizonsesardeserwa', 'space research', 'digital media children', 'children']</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>['sensing computing', 'computation based design', 'applied macro', 'galactic astronomy', 'computing applied', 'computational theory', 'research methods', 'digital european', 'sky exploratory', 'european union', 'quantum electronics', 'applied atm', 'exploratory research', 'quantitative finance', 'investigate quantum', 'qualitative research', 'sensor reader circuits', 'sensors', 'european sky', 'sensor networks', 'computational design', 'research horizonsesardeserwa', 'digital services', 'digitalization', 'banking', 'digital systems', 'quantum sensing', 'horizonsesardeserwa horizonsesardeser', 'astrophysics', 'quantum computing', 'atm digital', 'quantum mechanics', 'digital', 'social research', 'planetary science', 'space research']</t>
+          <t>['social research', 'quantum sensing', 'quantum electronics', 'atm digital', 'quantitative finance', 'investigate quantum', 'digital european', 'research methods', 'sensors', 'sensor reader circuits', 'quantum computing', 'applied macro', 'horizonsesardeserwa horizonsesardeser', 'sensor networks', 'planetary science', 'exploratory research', 'computing applied', 'sky exploratory', 'european sky', 'computational design', 'computation based design', 'quantum mechanics', 'digital', 'qualitative research', 'astrophysics', 'galactic astronomy', 'computational theory', 'applied atm', 'banking', 'digitalization', 'digital services', 'digital systems', 'european union', 'sensing computing', 'research horizonsesardeserwa', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'airports', 'flight rules', 'research methods', 'aviation', 'digital european', 'sky exploratory', 'european union', 'digital flight', 'digital law', 'exploratory research', 'rules digital', 'qualitative research', 'digital game', 'european sky', 'research horizonsesardeserwa', 'digitalization', 'horizonsesardeserwa horizonsesardeser', 'aviation management', 'astrophysics', 'digital', 'social research', 'planetary science', 'space research']</t>
+          <t>['social research', 'digital game', 'digital flight', 'digital law', 'digital european', 'flight rules', 'research methods', 'horizonsesardeserwa horizonsesardeser', 'aviation', 'planetary science', 'exploratory research', 'sky exploratory', 'airports', 'european sky', 'digital', 'qualitative research', 'astrophysics', 'galactic astronomy', 'aviation management', 'digitalization', 'rules digital', 'european union', 'research horizonsesardeserwa', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2570,7 +2570,7 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>['transformation trajectorybased', 'galactic astronomy', 'operations digital', 'space research', 'sky industrial', 'trajectorybased operations', 'aviation', 'digital european', 'european union', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'space coordination', 'european sky', 'digital company', 'digital services', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'digitalization', 'astrophysics', 'dynamical systems', 'digital', 'data transformation', 'planetary science', 'industrial design']</t>
+          <t>['industrial design', 'space coordination', 'dynamical systems', 'sky industrial', 'digital european', 'industrial data', 'research horizonsesardesirwa', 'aviation', 'planetary science', 'data transformation', 'european sky', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'astrophysics', 'galactic astronomy', 'trajectorybased operations', 'operations digital', 'digital company', 'industrial engineering', 'transformation trajectorybased', 'digitalization', 'digital services', 'european union', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'airports', 'automated atm', 'space research', 'atm airspace', 'sky industrial', 'airspace users', 'aviation', 'digital european', 'european union', 'automation', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'machine automation', 'airport access', 'european sky', 'automated systems', 'users digital', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'digitalization', 'banking', 'astrophysics', 'highly automated', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['atm airspace', 'airspace users', 'automated systems', 'industrial design', 'sky industrial', 'digital european', 'highly automated', 'airport access', 'industrial data', 'research horizonsesardesirwa', 'aviation', 'planetary science', 'airports', 'european sky', 'automated atm', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'machine automation', 'astrophysics', 'galactic astronomy', 'industrial engineering', 'banking', 'digitalization', 'automation', 'european union', 'users digital', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>['neuroscience', 'galactic astronomy', 'cns capabilities', 'biomedical electronics', 'space research', 'sky industrial', 'enhanced cns', 'aviation', 'digital european', 'capabilities digital', 'european union', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'european sky', 'cad/cam technologies', 'horizonsesardesirwa horizonsesardesir', 'industrial data', 'digitalization', 'astrophysics', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['capabilities digital', 'industrial design', 'cad/cam technologies', 'sky industrial', 'cns capabilities', 'digital european', 'industrial data', 'neuroscience', 'research horizonsesardesirwa', 'enhanced cns', 'aviation', 'planetary science', 'european sky', 'biomedical electronics', 'aerospace engineering', 'space industry', 'horizonsesardesirwa horizonsesardesir', 'digital', 'industrial research', 'astrophysics', 'galactic astronomy', 'industrial engineering', 'digitalization', 'european union', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2681,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>['impunity', 'hinfinity control', 'mobility iam', 'space transportation', 'galactic astronomy', 'operations digital', 'aircraft systems', 'operations research', 'space research', 'sky industrial', 'digital trace', 'air pollution control', 'land reclamation', 'rocket propulsion', 'biotechnology innovation', 'social media innovation', 'aviation', 'digital european', 'fit', 'documentary', 'mode choice', 'european union', 'uncrewed operations', 'change innovation.', 'television series', 'space industry', 'industrial engineering', 'crewed uncrewed', 'aerospace engineering', 'air mobility', 'industrial research', 'enabling innovative', 'research horizonsesardesirwa', 'transportation engineering', 'capable aircraft', 'education urban space / traffic)', 'industrial design', 'fasttrack enabling', 'aircraft vca', 'european sky', 'discipline', 'creative labor', 'vca crewed', 'innovative air', 'digital company', 'space innovation', 'digital services', 'horizonsesardesirwa horizonsesardesir', 'industrial data', 'digitalization', 'takeoff landing', 'iam vertical', 'documentary cinema', 'transportation planning', 'vertical takeoff', 'aviation management', 'astrophysics', 'landing capable', 'digital', 'planetary science', 'mems']</t>
+          <t>['vca crewed', 'vertical takeoff', 'capable aircraft', 'industrial design', 'innovative air', 'air pollution control', 'enabling innovative', 'sky industrial', 'operations research', 'air mobility', 'digital european', 'discipline', 'fasttrack enabling', 'creative labor', 'industrial data', 'impunity', 'research horizonsesardesirwa', 'space transportation', 'transportation planning', 'aircraft systems', 'aviation', 'change innovation.', 'fit', 'mobility iam', 'landing capable', 'planetary science', 'uncrewed operations', 'mode choice', 'space innovation', 'land reclamation', 'rocket propulsion', 'european sky', 'takeoff landing', 'social media innovation', 'aircraft vca', 'hinfinity control', 'documentary cinema', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'transportation engineering', 'astrophysics', 'galactic astronomy', 'documentary', 'iam vertical', 'operations digital', 'digital company', 'biotechnology innovation', 'mems', 'education urban space / traffic)', 'industrial engineering', 'aviation management', 'digital services', 'television series', 'digitalization', 'european union', 'crewed uncrewed', 'space research', 'digital trace']</t>
         </is>
       </c>
     </row>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'airports', 'airports airports', 'passenger experience', 'space research', 'graph theory', 'sky industrial', 'digital culture', 'experience design', 'aviation', 'digital european', 'nodes passenger', 'experience digital', 'generative algorithms', 'european union', 'smart airports', 'airports multimodal', 'space industry', 'industrial engineering', 'aerospace engineering', 'multimodal nodes', 'industrial research', 'smart city', 'research horizonsesardesirwa', 'transportation engineering', 'airport access', 'customer experience', 'european sky', 'multisensory design', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'multi-object recognition', 'digitalization', 'electric vehicles', 'transportation planning', 'astrophysics', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['passenger experience', 'industrial design', 'customer experience', 'sky industrial', 'multimodal nodes', 'digital european', 'airport access', 'experience digital', 'industrial data', 'research horizonsesardesirwa', 'airports multimodal', 'transportation planning', 'graph theory', 'aviation', 'multi-object recognition', 'planetary science', 'airports', 'european sky', 'experience design', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'electric vehicles', 'transportation engineering', 'digital culture', 'astrophysics', 'galactic astronomy', 'multisensory design', 'smart airports', 'industrial engineering', 'generative algorithms', 'digitalization', 'nodes passenger', 'smart city', 'european union', 'airports airports', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'social media support', 'space deployment', 'space research', 'deployment planning', 'urban planning', 'sky industrial', 'digital trace', 'programme execution', 'support programme', 'planning design', 'aviation', 'digital european', 'disabled care)', 'european union', 'architecture strategic', 'execution sesar', 'mechanical engineering support', 'sesar architecture', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'criminal criminal procedure law', 'architectural design', 'monitoring digital', 'bioprocessing', 'european sky', 'software design', 'criminal procedure law', 'planning monitoring', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'strategic management', 'digitalization', 'software', 'digital systems', 'strategic deployment', 'astrophysics', 'architectural design.', 'architecture', 'robotic deployment', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['strategic management', 'software design', 'industrial design', 'sky industrial', 'bioprocessing', 'digital european', 'architecture strategic', 'programme execution', 'industrial data', 'research horizonsesardesirwa', 'space deployment', 'social media support', 'aviation', 'strategic deployment', 'planetary science', 'support programme', 'sesar architecture', 'deployment planning', 'mechanical engineering support', 'european sky', 'criminal criminal procedure law', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'disabled care)', 'digital', 'industrial research', 'astrophysics', 'galactic astronomy', 'architecture', 'execution sesar', 'criminal procedure law', 'monitoring digital', 'robotic deployment', 'urban planning', 'industrial engineering', 'software', 'digitalization', 'planning monitoring', 'digital systems', 'european union', 'planning design', 'architectural design.', 'space research', 'digital trace', 'architectural design']</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2792,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'social media support', 'space research', 'sky industrial', 'programme execution', 'support programme', 'aviation', 'digital european', 'disabled care)', 'european union', 'performance studies', 'performance based design', 'mechanical engineering support', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'bioprocessing', 'european sky', 'software design', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'performance', 'digitalization', 'software', 'execution framework', 'digital systems', 'performance digital', 'framework performance', 'astrophysics', 'architecture', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['performance digital', 'software design', 'industrial design', 'sky industrial', 'bioprocessing', 'digital european', 'programme execution', 'industrial data', 'research horizonsesardesirwa', 'social media support', 'performance', 'aviation', 'planetary science', 'support programme', 'mechanical engineering support', 'european sky', 'framework performance', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'disabled care)', 'performance based design', 'industrial research', 'digital', 'astrophysics', 'galactic astronomy', 'architecture', 'execution framework', 'industrial engineering', 'software', 'digitalization', 'digital systems', 'european union', 'performance studies', 'space research']</t>
         </is>
       </c>
     </row>
@@ -2829,7 +2829,7 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>['youth work', 'galactic astronomy', 'platform airport', 'operations digital', 'airports', 'space research', 'airport operations', 'genetic predisposition', 'sky industrial', 'ats platform', 'aviation', 'digital european', 'children', 'information systems', 'european union', 'digital media children', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'airport access', 'european sky', 'generation ats', 'platform employees', 'digital company', 'digital services', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'digitalization', 'aviation management', 'astrophysics', 'demographic change', 'social media platforms', 'next generation', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['ats platform', 'information systems', 'industrial design', 'sky industrial', 'digital european', 'airport access', 'industrial data', 'research horizonsesardesirwa', 'aviation', 'generation ats', 'planetary science', 'genetic predisposition', 'airports', 'european sky', 'demographic change', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'astrophysics', 'galactic astronomy', 'operations digital', 'digital company', 'social media platforms', 'industrial engineering', 'platform employees', 'next generation', 'aviation management', 'airport operations', 'digital services', 'digitalization', 'european union', 'youth work', 'platform airport', 'space research', 'digital media children', 'children']</t>
         </is>
       </c>
     </row>
@@ -2866,7 +2866,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>['capabilities supporting', 'galactic astronomy', 'aircraft systems', 'carbon footprint', 'architectural digital design', 'environmental sustainability', 'space research', 'environmental footprint', 'sky industrial', 'embedded technologies', 'business capabilities', 'disadvantaged groups', 'sustainability', 'aviation', 'digital european', 'european union', 'environmental economics', 'robotic support', 'footprint digital', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'airborne capabilities', 'european sky', 'environmental science', 'atm environmental', 'waste management', 'horizonsesardesirwa horizonsesardesir', 'industrial data', 'digitalization', 'banking', 'supporting reducing', 'reducing atm', 'aviation management', 'environmental policy', 'astrophysics', 'carbon reduction', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['sustainability', 'waste management', 'industrial design', 'sky industrial', 'reducing atm', 'digital european', 'architectural digital design', 'industrial data', 'environmental sustainability', 'research horizonsesardesirwa', 'capabilities supporting', 'supporting reducing', 'aircraft systems', 'aviation', 'planetary science', 'atm environmental', 'european sky', 'disadvantaged groups', 'environmental policy', 'airborne capabilities', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'robotic support', 'environmental economics', 'carbon footprint', 'astrophysics', 'galactic astronomy', 'space research', 'business capabilities', 'industrial engineering', 'carbon reduction', 'banking', 'aviation management', 'digitalization', 'footprint digital', 'european union', 'embedded technologies', 'environmental science', 'environmental footprint']</t>
         </is>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>['youth work', 'galactic astronomy', 'operations digital', 'airports', 'operations research', 'space research', 'genetic predisposition', 'sky industrial', 'multipurpose / hybrid offshore platforms', 'aviation', 'digital european', 'children', 'information systems', 'european union', 'platforms enroute', 'twitter', 'digital media children', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'airport access', 'european sky', 'generation ats', 'digital', 'tma operations', 'platform employees', 'digital company', 'digital services', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'digitalization', 'enroute tma', 'astrophysics', 'demographic change', 'social media platforms', 'next generation', 'ats platforms', 'planetary science', 'industrial design']</t>
+          <t>['tma operations', 'platforms enroute', 'information systems', 'industrial design', 'sky industrial', 'operations research', 'twitter', 'digital european', 'airport access', 'industrial data', 'research horizonsesardesirwa', 'multipurpose / hybrid offshore platforms', 'aviation', 'generation ats', 'planetary science', 'genetic predisposition', 'airports', 'european sky', 'demographic change', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'ats platforms', 'astrophysics', 'galactic astronomy', 'operations digital', 'digital company', 'social media platforms', 'industrial engineering', 'platform employees', 'next generation', 'digitalization', 'digital services', 'european union', 'enroute tma', 'youth work', 'space research', 'digital media children', 'children']</t>
         </is>
       </c>
     </row>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>['spacecraft design', 'galactic astronomy', 'technology business', 'market commercial', 'space research', 'technology', 'labor market', 'graph theory', 'electromagnetic interference', 'sky industrial', 'horizonsesardesir technology', 'multilink digital', 'airground connectivity', 'aviation', 'digital european', 'business market', 'service marketing', 'european union', 'performance studies', 'space monitoring', 'change innovation.', 'performance based design', 'network analysis', 'space industry', 'social change', 'industrial engineering', 'aerospace engineering', 'information technology', 'industrial research', 'high performance', 'wireless communication', 'research horizonsesardesirwa', 'corporate marketing', 'transition towards', 'european sky', 'digital', 'space exploration technologies', 'space technology', 'wireless technology', 'digital services', 'horizonsesardesirwa horizonsesardesir', 'performance airground', 'high energy physics', 'performance', 'digitalization', 'industrial data', 'technology society', 'digital communication', 'advertising', 'astrophysics', 'strategy', 'connectivity multilink', 'towards high', 'planetary science', 'industrial design']</t>
+          <t>['industrial design', 'business market', 'sky industrial', 'digital european', 'high performance', 'wireless technology', 'industrial data', 'technology business', 'research horizonsesardesirwa', 'performance', 'graph theory', 'aviation', 'change innovation.', 'information technology', 'planetary science', 'technology society', 'space exploration technologies', 'european sky', 'strategy', 'electromagnetic interference', 'service marketing', 'aerospace engineering', 'airground connectivity', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'performance based design', 'digital', 'multilink digital', 'industrial research', 'astrophysics', 'galactic astronomy', 'digital communication', 'space research', 'labor market', 'corporate marketing', 'advertising', 'space monitoring', 'industrial engineering', 'market commercial', 'digital services', 'network analysis', 'digitalization', 'transition towards', 'connectivity multilink', 'high energy physics', 'spacecraft design', 'space technology', 'european union', 'performance studies', 'technology', 'towards high', 'horizonsesardesir technology', 'performance airground', 'social change', 'wireless communication']</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>['galactic astronomy', 'ecosystem services', 'space research', 'sky industrial', 'aviation', 'digital european', 'ecosystem', 'space habitats', 'european union', 'uspace ecosystem', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'extending uspace', 'space implementation', 'research horizonsesardesirwa', 'european sky', 'fasttrack extending', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'digitalization', 'ecosystem digital', 'space compliance', 'astrophysics', 'artificial ecosystems', 'digital', 'planetary science', 'industrial design']</t>
+          <t>['industrial design', 'extending uspace', 'sky industrial', 'digital european', 'industrial data', 'fasttrack extending', 'research horizonsesardesirwa', 'ecosystem digital', 'aviation', 'planetary science', 'space compliance', 'european sky', 'uspace ecosystem', 'space implementation', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'artificial ecosystems', 'digital', 'industrial research', 'astrophysics', 'galactic astronomy', 'industrial engineering', 'space habitats', 'ecosystem', 'digitalization', 'european union', 'space research', 'ecosystem services']</t>
         </is>
       </c>
     </row>
@@ -3014,7 +3014,7 @@
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>['increased automation', 'galactic astronomy', 'digital craft', 'operations research', 'space research', 'sky industrial', 'pilot atm', 'aviation', 'digital european', 'atm tasks', 'european union', 'space industry', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'machine automation', 'assistance pilot', 'european sky', 'digital', 'automation assistance', 'tasks digital', 'industrial data', 'horizonsesardesirwa horizonsesardesir', 'digitalization', 'banking', 'digital systems', 'aviation management', 'teleoperation', 'scheduling', 'astrophysics', 'automation', 'planetary science', 'industrial design']</t>
+          <t>['industrial design', 'pilot atm', 'sky industrial', 'operations research', 'digital european', 'industrial data', 'research horizonsesardesirwa', 'aviation', 'scheduling', 'planetary science', 'assistance pilot', 'atm tasks', 'european sky', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'increased automation', 'industrial research', 'teleoperation', 'digital', 'tasks digital', 'machine automation', 'astrophysics', 'galactic astronomy', 'industrial engineering', 'digital craft', 'banking', 'aviation management', 'digitalization', 'automation assistance', 'digital systems', 'automation', 'european union', 'space research']</t>
         </is>
       </c>
     </row>
@@ -3051,7 +3051,7 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>['europe partnership', 'composition', 'chain orchestration', 'supply chain', 'circular value', 'fashion supply chain', 'mechanical engineering manufacturing', 'manufacturing systems', 'technology', 'environmental sustainability', 'literary modernism', 'resistors', 'circular dynamic', 'literature film', 'africa', 'political activism', 'literature', 'global value chains', 'biotechnology innovation', 'ims made', 'business capabilities', 'moral values', 'oc building', 'sustainability', 'orchestration optimisation', 'city', 'musical composition.', 'information systems', 'european union', 'made europe', 'sustainability smes', 'change innovation.', 'supporters', 'information technology', 'partnership ia', 'smes ims', 'supply chain modeling', 'innovation manufacturing', 'dynamic', 'architectural design', 'dynamic manufacturing', 'international organizations', 'european integration', 'value chain', 'mems', 'europeanization', 'demonstrators circular', 'social media services', 'construction management', 'accreditation', 'novel circular', 'mems microtechnology', 'chain demonstrators', 'building novel', 'ict innovation', 'craft architecture', 'electronics manufacturing', 'manufacturing supply', 'activist public relations', 'collective identities', 'values', 'inflation', 'ia oc', 'educational buildings', 'logistics optimization', 'dynamical systems', 'supply chain management', 'design sustainability', 'architecture', 'manufacturing sustainability', 'industrial design']</t>
+          <t>['orchestration optimisation', 'supply chain', 'supporters', 'mechanical engineering manufacturing', 'activist public relations', 'information systems', 'building novel', 'industrial design', 'sustainability', 'dynamical systems', 'ia oc', 'africa', 'design sustainability', 'social media services', 'circular value', 'political activism', 'fashion supply chain', 'environmental sustainability', 'ict innovation', 'manufacturing supply', 'europeanization', 'chain orchestration', 'international organizations', 'craft architecture', 'change innovation.', 'resistors', 'dynamic', 'european integration', 'value chain', 'city', 'manufacturing sustainability', 'manufacturing systems', 'supply chain management', 'literature', 'supply chain modeling', 'demonstrators circular', 'accreditation', 'logistics optimization', 'novel circular', 'ims made', 'mems microtechnology', 'global value chains', 'architecture', 'inflation', 'construction management', 'literature film', 'biotechnology innovation', 'mems', 'collective identities', 'chain demonstrators', 'business capabilities', 'europe partnership', 'moral values', 'partnership ia', 'oc building', 'made europe', 'educational buildings', 'electronics manufacturing', 'literary modernism', 'dynamic manufacturing', 'sustainability smes', 'innovation manufacturing', 'technology', 'european union', 'values', 'composition', 'circular dynamic', 'smes ims', 'information technology', 'musical composition.', 'architectural design']</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>['neuroscience', 'robotic services', 'galactic astronomy', 'fasttrack u', 'cns capabilities', 'space research', 'sky industrial', 'u uspace', 'aviation', 'digital european', 'capabilities digital', 'fit', 'service marketing', 'european union', 'uspace advanced', 'space industry', 'advanced services', 'industrial engineering', 'aerospace engineering', 'industrial research', 'research horizonsesardesirwa', 'services cns', 'european sky', 'identity', 'digital services', 'cad/cam technologies', 'horizonsesardesirwa horizonsesardesir', 'industrial data', 'performance', 'digitalization', 'space evaluation', 'astrophysics', 'digital', 'space', 'planetary science', 'industrial design']</t>
+          <t>['fasttrack u', 'identity', 'capabilities digital', 'industrial design', 'cad/cam technologies', 'sky industrial', 'cns capabilities', 'digital european', 'industrial data', 'space evaluation', 'research horizonsesardesirwa', 'neuroscience', 'performance', 'aviation', 'fit', 'planetary science', 'space', 'uspace advanced', 'european sky', 'robotic services', 'service marketing', 'services cns', 'aerospace engineering', 'horizonsesardesirwa horizonsesardesir', 'space industry', 'digital', 'industrial research', 'astrophysics', 'galactic astronomy', 'industrial engineering', 'digitalization', 'digital services', 'advanced services', 'european union', 'space research', 'u uspace']</t>
         </is>
       </c>
     </row>
@@ -3125,7 +3125,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>['tide', 'performance arts', 'estuaries rivers (wave', 'contribution creative', 'water arts', 'deep ecology', 'space services', 'landscapes art', 'ocean energy', 'transforming inspiring', 'inspiring aquatic', 'law sea', 'arts transforming', 'arts contribution', 'urban communication', 'ecology', 'mission ocean', 'ocean waters', 'revolutionary changes world', 'telemedicine', 'danube riverblack', 'performing arts', 'adaptation', 'lighthouse call', 'teleworking', 'ocean water', 'creative sectors', 'sectors mission', 'seas', 'creativity', 'creative industry', 'sediment transport', 'aquatic landscapes', 'art culture', 'call tidal', 'creative labor', 'riverblack sea', 'space exploration', 'balkans', 'cultural industries creative economy', 'waters danube', 'oceanography', 'coastal structures', 'art sustainability', 'art sciences', 'cultural landscapes', 'visual arts', 'tidal arts', 'sea lighthouse']</t>
+          <t>['space exploration', 'water arts', 'call tidal', 'revolutionary changes world', 'lighthouse call', 'seas', 'cultural landscapes', 'arts transforming', 'ocean energy', 'sediment transport', 'oceanography', 'inspiring aquatic', 'cultural industries creative economy', 'law sea', 'telemedicine', 'transforming inspiring', 'ocean water', 'visual arts', 'danube riverblack', 'art sustainability', 'urban communication', 'balkans', 'contribution creative', 'landscapes art', 'art sciences', 'waters danube', 'mission ocean', 'ocean waters', 'teleworking', 'riverblack sea', 'adaptation', 'deep ecology', 'aquatic landscapes', 'coastal structures', 'performance arts', 'art culture', 'ecology', 'tide', 'tidal arts', 'performing arts', 'creative industry', 'estuaries rivers (wave', 'space services', 'creativity', 'arts contribution', 'creative sectors', 'sea lighthouse', 'creative labor', 'sectors mission']</t>
         </is>
       </c>
     </row>
@@ -3162,7 +3162,7 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>['tide', 'performance arts', 'contribution creative', 'deep ecology', 'space services', 'landscapes art', 'waters atlantic', 'transforming inspiring', 'inspiring aquatic', 'ocean energy', 'arts transforming', 'law sea', 'atlantic arctic', 'arts contribution', 'urban communication', 'ecology', 'mission ocean', 'ocean waters', 'climate', 'aesthetics place', 'revolutionary changes world', 'telemedicine', 'performing arts', 'adaptation', 'lighthouse call', 'teleworking', 'arctic lighthouse', 'ocean water', 'creative sectors', 'sectors mission', 'seas', 'creativity', 'creative industry', 'russia', 'aquatic landscapes', 'art culture', 'call tidal', 'creative labor', 'space exploration', 'cultural industries creative economy', 'oceanography', 'art sustainability', 'art sciences', 'cultural landscapes', 'visual arts', 'tidal arts', 'water arts']</t>
+          <t>['space exploration', 'water arts', 'call tidal', 'revolutionary changes world', 'lighthouse call', 'seas', 'cultural landscapes', 'arctic lighthouse', 'arts transforming', 'ocean energy', 'oceanography', 'inspiring aquatic', 'cultural industries creative economy', 'law sea', 'telemedicine', 'transforming inspiring', 'ocean water', 'visual arts', 'art sustainability', 'climate', 'urban communication', 'contribution creative', 'waters atlantic', 'landscapes art', 'art sciences', 'adaptation', 'mission ocean', 'ocean waters', 'teleworking', 'atlantic arctic', 'deep ecology', 'aquatic landscapes', 'performance arts', 'art culture', 'aesthetics place', 'ecology', 'tide', 'tidal arts', 'performing arts', 'creative industry', 'space services', 'russia', 'creativity', 'arts contribution', 'creative sectors', 'creative labor', 'sectors mission']</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3199,7 @@
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>['transnational adaptations', 'higher education', 'communication consultancy', 'robotic innovation', 'digital humanities', 'sustainable finance', 'green finance', 'social media innovation', 'interdisciplinary mobility', 'clinical psychology', 'change innovation.', 'space consulting', 'postdoctoral ri', 'ri interdisciplinary', 'education urban space / traffic)', 'msca cofund', 'sociology.', 'financial analysis', 'community studies', 'horizonmscacofund horizonmscacofund', 'accreditation', 'crowdfunding', 'cofund msca', 'postdoc postdoctoral', 'transportation planning', 'mobility innovation', 'cofund horizonmscacofund', 'horizonmscacofund phd', 'phd doctoral', 'doctoral postdoc']</t>
+          <t>['robotic innovation', 'communication consultancy', 'phd doctoral', 'clinical psychology', 'higher education', 'space consulting', 'crowdfunding', 'transportation planning', 'cofund horizonmscacofund', 'change innovation.', 'community studies', 'mobility innovation', 'financial analysis', 'accreditation', 'social media innovation', 'doctoral postdoc', 'cofund msca', 'sustainable finance', 'postdoctoral ri', 'interdisciplinary mobility', 'horizonmscacofund phd', 'digital humanities', 'transnational adaptations', 'education urban space / traffic)', 'postdoc postdoctoral', 'ri interdisciplinary', 'sociology.', 'horizonmscacofund horizonmscacofund', 'green finance', 'msca cofund']</t>
         </is>
       </c>
     </row>
@@ -3236,7 +3236,7 @@
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>['social capital', 'horizoneicaccelerator horizoneicaccelerator', 'accelerator short', 'short film', 'hinfinity control', 'deep ecology', 'technology', 'electronic commerce', 'rocket propulsion', 'biotechnology innovation', 'horizoneicaccelerator deep', 'enterprise software systems', 'healthcare technology', 'short application', 'application eic', 'application stepdigitaldeep', 'patient satisfaction', 'capital markets law', 'patient capital', 'carbon capture', 'patient safety', 'mobile applications', 'change innovation.', 'information technology', 'mechatronics engineering', 'eic accelerator', 'innovation technology', 'software design', 'stepdigitaldeep tech', 'electronic devices', 'electronic payment services', 'research innovation', 'mechatronics', 'detector rd', 'technology eic', 'deep tech', 'software', 'capital research', 'computer engineering', 'technology society', 'tech horizoneicaccelerator', 'research performance', 'deep neural network', 'microelectronics', 'tech patient', 'deep learning']</t>
+          <t>['patient capital', 'electronic payment services', 'technology eic', 'software design', 'research performance', 'capital markets law', 'eic accelerator', 'deep neural network', 'tech patient', 'deep tech', 'enterprise software systems', 'social capital', 'electronic devices', 'horizoneicaccelerator deep', 'change innovation.', 'technology society', 'detector rd', 'accelerator short', 'mechatronics engineering', 'rocket propulsion', 'electronic commerce', 'hinfinity control', 'capital research', 'short application', 'deep ecology', 'innovation technology', 'deep learning', 'carbon capture', 'biotechnology innovation', 'healthcare technology', 'software', 'horizoneicaccelerator horizoneicaccelerator', 'research innovation', 'tech horizoneicaccelerator', 'computer engineering', 'mechatronics', 'microelectronics', 'application stepdigitaldeep', 'technology', 'patient safety', 'stepdigitaldeep tech', 'application eic', 'short film', 'information technology', 'patient satisfaction', 'mobile applications']</t>
         </is>
       </c>
     </row>
@@ -3273,7 +3273,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>['transnational adaptations', 'higher education', 'communication consultancy', 'robotic innovation', 'horizonmscase phd', 'electronic commerce', 'digital humanities', 'social media innovation', 'horizonmscase horizonmscase', 'interdisciplinary mobility', 'international arbitration', 'clinical psychology', 'cosmology', 'staff exchanges', 'exchanges horizonmscase', 'management organization', 'postdoctoral ri', 'capital markets law', 'black hole physics', 'space consulting', 'change innovation.', 'exchanges msca', 'ri interdisciplinary', 'education urban space / traffic)', 'human resources management', 'international organizations', 'sociology.', 'community studies', 'msca staff', 'postdoc postdoctoral', 'international commercial arbitration', 'world trade organization', 'transportation planning', 'women managerial positions', 'mobility innovation', 'phd doctoral', 'scheduling', 'doctoral postdoc']</t>
+          <t>['robotic innovation', 'exchanges msca', 'international arbitration', 'communication consultancy', 'capital markets law', 'phd doctoral', 'clinical psychology', 'higher education', 'staff exchanges', 'cosmology', 'space consulting', 'transportation planning', 'international organizations', 'international commercial arbitration', 'change innovation.', 'scheduling', 'community studies', 'electronic commerce', 'mobility innovation', 'world trade organization', 'social media innovation', 'msca staff', 'horizonmscase horizonmscase', 'doctoral postdoc', 'women managerial positions', 'postdoctoral ri', 'interdisciplinary mobility', 'digital humanities', 'transnational adaptations', 'education urban space / traffic)', 'horizonmscase phd', 'postdoc postdoctoral', 'ri interdisciplinary', 'exchanges horizonmscase', 'management organization', 'human resources management', 'sociology.', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -3310,7 +3310,7 @@
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>['ai data', 'robotics capabilities', 'mobilization', 'robotic verification', 'increased robotics', 'technology', 'robotic safety', 'demonstrators soprano', 'robotics', 'call industry', 'sectors ai', 'political activism', 'trust service provider', 'sociallyacceptable trustworthy', 'business capabilities', 'soprano technologiesn', 'capabilities demonstrated', 'enterprise software systems', 'open data', 'telemedicine', 'musicology', 'open call', 'robotic validation', 'software development', 'robotic collaboration', 'teleworking', 'supporters', 'industry demonstrators', 'partnership ia', 'key sectors', 'theater', 'data robotics', 'creative industry', 'international organizations', 'trustworthy humanrobot', 'open banking', 'blockchain', 'identity', 'social media technology', 'accreditation', 'soprano open', 'artificial intelligence', 'design ability', 'diodes', 'trust law', 'detector rd', 'corporate communication', 'trust services', 'humanrobot teaming', 'strategic management', 'teaming agile', 'electronic signature', 'activist public relations', 'robotics partnership', 'demonstrated key', 'agile industries', 'ia soprano', 'transmedia', 'strategy', 'robotic deployment', 'technology society', 'technologiesn sociallyacceptable']</t>
+          <t>['robotic collaboration', 'supporters', 'trust service provider', 'activist public relations', 'sectors ai', 'identity', 'increased robotics', 'blockchain', 'trust services', 'trust law', 'robotic validation', 'strategic management', 'soprano technologiesn', 'design ability', 'political activism', 'sociallyacceptable trustworthy', 'enterprise software systems', 'corporate communication', 'capabilities demonstrated', 'social media technology', 'humanrobot teaming', 'diodes', 'data robotics', 'telemedicine', 'industry demonstrators', 'agile industries', 'international organizations', 'open call', 'technology society', 'detector rd', 'ai data', 'artificial intelligence', 'accreditation', 'strategy', 'mobilization', 'transmedia', 'teleworking', 'call industry', 'key sectors', 'teaming agile', 'robotics', 'ia soprano', 'robotic verification', 'technologiesn sociallyacceptable', 'robotics capabilities', 'robotic deployment', 'business capabilities', 'robotic safety', 'partnership ia', 'theater', 'electronic signature', 'software development', 'trustworthy humanrobot', 'open data', 'creative industry', 'demonstrators soprano', 'technology', 'musicology', 'robotics partnership', 'soprano open', 'demonstrated key', 'open banking']</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3347,7 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>['social capital', 'hinfinity control', 'open eic', 'open pathfinderopen', 'pathfinderopen horizoneicpathfinderopen', 'eic pathfinder', 'deep ecology', 'technology', 'robotics', 'electronic commerce', 'pathfinder open', 'biotechnology innovation', 'free associations', 'healthcare technology', 'open data', 'patient satisfaction', 'capital markets law', 'patient capital', 'patient safety', 'change innovation.', 'black hole physics', 'information technology', 'horizoneicpathfinderopen deep', 'algorithm design', 'open banking', 'innovation technology', 'tech patient', 'electronic devices', 'research innovation', 'algorithm optimization', 'space exploration', 'technology eic', 'deep tech', 'deep learning algorithms', 'capital research', 'technology society', 'research performance', 'deep neural network', 'optimization algorithms', 'pathfinder pathfinder', 'horizoneicpathfinderopen horizoneicpathfinderopen', 'deep learning']</t>
+          <t>['patient capital', 'horizoneicpathfinderopen horizoneicpathfinderopen', 'space exploration', 'technology eic', 'pathfinder open', 'research performance', 'capital markets law', 'deep neural network', 'tech patient', 'deep tech', 'algorithm optimization', 'social capital', 'free associations', 'electronic devices', 'open eic', 'change innovation.', 'technology society', 'patient satisfaction', 'deep learning algorithms', 'pathfinderopen horizoneicpathfinderopen', 'electronic commerce', 'eic pathfinder', 'hinfinity control', 'capital research', 'optimization algorithms', 'horizoneicpathfinderopen deep', 'deep ecology', 'innovation technology', 'deep learning', 'robotics', 'open pathfinderopen', 'biotechnology innovation', 'algorithm design', 'healthcare technology', 'research innovation', 'open data', 'technology', 'patient safety', 'open banking', 'information technology', 'pathfinder pathfinder', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>['social capital', 'mechanical devices', 'stepbiotech stepdigitaldeep', 'microtechnology', 'technology', 'thermofluids', 'electronic commerce', 'tech stepcleantech', 'mechanical equipment', 'biotechnology innovation', 'horizoneiceicstep deep', 'healthcare technology', 'eic step', 'biosimilars', 'patient satisfaction', 'multidimensional scaling', 'patient capital', 'patient safety', 'capital markets law', 'change innovation.', 'information technology', 'health biotechnology', 'growth', 'step scale', 'scale stepbiotech', 'proteomics', 'innovation technology', 'stepdigitaldeep tech', 'electronic devices', 'electronic payment services', 'research innovation', 'mechatronics', 'stepcleantech horizoneiceicstep', 'scale eic', 'multiscale fracture', 'technology eic', 'deep tech', 'biotech startups', 'capital research', 'microtechnology.', 'high frequency technique', 'ultra wideband', 'computer engineering', 'electronic signature', 'optoelectronics', 'technology society', 'research performance', 'values', 'horizoneiceicstep horizoneiceicstep', 'deep neural network', 'microelectronics', 'tech patient', 'deep learning']</t>
+          <t>['patient capital', 'microtechnology.', 'multidimensional scaling', 'electronic payment services', 'technology eic', 'biotech startups', 'ultra wideband', 'research performance', 'capital markets law', 'deep neural network', 'tech patient', 'stepbiotech stepdigitaldeep', 'deep tech', 'social capital', 'tech stepcleantech', 'stepcleantech horizoneiceicstep', 'thermofluids', 'electronic devices', 'change innovation.', 'technology society', 'electronic commerce', 'mechanical equipment', 'multiscale fracture', 'health biotechnology', 'capital research', 'step scale', 'microtechnology', 'deep learning', 'innovation technology', 'scale eic', 'scale stepbiotech', 'growth', 'eic step', 'biotechnology innovation', 'horizoneiceicstep horizoneiceicstep', 'healthcare technology', 'electronic signature', 'research innovation', 'horizoneiceicstep deep', 'computer engineering', 'mechanical devices', 'microelectronics', 'values', 'mechatronics', 'technology', 'biosimilars', 'high frequency technique', 'patient safety', 'stepdigitaldeep tech', 'optoelectronics', 'information technology', 'proteomics', 'patient satisfaction']</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>['drug resistance', 'geared turbofan', 'hinfinity control', 'preparation flight', 'quantum heat engines', 'engine smr', 'electronic testing', 'aircraft systems', 'robotic testing', 'smr aircraft', 'inductors', 'horizonjucleanaviationsmr horizonjucleanaviation', 'resistors', 'presentation', 'mechanical components', 'rocket propulsion', 'mechanical equipment', 'space validation', 'test ultra', 'aircraft clean', 'aviation', 'astrobiology', 'turbulence', 'disabled care)', 'flight test', 'turbofan engine', 'fit', 'combustion engines', 'cosmology', 'ground test', 'ratio ducted', 'mechanical testing', 'mechanical', 'black hole physics', 'aerospace engineering', 'clean aviation', 'HVAC systems', 'experimental design', 'signal conversion', 'high bypass', 'bypass ratio', 'space testing', 'computational ornament', 'high energy physics', 'demonstration preparation', 'ultra wideband', 'cfp horizonjucleanaviationsmr', 'boundary layer)', 'ducted geared', 'ultra high', 'aviation cfp', 'aviation management', 'test demonstration']</t>
+          <t>['flight test', 'ultra wideband', 'signal conversion', 'cfp horizonjucleanaviationsmr', 'drug resistance', 'electronic testing', 'combustion engines', 'cosmology', 'ground test', 'test ultra', 'aircraft systems', 'aviation', 'resistors', 'experimental design', 'fit', 'engine smr', 'smr aircraft', 'horizonjucleanaviationsmr horizonjucleanaviation', 'quantum heat engines', 'mechanical equipment', 'turbulence', 'rocket propulsion', 'hinfinity control', 'inductors', 'aerospace engineering', 'test demonstration', 'space testing', 'disabled care)', 'aviation cfp', 'high bypass', 'preparation flight', 'presentation', 'astrobiology', 'ratio ducted', 'demonstration preparation', 'geared turbofan', 'boundary layer)', 'space validation', 'robotic testing', 'mechanical testing', 'aviation management', 'ducted geared', 'aircraft clean', 'high energy physics', 'mechanical components', 'bypass ratio', 'turbofan engine', 'computational ornament', 'clean aviation', 'HVAC systems', 'ultra high', 'black hole physics', 'mechanical']</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>['rewriting', 'propulsion system', 'microelectromechanical systems', 'systems engineering', 'aircraft systems', 'deconstruction', 'space integration', 'smart systems', 'thermofluids', 'system regional', 'genetic modification', 'rocket propulsion', 'nacelle integration', 'aviation', 'regional aircraft', 'astrobiology', 'exotic meson analysis', 'hybrid', 'cfp horizonjucleanaviationreg', 'demonstration hybridelectric', 'combustion engines', 'cosmology', 'black hole physics', 'ferroelectric materials', 'aerospace engineering', 'clean aviation', 'biological agents', 'biomolecular interactions', 'hybridelectric propulsion', 'turkish', 'biopolymer', 'syntaxprosody', 'system design', 'electric vehicles', 'integration modification', 'modification clean', 'pylon nacelle', 'horizonjucleanaviationreg horizonjucleanaviation', 'macro', 'including pylon', 'aviation cfp', 'aviation management', 'aircraft including', 'mechanical systems']</t>
+          <t>['smart systems', 'including pylon', 'biomolecular interactions', 'biological agents', 'mechanical systems', 'modification clean', 'macro', 'demonstration hybridelectric', 'horizonjucleanaviationreg horizonjucleanaviation', 'combustion engines', 'cosmology', 'aircraft systems', 'thermofluids', 'aviation', 'space integration', 'rewriting', 'system regional', 'ferroelectric materials', 'exotic meson analysis', 'pylon nacelle', 'turkish', 'rocket propulsion', 'syntaxprosody', 'aerospace engineering', 'biopolymer', 'electric vehicles', 'aviation cfp', 'hybridelectric propulsion', 'propulsion system', 'astrobiology', 'hybrid', 'deconstruction', 'aviation management', 'genetic modification', 'microelectromechanical systems', 'systems engineering', 'system design', 'clean aviation', 'regional aircraft', 'aircraft including', 'nacelle integration', 'integration modification', 'cfp horizonjucleanaviationreg', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -3495,7 +3495,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>['demonstration trl', 'hinfinity control', 'aircraft systems', 'electronic testing', 'robotic testing', 'smr aircraft', 'horizonjucleanaviationsmr horizonjucleanaviation', 'manipulation', 'npe systems', 'architectural representation', 'space validation', 'aircraft clean', 'cae methodology development', 'aviation', 'astrobiology', 'maritime security', 'cosmology', 'ground test', 'mechanical testing', 'black hole physics', 'trl onboard', 'aerospace engineering', 'systems architecture', 'clean aviation', 'architectural design', 'distributed computing', 'automated systems', 'space testing', 'computational ornament', 'architecture smr', 'cfp horizonjucleanaviationsmr', 'aviation cfp', 'aviation management', 'teleoperation', 'multi-agent systems', 'test demonstration', 'architecture', 'robotic deployment', 'onboard npe']</t>
+          <t>['onboard npe', 'black hole physics', 'automated systems', 'manipulation', 'cfp horizonjucleanaviationsmr', 'electronic testing', 'cae methodology development', 'ground test', 'cosmology', 'architectural representation', 'aircraft systems', 'aviation', 'distributed computing', 'smr aircraft', 'horizonjucleanaviationsmr horizonjucleanaviation', 'hinfinity control', 'aerospace engineering', 'test demonstration', 'space testing', 'maritime security', 'teleoperation', 'aviation cfp', 'trl onboard', 'systems architecture', 'architecture', 'astrobiology', 'npe systems', 'architecture smr', 'robotic deployment', 'space validation', 'robotic testing', 'demonstration trl', 'mechanical testing', 'aviation management', 'aircraft clean', 'computational ornament', 'clean aviation', 'multi-agent systems', 'architectural design']</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3532,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>['systems relevant', 'embedded systems', 'aircraft systems', 'relevant hybridization', 'urbanization', 'thermofluids', 'demonstration onboard', 'onboard systems', 'aircraft clean', 'aviation', 'regional aircraft', 'astrobiology', 'information systems', 'hybrid', 'cfp horizonjucleanaviationreg', 'cosmology', 'heterogeneous computing', 'black hole physics', 'aerospace engineering', 'clean aviation', 'hybridization regional', 'europeanization', 'space training', 'syntaxprosody', 'biocompability', 'digital systems', 'horizonjucleanaviationreg horizonjucleanaviation', 'systems theory', 'macro', 'aviation cfp', 'aviation management']</t>
+          <t>['onboard systems', 'information systems', 'heterogeneous computing', 'biocompability', 'macro', 'horizonjucleanaviationreg horizonjucleanaviation', 'cosmology', 'europeanization', 'relevant hybridization', 'aircraft systems', 'aviation', 'thermofluids', 'space training', 'systems theory', 'hybridization regional', 'urbanization', 'systems relevant', 'syntaxprosody', 'aerospace engineering', 'embedded systems', 'aviation cfp', 'astrobiology', 'hybrid', 'aviation management', 'aircraft clean', 'digital systems', 'clean aviation', 'demonstration onboard', 'regional aircraft', 'cfp horizonjucleanaviationreg', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -3569,7 +3569,7 @@
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>['quantum heat engines', 'hinfinity control', 'inductors', 'electronic testing', 'aircraft systems', 'robotic testing', 'smr aircraft', 'circuits', 'horizonjucleanaviationsmr horizonjucleanaviation', 'architectural representation', 'space validation', 'aircraft clean', 'aviation', 'astrobiology', 'flight test', 'combustion engines', 'cosmology', 'mechanical testing', 'black hole physics', 'aerospace engineering', 'clean aviation', 'demonstration unducted', 'engine architecture', 'craft architecture', 'computational ornament', 'architecture smr', 'cfp horizonjucleanaviationsmr', 'aviation cfp', 'aviation management', 'test demonstration', 'architecture', 'unducted engine']</t>
+          <t>['flight test', 'circuits', 'cfp horizonjucleanaviationsmr', 'electronic testing', 'combustion engines', 'cosmology', 'architectural representation', 'craft architecture', 'aircraft systems', 'aviation', 'smr aircraft', 'horizonjucleanaviationsmr horizonjucleanaviation', 'quantum heat engines', 'hinfinity control', 'inductors', 'aerospace engineering', 'test demonstration', 'aviation cfp', 'astrobiology', 'architecture', 'engine architecture', 'architecture smr', 'space validation', 'robotic testing', 'mechanical testing', 'demonstration unducted', 'aviation management', 'aircraft clean', 'computational ornament', 'unducted engine', 'clean aviation', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>['space transportation', 'microelectromechanical systems', 'aircraft systems', 'electronic testing', 'robotic testing', 'thermofluids', 'rocket propulsion', 'aircraft clean', 'aviation', 'regional aircraft', 'astrobiology', 'flight test', 'hybrid', 'cfp horizonjucleanaviationreg', 'demonstration hybridelectric', 'combustion engines', 'cosmology', 'mechanical testing', 'black hole physics', 'ferroelectric materials', 'aerospace engineering', 'clean aviation', 'hybridelectric propulsion', 'propulsion regional', 'syntaxprosody', 'electric vehicles', 'horizonjucleanaviationreg horizonjucleanaviation', 'macro', 'aviation cfp', 'aviation management', 'test demonstration']</t>
+          <t>['flight test', 'macro', 'demonstration hybridelectric', 'horizonjucleanaviationreg horizonjucleanaviation', 'electronic testing', 'space transportation', 'combustion engines', 'cosmology', 'aircraft systems', 'thermofluids', 'aviation', 'ferroelectric materials', 'rocket propulsion', 'syntaxprosody', 'aerospace engineering', 'test demonstration', 'electric vehicles', 'aviation cfp', 'hybridelectric propulsion', 'astrobiology', 'hybrid', 'robotic testing', 'mechanical testing', 'aviation management', 'aircraft clean', 'propulsion regional', 'microelectromechanical systems', 'clean aviation', 'regional aircraft', 'cfp horizonjucleanaviationreg', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3643,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>['hinfinity control', 'aircraft systems', 'space integration', 'technology', 'thermofluids', 'key technologies', 'embedded technologies', 'aircraft concept', 'robotic assessment', 'aviation', 'astrobiology', 'concept key', 'cosmology', 'technologies integration', 'black hole physics', 'conceptual design', 'educational technologies', 'horizonjucleanaviationaci horizonjucleanaviation', 'information technology', 'aerospace engineering', 'clean aviation', 'theory', 'european integration', 'cfp horizonjucleanaviationaci', 'impact assessment', 'psychological assessment', 'syntaxprosody', 'integration impact', 'assessment clean', 'risk assessment', 'aviation cfp', 'aviation management', 'evaluation', 'technology society']</t>
+          <t>['evaluation', 'educational technologies', 'cfp horizonjucleanaviationaci', 'technologies integration', 'assessment clean', 'cosmology', 'aircraft concept', 'aircraft systems', 'robotic assessment', 'aviation', 'space integration', 'thermofluids', 'technology society', 'conceptual design', 'european integration', 'concept key', 'key technologies', 'integration impact', 'hinfinity control', 'aerospace engineering', 'aviation cfp', 'risk assessment', 'astrobiology', 'impact assessment', 'theory', 'aviation management', 'psychological assessment', 'technology', 'clean aviation', 'embedded technologies', 'horizonjucleanaviationaci horizonjucleanaviation', 'information technology', 'syntaxprosody', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3680,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>['equity related', 'plan business', 'development economics', 'strategic business management', 'eg gender', 'women techeu', 'planning design', 'biotechnology innovation', 'entrepreneurship', 'seed capital', 'startup companies', 'gender economy', 'horizoneicwomentech horizoneicwomentech', 'capital markets law', 'mechanical engineering support', 'development incubator', 'competitive strategies', 'womens entrepreneurship', 'business development', 'international finance', 'financial analysis', 'sme startup', 'models theory', 'women', 'architecture', 'business strategies', 'innovation development', 'companies startup', 'small medium enterprises', 'community development', 'private equity', 'support seed', 'international investment law', 'business capabilities', 'investor behavior', 'gender construction', 'software development', 'investment business', 'information technology', 'biotech innovation', 'virtual archeology', 'entrepreneurship gender', 'initiative women', 'horizoneicwomentech angel', 'space support', 'techeu horizoneicwomentech', 'biotech startups', 'support sme', 'angel investment', 'marketing strategy', 'business model studies', 'feminism', 'innovation diversity', 'youth work', 'social media support', 'strategies entrepreneurship', 'green finance', 'related sme', 'mentoring business', 'city', 'incubator companies', 'coaching mentoring', 'change innovation.', 'biotechnology companies', 'd esign education', 'gender', 'capital spinoff', 'cultural diversity', 'diversity eg', 'gender studies', 'social networks', 'business models social enterprises', 'gender innovation', 'leadership', 'business plan', 'economic development', 'strategy', 'architectural design.', 'models business', 'business history', 'startup support', 'growth development', 'gender diversity', 'technology', 'spinoff companies', 'gender private', 'corporate marketing', 'internal entrepreneurship', 'social media support tools', 'corporate governance', 'business coaching', 'development business', 'race and ethnicity', 'sponsorship management', 'techeu initiative', 'sme support', 'economics', 'business models', 'technology society', 'companies innovation']</t>
+          <t>['companies startup', 'sme support', 'cultural diversity', 'economic development', 'models business', 'private equity', 'support sme', 'development economics', 'change innovation.', 'race and ethnicity', 'innovation development', 'community development', 'angel investment', 'mechanical engineering support', 'development incubator', 'gender innovation', 'gender', 'capital spinoff', 'womens entrepreneurship', 'gender studies', 'startup companies', 'business capabilities', 'business development', 'equity related', 'spinoff companies', 'green finance', 'youth work', 'architectural design.', 'information technology', 'business history', 'initiative women', 'investment business', 'biotech startups', 'capital markets law', 'social media support', 'gender private', 'entrepreneurship gender', 'coaching mentoring', 'plan business', 'd esign education', 'gender construction', 'gender economy', 'business coaching', 'business strategies', 'virtual archeology', 'techeu horizoneicwomentech', 'mentoring business', 'architecture', 'international finance', 'growth development', 'entrepreneurship', 'development business', 'strategies entrepreneurship', 'biotechnology innovation', 'women techeu', 'competitive strategies', 'marketing strategy', 'technology', 'biotechnology companies', 'companies innovation', 'horizoneicwomentech horizoneicwomentech', 'investor behavior', 'economics', 'incubator companies', 'sme startup', 'eg gender', 'business models social enterprises', 'international investment law', 'technology society', 'innovation diversity', 'financial analysis', 'strategy', 'leadership', 'related sme', 'corporate governance', 'business plan', 'corporate marketing', 'software development', 'social networks', 'gender diversity', 'seed capital', 'biotech innovation', 'business model studies', 'techeu initiative', 'internal entrepreneurship', 'small medium enterprises', 'diversity eg', 'space support', 'startup support', 'feminism', 'support seed', 'models theory', 'city', 'horizoneicwomentech angel', 'business models', 'strategic business management', 'women', 'sponsorship management', 'planning design', 'social media support tools']</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>['composition', 'polymers plastics', 'engineering materials', 'cermets combined', 'properties circular', 'combined natural', 'synthetic fibre', 'fibrebased packaging', 'chemical engineering', 'biotechnology innovation', 'material feedstock', 'including laminates', 'fit', 'denture adhesives', 'european union', 'europe joint', 'semiconductors', 'european studies', 'quality', 'black hole physics', 'circular packaging', 'synthetic biology', 'biobased packaging', 'biomolecular research', 'packaging materials', 'biodefense', 'nutritional biotechnology', 'packaging circularity', 'bulk fine', 'laminates reinforced', 'electronics manufacturing', 'astrophysics', 'fabrics filled', 'biosecurity', 'technical textiles', 'marketing product brand management', 'biodegradable polymers', 'packaging circular', 'yarn', 'materials biobased', 'composites', 'biobased products', 'medical biotechnology', 'operations research', 'packaging recycling', 'biobased materials', 'biobased europe', 'biomaterials', 'mechanical components', 'humanitarian logistics', 'reinforced plastics', 'recycling safeandsustainablebydesign', 'freight transportation', 'coatings fibrebased', 'robotic collaboration', 'bioinformatics', 'biotech innovation', 'technology fashion products', 'materials composites', 'materials engineering', 'safeandsustainablebydesign stepbiotech', 'products manufactured', 'plasticity', 'bioenergy', 'circular biobased', 'improved properties', 'waste management', 'packaging improved', 'mechanical engineering materials', 'biopolymer', 'biotech startups', 'bioengineering', 'adaptive reuse industrial heritage', 'etc polymers', 'convergans clubs', 'using biological', 'circularity coatings', 'drug delivery', 'mechanical engineering safety', 'packaging packaging', 'distribution agreements', 'feedstock biobased', 'polymer materials engineering behaviors civil engineering', 'plastics cermets', 'biotechnology', 'circular bioeconomy', 'joint undertaking', 'undertaking additives', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'steel', 'biosimilars', 'products products', 'mechanical properties', 'filled composites', 'biochemistry', 'biomaterials metals', 'mechanical structures', 'biomedical', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'composite materials', 'performance', 'biomechanics', 'materials packaging', 'plastics biofuels', 'novel materials', 'metals ceramics', 'biotech industry', 'logistics optimization', 'natural synthetic', 'biobased plastics', 'recycling technologies', 'pharmaceutical industry', 'biological systems', 'adhesives biobased', 'circularbydesign fibrebased', 'manufacturing systems', 'technology', 'product liability', 'bioeconomy circular', 'manufactured using', 'toxicology', 'biodegradable materials', 'composites materials', 'bioderived bulk', 'property law', 'engineering biomaterials', 'ecological design', 'textile art', 'stepbiotech horizonjucbeiaflag', 'biofuels biobased', 'fiber art', 'thin-film electronics', 'fibre fabrics', 'natural resource management', 'health biotechnology', 'ferroelectric materials', 'composites etc', 'contract law', 'european integration', 'transportation logistics problems', 'polymers composites', 'theory restoration', 'horizonjucbe biobased', 'electronic packaging', 'fine chemicals', 'morphology', 'optical fibers', 'additives adhesives', 'composites including', 'ceramics polymers', 'bioreactors', 'material based design', 'horizonjucbeiaflag horizonjucbe']</t>
+          <t>['robotic collaboration', 'waste management', 'marketing product brand management', 'medical biotechnology', 'biological agents', 'biological material', 'bioinformatics', 'toxicology', 'nutritional biotechnology', 'reinforced plastics', 'circularbydesign fibrebased', 'horizonjucbe biobased', 'etc polymers', 'yarn', 'recycling safeandsustainablebydesign', 'ceramics polymers', 'biobased europe', 'adhesives biobased', 'metals ceramics', 'biobased products', 'fabrics filled', 'packaging circular', 'materials packaging', 'circular packaging', 'steel', 'plastics cermets', 'biodegradable polymers', 'feedstock biobased', 'biotech industry', 'biosimilars', 'composition', 'laminates reinforced', 'adaptive reuse industrial heritage', 'biotech startups', 'chemical engineering', 'mechanical properties', 'operations research', 'plasticity', 'recycling technologies', 'biodefense', 'circular bioeconomy', 'biodegradable materials', 'circularity coatings', 'biomechanics', 'bulk fine', 'materials composites', 'quality', 'fibrebased packaging', 'bioreactors', 'european integration', 'humanitarian logistics', 'contract law', 'biological systems', 'fibre fabrics', 'logistics optimization', 'polymers plastics', 'natural resource management', 'filled composites', 'bioeconomy circular', 'astrophysics', 'biomaterials', 'circular biobased', 'biosecurity', 'technology fashion products', 'properties circular', 'pharmaceutical industry', 'biotechnology innovation', 'electronics manufacturing', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'mechanical engineering safety', 'european union', 'using biological', 'biomedical', 'products manufactured', 'black hole physics', 'packaging recycling', 'engineering biomaterials', 'property law', 'thin-film electronics', 'textile art', 'manufactured using', 'cermets combined', 'biotechnology', 'polymer materials engineering behaviors civil engineering', 'transportation logistics problems', 'freight transportation', 'theory restoration', 'morphology', 'mechanical structures', 'synthetic fibre', 'composites etc', 'health biotechnology', 'bioengineering', 'ecological design', 'composites including', 'materials science', 'safeandsustainablebydesign stepbiotech', 'biopolymer', 'astrobiology', 'coatings fibrebased', 'denture adhesives', 'materials engineering', 'product liability', 'composite materials', 'packaging improved', 'chemicals biobased', 'improved properties', 'additives adhesives', 'europe joint', 'synthetic biology', 'convergans clubs', 'materials biobased', 'european studies', 'biotech innovation', 'engineering materials', 'drug delivery', 'biomaterials metals', 'joint undertaking', 'stepbiotech horizonjucbeiaflag', 'fiber art', 'packaging packaging', 'including laminates', 'biofuels biobased', 'material based design', 'performance', 'packaging materials', 'polymers composites', 'bioderived bulk', 'fit', 'ferroelectric materials', 'bioenergy', 'biochemistry', 'manufacturing systems', 'optical fibers', 'products products', 'novel materials', 'biobased packaging', 'semiconductors', 'composites', 'plastics biofuels', 'packaging circularity', 'horizonjucbeiaflag horizonjucbe', 'biobased materials', 'natural synthetic', 'undertaking additives', 'biobased bioderived', 'technical textiles', 'electronic packaging', 'fine chemicals', 'composites materials', 'combined natural', 'biobased plastics', 'mechanical components', 'mechanical engineering materials']</t>
         </is>
       </c>
     </row>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>['nonwood forest', 'production planning', 'digital craft', 'carbon footprint', 'reverse logistics', 'logistics management', 'chemical engineering', 'forestry biomass', 'ecology', 'climate adaptation', 'material feedstock', 'undertaking agroforestry', 'biomass production', 'fit', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'synthetic biology', 'forest forest', 'biomolecular research', 'forestry forestry', 'bioprocessing', 'biodefense', 'nutritional biotechnology', 'stabilization programs banking', 'bulk fine', 'valorisation untapped', 'electronics manufacturing', 'biosecurity', 'marketing product brand management', 'biodegradable polymers', 'materials biobased', 'biobased products', 'deep ecology', 'biobased materials', 'biobased europe', 'untapped forest', 'biomaterials', 'humanitarian logistics', 'forest management', 'adaptation climate', 'robotic collaboration', 'bioinformatics', 'biotech innovation', 'virtual archeology', 'technology fashion products', 'products manufactured', 'logistics (warehouse management)', 'bioenergy', 'circular biobased', 'mechanical engineering materials', 'biotech startups', 'biopolymer', 'bioengineering', 'using biological', 'carbon reduction', 'agroforestry biobased', 'eg biofuels', 'restoration logistics', 'distribution agreements', 'ecosystem services', 'feedstock biobased', 'global value chains', 'biotechnology', 'joint undertaking', 'productivity', 'management forest', 'climate change', 'materials forest', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'steel', 'biobased chemicals', 'biosimilars', 'forest adaptation', 'management organization', 'products products', 'biochemistry', 'precision agriculture', 'biomedical', 'biological material', 'materials science', 'biomass circular', 'biobased bioderived', 'sustainable agriculture', 'biological agents', 'production eg', 'composite materials', 'concordat', 'logistics nonwood', 'plastics biofuels', 'novel materials', 'biotech industry', 'biodiversity conservation', 'logistics optimization', 'biobased plastics', 'pharmaceutical industry', 'carbon tax', 'change forestry', 'biofuels nonwood', 'biological systems', 'wood horizonjucberia', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'toxicology', 'biodegradable materials', 'land reclamation', 'bioderived bulk', 'biomass forest', 'biofuels biobased', 'climate', 'nonwood wood', 'ecosystem', 'adaptation', 'carbon capture', 'decision tree', 'natural resource management', 'contract law', 'european integration', 'theory restoration', 'logistics strategies', 'horizonjucberia horizonjucbe', 'horizonjucbe biobased', 'forest biomass', 'forest restoration', 'fine chemicals', 'pulp', 'forest products', 'bioreactors', 'material based design']</t>
+          <t>['robotic collaboration', 'stabilization programs banking', 'marketing product brand management', 'biological agents', 'biological material', 'nonwood wood', 'bioinformatics', 'toxicology', 'agroforestry biobased', 'nutritional biotechnology', 'logistics strategies', 'forest restoration', 'forestry biomass', 'logistics management', 'horizonjucbe biobased', 'biobased chemicals', 'land reclamation', 'restoration logistics', 'forest biomass', 'biobased europe', 'biobased products', 'carbon capture', 'sustainable agriculture', 'steel', 'carbon tax', 'ecology', 'wood horizonjucberia', 'biodegradable polymers', 'production planning', 'feedstock biobased', 'digital craft', 'undertaking agroforestry', 'biotech industry', 'carbon reduction', 'untapped forest', 'management organization', 'biosimilars', 'concordat', 'ecosystem services', 'adaptation climate', 'biotech startups', 'chemical engineering', 'biofuels nonwood', 'climate adaptation', 'biodefense', 'forestry forestry', 'biodegradable materials', 'bulk fine', 'quality', 'bioreactors', 'european integration', 'humanitarian logistics', 'contract law', 'climate', 'biological systems', 'virtual archeology', 'materials forest', 'logistics optimization', 'global value chains', 'horizonjucberia horizonjucbe', 'natural resource management', 'biomaterials', 'circular biobased', 'biosecurity', 'technology fashion products', 'forest products', 'biodiversity conservation', 'pulp', 'pharmaceutical industry', 'climate change', 'electronics manufacturing', 'material feedstock', 'biomolecular research', 'management forest', 'distribution agreements', 'technology', 'bioderived novel', 'european union', 'using biological', 'biomedical', 'products manufactured', 'black hole physics', 'logistics (warehouse management)', 'bioprocessing', 'valorisation untapped', 'change forestry', 'forest management', 'manufactured using', 'biomass forest', 'biotechnology', 'theory restoration', 'nonwood forest', 'logistics nonwood', 'eg biofuels', 'bioengineering', 'materials science', 'biopolymer', 'carbon footprint', 'deep ecology', 'astrobiology', 'biomass production', 'product liability', 'composite materials', 'ecosystem', 'chemicals biobased', 'decision tree', 'europe joint', 'synthetic biology', 'european studies', 'materials biobased', 'biotech innovation', 'joint undertaking', 'production eg', 'biofuels biobased', 'material based design', 'biomass circular', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'productivity', 'products products', 'novel materials', 'reverse logistics', 'plastics biofuels', 'adaptation', 'forest adaptation', 'biobased materials', 'biobased bioderived', 'fine chemicals', 'biobased plastics', 'precision agriculture', 'forest forest', 'mechanical engineering materials']</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>['geotechnics waste', 'civil engineering', 'logistics management', 'urban ecology', 'chemical engineering', 'waste prevention', 'material feedstock', 'fit', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'urban graphics', 'food waste', 'biotechnology urban', 'biomolecular research', 'engineering', 'bioprocessing', 'biodefense', 'nutritional biotechnology', 'bulk fine', 'waste treatment', 'electronics manufacturing', 'logistics safeandsustainablebydesign', 'astrophysics', 'biosecurity', 'marketing product brand management', 'biodegradable polymers', 'marine technology', 'materials biobased', 'biobased products', 'medical biotechnology', 'biobased materials', 'biobased europe', 'biomaterials', 'collection waste', 'materials civil', 'robotic collaboration', 'bioinformatics', 'biotech innovation', 'technology fashion products', 'products manufactured', 'urban waste', 'logistics (warehouse management)', 'bioenergy', 'urban studies', 'circular biobased', 'waste management', 'mechanical engineering materials', 'maritimehydraulic engineering', 'biopolymer', 'biotech startups', 'hydraulic engineering', 'bioengineering', 'waste collection', 'using biological', 'biorefinery circular', 'evaluation', 'biowaste biorefinery', 'bioimpedance analysis', 'engineering maritimehydraulic', 'distribution agreements', 'disease prevention', 'feedstock biobased', 'bioremediation', 'global value chains', 'biotechnology', 'circular bioeconomy', 'joint undertaking', 'products biowaste', 'geotechnical engineering', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'biosimilars', 'management organization', 'urban design', 'symbiosis waste', 'industrial engineering', 'products products', 'biochemistry', 'biomedical', 'undertaking biobased', 'safeandsustainablebydesign urbanindustrial', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'composite materials', 'biomechanics', 'valorisation circular', 'plastics biofuels', 'novel materials', 'biotech industry', 'urbanindustrial symbiosis', 'bioengineering solutions', 'industrial biotechnology', 'biobased plastics', 'logistics optimization', 'recycling technologies', 'pharmaceutical industry', 'industrial design', 'biological systems', 'management waste', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'toxicology', 'biodegradable materials', 'engineering geotechnics', 'bioderived bulk', 'treatment industrial', 'ecological design', 'stepbiotech horizonjucbeiaflag', 'biofuels biobased', 'prevention stepbiotech', 'health biotechnology', 'urban morhology', 'contract law', 'european integration', 'waste waste', 'logistics strategies', 'horizonjucbe biobased', 'bioeconomy logistics', 'fine chemicals', 'morphology', 'symbiosis biowaste', 'values', 'bioreactors', 'biowaste valorisation', 'material based design', 'maritime delimitation', 'horizonjucbeiaflag horizonjucbe']</t>
+          <t>['robotic collaboration', 'evaluation', 'waste management', 'waste treatment', 'marketing product brand management', 'medical biotechnology', 'biological agents', 'maritimehydraulic engineering', 'biological material', 'bioinformatics', 'toxicology', 'nutritional biotechnology', 'logistics strategies', 'logistics management', 'horizonjucbe biobased', 'geotechnical engineering', 'prevention stepbiotech', 'biobased europe', 'biobased products', 'biodegradable polymers', 'logistics safeandsustainablebydesign', 'feedstock biobased', 'biotech industry', 'valorisation circular', 'civil engineering', 'management organization', 'values', 'bioimpedance analysis', 'biosimilars', 'bioengineering solutions', 'disease prevention', 'maritime delimitation', 'biotech startups', 'chemical engineering', 'urban morhology', 'recycling technologies', 'biodefense', 'circular bioeconomy', 'biodegradable materials', 'waste prevention', 'biomechanics', 'bulk fine', 'quality', 'safeandsustainablebydesign urbanindustrial', 'geotechnics waste', 'bioreactors', 'european integration', 'contract law', 'biological systems', 'urban design', 'logistics optimization', 'products biowaste', 'urban waste', 'global value chains', 'astrophysics', 'biomaterials', 'circular biobased', 'biosecurity', 'technology fashion products', 'pharmaceutical industry', 'urbanindustrial symbiosis', 'biowaste biorefinery', 'urban graphics', 'electronics manufacturing', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'european union', 'using biological', 'biomedical', 'engineering geotechnics', 'biotechnology urban', 'symbiosis biowaste', 'products manufactured', 'engineering', 'black hole physics', 'urban studies', 'industrial design', 'logistics (warehouse management)', 'bioprocessing', 'engineering maritimehydraulic', 'urban ecology', 'biorefinery circular', 'manufactured using', 'biotechnology', 'industrial biotechnology', 'food waste', 'morphology', 'health biotechnology', 'bioengineering', 'ecological design', 'bioeconomy logistics', 'materials civil', 'materials science', 'biopolymer', 'biowaste valorisation', 'waste waste', 'astrobiology', 'waste collection', 'management waste', 'product liability', 'composite materials', 'industrial engineering', 'chemicals biobased', 'europe joint', 'european studies', 'materials biobased', 'biotech innovation', 'joint undertaking', 'stepbiotech horizonjucbeiaflag', 'symbiosis waste', 'marine technology', 'biofuels biobased', 'hydraulic engineering', 'material based design', 'bioderived bulk', 'fit', 'bioremediation', 'bioenergy', 'biochemistry', 'manufacturing systems', 'undertaking biobased', 'products products', 'novel materials', 'plastics biofuels', 'horizonjucbeiaflag horizonjucbe', 'collection waste', 'biobased materials', 'biobased bioderived', 'fine chemicals', 'biobased plastics', 'mechanical engineering materials', 'treatment industrial']</t>
         </is>
       </c>
     </row>
@@ -3828,7 +3828,7 @@
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>['actor training', 'space deployment', 'strategic communication', 'systems institutions', 'chemical engineering', 'material feedstock', 'fit', 'learning systems', 'european union', 'europe joint', 'knowledge infrastructure', 'european studies', 'quality', 'black hole physics', 'biomolecular research', 'qualitative research', 'biodefense', 'nutritional biotechnology', 'new curricula', 'bulk fine', 'ability capabilities', 'electronics manufacturing', 'exchange practices', 'ontology', 'institutions teaching', 'marketing product brand management', 'biodegradable polymers', 'knowledge technology', 'capabilities capability', 'materials biobased', 'biobased products', 'higher education', 'biobased materials', 'biobased europe', 'biobased systems', 'competence competencies', 'biomaterials', 'semantic networks', 'quality management system', 'research methods', 'business capabilities', 'relevant biobased', 'social media best practices', 'intellectual history', 'robotic collaboration', 'information technology', 'bioinformatics', 'biotech innovation', 'technology fashion products', 'products manufactured', 'turkeyeu relations', 'develop deploy', 'qualitifcation horizonjucbecsa', 'bioenergy', 'technology transfer', 'circular biobased', 'practices relevant', 'mechanical engineering materials', 'horizonjucbecsa horizonjucbe', 'biotech startups', 'biopolymer', 'bioengineering', 'using biological', 'teaching learning', 'education', 'capability competence', 'systems engineering', 'abilities ability', 'distribution agreements', 'feedstock biobased', 'electronic commerce', 'biotechnology', 'joint undertaking', 'systems circular', 'deploy new', 'cae methodology development', 'chemicals biobased', 'learning knowledge', 'bioderived novel', 'biomedical systems', 'social institutions', 'performance studies', 'public relations', 'dynamic systems', 'products products', 'biochemistry', 'biomedical', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'marketing communication', 'design ability', 'composite materials', 'performance', 'concordat', 'plastics biofuels', 'novel materials', 'biotech industry', 'materials education', 'sociology of education', 'transmedia', 'bioengineering solutions', 'logistics optimization', 'expertise qualitifcation', 'biobased plastics', 'pharmaceutical industry', 'competencies competency', 'competency expertise', 'educational psychology', 'system dynamics', 'biological systems', 'cognitive learning', 'bioethics', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'toxicology', 'biodegradable materials', 'bioderived bulk', 'biofuels biobased', 'foreign language teaching', 'autonomy development', 'knowledge exchange', 'adaptation', 'child studies', 'educational technologies', 'communication', 'undertaking abilities', 'education systems', 'contract law', 'european integration', 'knowledge discovery', 'horizonjucbe biobased', 'curricula knowledge', 'accreditation', 'artificial intelligence research', 'fine chemicals', 'transfer knowledge', 'systems theory', 'bioreactors', 'material based design', 'robotic deployment']</t>
+          <t>['marketing communication', 'robotic collaboration', 'sociology of education', 'strategic communication', 'learning systems', 'marketing product brand management', 'biological agents', 'higher education', 'biological material', 'bioinformatics', 'toxicology', 'competency expertise', 'nutritional biotechnology', 'horizonjucbe biobased', 'artificial intelligence research', 'systems theory', 'biobased europe', 'biobased products', 'bioethics', 'transmedia', 'capabilities capability', 'qualitative research', 'biodegradable polymers', 'robotic deployment', 'feedstock biobased', 'learning knowledge', 'business capabilities', 'biotech industry', 'foreign language teaching', 'qualitifcation horizonjucbecsa', 'child studies', 'systems engineering', 'concordat', 'education systems', 'bioengineering solutions', 'information technology', 'social institutions', 'educational technologies', 'biotech startups', 'chemical engineering', 'biodefense', 'biodegradable materials', 'bulk fine', 'horizonjucbecsa horizonjucbe', 'quality', 'bioreactors', 'european integration', 'contract law', 'biological systems', 'logistics optimization', 'communication', 'ontology', 'biobased systems', 'deploy new', 'biomaterials', 'circular biobased', 'public relations', 'technology fashion products', 'pharmaceutical industry', 'education', 'actor training', 'competencies competency', 'knowledge discovery', 'electronics manufacturing', 'develop deploy', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'european union', 'using biological', 'system dynamics', 'biomedical', 'products manufactured', 'knowledge technology', 'undertaking abilities', 'capability competence', 'black hole physics', 'transfer knowledge', 'curricula knowledge', 'research methods', 'cae methodology development', 'space deployment', 'manufactured using', 'biotechnology', 'new curricula', 'electronic commerce', 'bioengineering', 'technology transfer', 'materials science', 'biopolymer', 'knowledge infrastructure', 'ability capabilities', 'relevant biobased', 'teaching learning', 'materials education', 'systems circular', 'exchange practices', 'product liability', 'composite materials', 'semantic networks', 'chemicals biobased', 'intellectual history', 'performance studies', 'europe joint', 'abilities ability', 'materials biobased', 'european studies', 'biotech innovation', 'biomedical systems', 'joint undertaking', 'design ability', 'institutions teaching', 'biofuels biobased', 'material based design', 'performance', 'systems institutions', 'educational psychology', 'cognitive learning', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'social media best practices', 'products products', 'novel materials', 'knowledge exchange', 'expertise qualitifcation', 'accreditation', 'quality management system', 'plastics biofuels', 'autonomy development', 'adaptation', 'biobased materials', 'competence competencies', 'biobased bioderived', 'fine chemicals', 'biobased plastics', 'dynamic systems', 'mechanical engineering materials', 'practices relevant', 'turkeyeu relations']</t>
         </is>
       </c>
     </row>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>['space maintenance', 'environmental sustainability', 'chemical engineering', 'experimental economics', 'materials bioprocessing', 'material feedstock', 'fit', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'bioconversion biorefinery', 'biocatalysis fermentation', 'synthetic biology', 'biobased dropinssmart', 'biomolecular research', 'bioengineering applications', 'biorefinery safeandsustainablebydesign', 'bioprocessing', 'biodefense', 'machine automation', 'nutritional biotechnology', 'bulk fine', 'variable selection', 'sustainable technology', 'drive process', 'electronics manufacturing', 'multi-agent systems', 'astrophysics', 'power conversion', 'horizonjucbe applied', 'biosecurity', 'marketing product brand management', 'biodegradable polymers', 'cognitive processes', 'materials biobased', 'regulatory biotechnology', 'biobased products', 'medical biotechnology', 'biobased materials', 'biobased europe', 'self-driving cars', 'dropin platform', 'biomaterials', 'applied industrial', 'fermentation industrial', 'robotic collaboration', 'metabolic engineering', 'conversion biomass', 'bioinformatics', 'biotech innovation', 'technology fashion products', 'products manufactured', 'resourceefficient conversion', 'platform employees', 'bioenergy', 'circular biobased', 'digital services', 'industrial data', 'mechanical engineering materials', 'sustainable energy', 'biotech startups', 'biopolymer', 'bioengineering', 'dropinssmart dropin', 'using biological', 'social media platforms', 'carbon reduction', 'sustainability stepbiotech', 'drug delivery', 'applied macro', 'distribution agreements', 'feedstock biobased', 'biotechnology', 'joint undertaking', 'sustainability', 'cae methodology development', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'robotic consulting', 'controlled drug delivery systems', 'biobased chemicals', 'dependency criteria', 'biosimilars', 'safeandsustainablebydesign sustainability', 'industrial engineering', 'processes relying', 'products products', 'products bioconversion', 'biochemistry', 'bioengineering industrial', 'energy efficiency', 'industrial processes', 'process biocatalysis', 'biomedical', 'undertaking biobased', 'biological material', 'materials science', 'industrial chemistry', 'biomass circular', 'via costeffective', 'biobased bioderived', 'biological agents', 'chemicals via', 'composite materials', 'software', 'relying biological', 'biocompability', 'plastics biofuels', 'novel materials', 'biotech industry', 'sustainable resourceefficient', 'costeffective sustainable', 'bioengineering solutions', 'logistics optimization', 'industrial biotechnology', 'biobased plastics', 'pharmaceutical industry', 'industrial design', 'chemistry biobased', 'biological systems', 'platform chemicals', 'bioprocessing technologies', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'radicalisation', 'toxicology', 'biodegradable materials', 'biobased dropin', 'bioderived bulk', 'agents drive', 'stepbiotech horizonjucbeiaflag', 'biofuels biobased', 'generative algorithms', 'bioengineering technologies', 'carbon capture', 'health biotechnology', 'decarbonization', 'technologies industrial', 'contract law', 'european integration', 'signal conversion', 'fine chemicals', 'industrial bioengineering', 'bioreactors', 'material based design', 'cognitive processes work', 'sustainable consumption', 'horizonjucbeiaflag horizonjucbe']</t>
+          <t>['sustainable technology', 'bioprocessing technologies', 'industrial processes', 'robotic collaboration', 'biocompability', 'biological agents', 'medical biotechnology', 'marketing product brand management', 'relying biological', 'biological material', 'bioinformatics', 'drive process', 'environmental sustainability', 'toxicology', 'nutritional biotechnology', 'fermentation industrial', 'biobased chemicals', 'sustainable consumption', 'biobased europe', 'biobased products', 'agents drive', 'carbon capture', 'industrial chemistry', 'biodegradable polymers', 'feedstock biobased', 'biotech industry', 'carbon reduction', 'chemistry biobased', 'biosimilars', 'bioengineering solutions', 'space maintenance', 'multi-agent systems', 'products bioconversion', 'biotech startups', 'chemical engineering', 'biodefense', 'biodegradable materials', 'applied macro', 'bulk fine', 'materials bioprocessing', 'quality', 'bioreactors', 'european integration', 'contract law', 'biological systems', 'logistics optimization', 'controlled drug delivery systems', 'astrophysics', 'biomaterials', 'circular biobased', 'biosecurity', 'technology fashion products', 'robotic consulting', 'conversion biomass', 'biobased dropin', 'pharmaceutical industry', 'platform employees', 'electronics manufacturing', 'software', 'bioengineering industrial', 'material feedstock', 'biomolecular research', 'distribution agreements', 'costeffective sustainable', 'bioderived novel', 'technology', 'european union', 'using biological', 'biomedical', 'sustainable resourceefficient', 'products manufactured', 'black hole physics', 'biobased dropinssmart', 'dropinssmart dropin', 'process biocatalysis', 'sustainability', 'industrial design', 'applied industrial', 'bioprocessing', 'horizonjucbe applied', 'decarbonization', 'industrial data', 'cae methodology development', 'manufactured using', 'cognitive processes work', 'biotechnology', 'industrial biotechnology', 'technologies industrial', 'biorefinery safeandsustainablebydesign', 'safeandsustainablebydesign sustainability', 'health biotechnology', 'bioengineering', 'materials science', 'biopolymer', 'via costeffective', 'machine automation', 'resourceefficient conversion', 'radicalisation', 'astrobiology', 'sustainable energy', 'industrial engineering', 'product liability', 'composite materials', 'bioengineering technologies', 'chemicals biobased', 'regulatory biotechnology', 'metabolic engineering', 'experimental economics', 'self-driving cars', 'europe joint', 'energy efficiency', 'synthetic biology', 'materials biobased', 'european studies', 'biotech innovation', 'industrial bioengineering', 'drug delivery', 'signal conversion', 'joint undertaking', 'stepbiotech horizonjucbeiaflag', 'bioengineering applications', 'dependency criteria', 'cognitive processes', 'biofuels biobased', 'material based design', 'biomass circular', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'undertaking biobased', 'dropin platform', 'products products', 'novel materials', 'biocatalysis fermentation', 'processes relying', 'plastics biofuels', 'sustainability stepbiotech', 'horizonjucbeiaflag horizonjucbe', 'chemicals via', 'biobased materials', 'variable selection', 'biobased bioderived', 'social media platforms', 'power conversion', 'fine chemicals', 'generative algorithms', 'digital services', 'biobased plastics', 'platform chemicals', 'mechanical engineering materials', 'bioconversion biorefinery']</t>
         </is>
       </c>
     </row>
@@ -3902,7 +3902,7 @@
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>['space maintenance', 'mechanical devices', 'elastomers isoprenoids', 'biomanufacturing elastomers', 'chemical engineering', 'plant genetics', 'biotechnology innovation', 'natural rubber', 'materials bioprocessing', 'material feedstock', 'microbiology', 'fit', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'rubber horizonjucberia', 'biocatalysis fermentation', 'synthetic biology', 'genetic testing', 'biomolecular research', 'plant genetic', 'bioengineering applications', 'machine automation', 'bioprocessing', 'biodefense', 'nutritional biotechnology', 'road engineering', 'bulk fine', 'drive process', 'electronics manufacturing', 'rubber circular', 'enzymology', 'multi-agent systems', 'marketing product brand management', 'biodegradable polymers', 'cognitive processes', 'materials biobased', 'composites', 'biobased products', 'medical biotechnology', 'transgenic organisms', 'biobased materials', 'biobased europe', 'self-driving cars', 'biomanufacturing routes', 'biomaterials', 'genetic modification', 'mechanical', 'biobased synthetic', 'robotic collaboration', 'metabolic engineering', 'bioinformatics', 'synthetic rubber', 'biotech innovation', 'technology fashion products', 'products manufactured', 'flexible electronics', 'travel writing', 'genetic engineering', 'bioenergy', 'circular biobased', 'mechanical engineering materials', 'biotech startups', 'biopolymer', 'bioengineering', 'using biological', 'isoprenoids natural', 'distribution agreements', 'genetic resources', 'feedstock biobased', 'products biobased', 'thermofluids', 'biotechnology', 'joint undertaking', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'robotic consulting', 'dependency criteria', 'industrial engineering', 'processes relying', 'products products', 'genetics rubber', 'biochemistry', 'industrial processes', 'process biocatalysis', 'biomedical', 'undertaking biobased', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'composite materials', 'concordat', 'relying biological', 'biocompability', 'plastics biofuels', 'novel materials', 'biotech industry', 'transportation planning', 'fermentation plant', 'bioengineering solutions', 'logistics optimization', 'biobased plastics', 'natural synthetic', 'space debris', 'pharmaceutical industry', 'anthropocene', 'industrial design', 'biological systems', 'bioprocessing technologies', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'toxicology', 'biodegradable materials', 'genetic predisposition', 'bioderived bulk', 'agents drive', 'biofuels biobased', 'bioengineering technologies', 'routes natural', 'technologies industrial', 'alternative biomanufacturing', 'contract law', 'european integration', 'horizonjucberia horizonjucbe', 'horizonjucbe biobased', 'fine chemicals', 'pulp', 'rubber plant', 'bioreactors', 'material based design', 'cognitive processes work', 'rubber biomanufacturing']</t>
+          <t>['bioprocessing technologies', 'industrial processes', 'robotic collaboration', 'space debris', 'biocompability', 'biomanufacturing elastomers', 'biological agents', 'rubber plant', 'medical biotechnology', 'relying biological', 'routes natural', 'marketing product brand management', 'biological material', 'alternative biomanufacturing', 'bioinformatics', 'drive process', 'biomanufacturing routes', 'toxicology', 'transportation planning', 'nutritional biotechnology', 'horizonjucbe biobased', 'rubber circular', 'biobased europe', 'biobased products', 'agents drive', 'biodegradable polymers', 'feedstock biobased', 'plant genetics', 'biotech industry', 'genetic modification', 'concordat', 'bioengineering solutions', 'space maintenance', 'multi-agent systems', 'mechanical', 'fermentation plant', 'biotech startups', 'chemical engineering', 'biodefense', 'biodegradable materials', 'natural rubber', 'bulk fine', 'materials bioprocessing', 'quality', 'bioreactors', 'european integration', 'genetic predisposition', 'genetics rubber', 'contract law', 'biological systems', 'logistics optimization', 'enzymology', 'horizonjucberia horizonjucbe', 'biomaterials', 'circular biobased', 'flexible electronics', 'technology fashion products', 'robotic consulting', 'pulp', 'pharmaceutical industry', 'biotechnology innovation', 'transgenic organisms', 'electronics manufacturing', 'mechanical devices', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'plant genetic', 'european union', 'using biological', 'biomedical', 'products manufactured', 'black hole physics', 'process biocatalysis', 'industrial design', 'bioprocessing', 'genetic engineering', 'manufactured using', 'thermofluids', 'cognitive processes work', 'biotechnology', 'technologies industrial', 'synthetic rubber', 'bioengineering', 'materials science', 'biopolymer', 'machine automation', 'astrobiology', 'isoprenoids natural', 'product liability', 'industrial engineering', 'bioengineering technologies', 'road engineering', 'composite materials', 'microbiology', 'chemicals biobased', 'genetic resources', 'metabolic engineering', 'self-driving cars', 'products biobased', 'europe joint', 'synthetic biology', 'european studies', 'materials biobased', 'biotech innovation', 'biobased synthetic', 'genetic testing', 'joint undertaking', 'bioengineering applications', 'dependency criteria', 'cognitive processes', 'rubber biomanufacturing', 'elastomers isoprenoids', 'biofuels biobased', 'material based design', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'undertaking biobased', 'travel writing', 'products products', 'novel materials', 'biocatalysis fermentation', 'processes relying', 'composites', 'plastics biofuels', 'biobased materials', 'natural synthetic', 'anthropocene', 'rubber horizonjucberia', 'biobased bioderived', 'fine chemicals', 'biobased plastics', 'mechanical engineering materials']</t>
         </is>
       </c>
     </row>
@@ -3939,7 +3939,7 @@
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>['space maintenance', 'carbon footprint', 'reconversion retrofitting', 'biotechnology industrial', 'logistics management', 'chemical engineering', 'biotechnology innovation', 'ecology', 'moral values', 'biomass conversion', 'material feedstock', 'materials bioprocessing', 'fit', 'european union', 'hybrid', 'europe joint', 'european studies', 'quality', 'black hole physics', 'data wrangling', 'biocatalysis fermentation', 'synthetic biology', 'biomolecular research', 'bioengineering applications', 'machine automation', 'bioprocessing', 'conflict resolution', 'biodefense', 'nutritional biotechnology', 'bulk fine', 'highervalue biobased', 'sustainable technology', 'drive process', 'electronics manufacturing', 'multi-agent systems', 'astrophysics', 'supply chain management', 'power conversion', 'biosecurity', 'marketing product brand management', 'biodegradable polymers', 'cognitive processes', 'materials biobased', 'economy', 'biobased products', 'medical biotechnology', 'biobased materials', 'biobased europe', 'self-driving cars', 'biomaterials', 'secondary biomass', 'cascading use', 'architectural restoration adaptive reuse', 'fermentation industrial', 'robotic collaboration', 'metabolic engineering', 'plants towards', 'conversion biomass', 'bioinformatics', 'biotech innovation', 'technology fashion products', 'products manufactured', 'biorefineries industrial', 'logistics (warehouse management)', 'bioenergy', 'retrofitting biorefineries', 'circular biobased', 'industrial data', 'mechanical engineering materials', 'biotech startups', 'modeling', 'sustainable energy', 'biopolymer', 'bioengineering', 'adaptive reuse industrial heritage', 'using biological', 'carbon reduction', 'sectoral change', 'sustainability stepbiotech', 'distribution agreements', 'economic transformation', 'feedstock biobased', 'bioremediation', 'global value chains', 'biotechnology', 'joint undertaking', 'supply logistics', 'sustainability', 'chemicals biobased', 'astrobiology', 'biorefinery cascading', 'bioderived novel', 'robotic consulting', 'biobased chemicals', 'dependency criteria', 'biosimilars', 'change innovation.', 'industrial engineering', 'processes relying', 'products products', 'biochemistry', 'industrial processes', 'process biocatalysis', 'biomedical', 'undertaking biobased', 'products biomass', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'products circular', 'biomass industrial', 'composite materials', 'plant industrial', 'retrofitting secondary', 'relying biological', 'use biomass', 'industrial sectoral', 'biocompability', 'plastics biofuels', 'novel materials', 'biotech industry', 'demographic change', 'bioengineering solutions', 'logistics optimization', 'industrial biotechnology', 'biobased plastics', 'pharmaceutical industry', 'industrial design', 'industrial plant', 'biological systems', 'bioprocessing technologies', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'toxicology', 'biodegradable materials', 'bioderived bulk', 'industrial reconversion', 'agents drive', 'stepbiotech horizonjucbeiaflag', 'biofuels biobased', 'energy harvesting', 'towards highervalue', 'ecosystem', 'bioengineering technologies', 'industrial plants', 'adaptation', 'logistics biorefinery', 'carbon capture', 'health biotechnology', 'technologies industrial', 'contract law', 'european integration', 'functional upgrade', 'logistics strategies', 'horizonjucbe biobased', 'biomass sustainability', 'biomass supply', 'fine chemicals', 'values', 'bioreactors', 'material based design', 'cognitive processes work', 'horizonjucbeiaflag horizonjucbe']</t>
+          <t>['sustainable technology', 'conflict resolution', 'bioprocessing technologies', 'industrial processes', 'robotic collaboration', 'economic transformation', 'biocompability', 'biorefineries industrial', 'biological agents', 'marketing product brand management', 'medical biotechnology', 'relying biological', 'biological material', 'bioinformatics', 'drive process', 'industrial plants', 'toxicology', 'nutritional biotechnology', 'logistics strategies', 'change innovation.', 'logistics management', 'horizonjucbe biobased', 'fermentation industrial', 'biobased chemicals', 'supply chain management', 'biobased products', 'biobased europe', 'agents drive', 'economy', 'cascading use', 'highervalue biobased', 'use biomass', 'carbon capture', 'ecology', 'biodegradable polymers', 'feedstock biobased', 'biotech industry', 'carbon reduction', 'values', 'biosimilars', 'bioengineering solutions', 'space maintenance', 'products biomass', 'multi-agent systems', 'adaptive reuse industrial heritage', 'biotech startups', 'chemical engineering', 'biodefense', 'biodegradable materials', 'bulk fine', 'materials bioprocessing', 'quality', 'reconversion retrofitting', 'bioreactors', 'european integration', 'contract law', 'industrial reconversion', 'biological systems', 'industrial plant', 'logistics optimization', 'demographic change', 'retrofitting secondary', 'global value chains', 'astrophysics', 'biomaterials', 'circular biobased', 'biosecurity', 'technology fashion products', 'robotic consulting', 'conversion biomass', 'pharmaceutical industry', 'biotechnology innovation', 'electronics manufacturing', 'modeling', 'material feedstock', 'biomolecular research', 'distribution agreements', 'biotechnology industrial', 'technology', 'bioderived novel', 'european union', 'using biological', 'biomedical', 'plants towards', 'products manufactured', 'black hole physics', 'process biocatalysis', 'industrial design', 'sustainability', 'logistics (warehouse management)', 'energy harvesting', 'bioprocessing', 'biorefinery cascading', 'data wrangling', 'industrial data', 'biomass conversion', 'functional upgrade', 'biomass supply', 'industrial sectoral', 'manufactured using', 'cognitive processes work', 'biotechnology', 'industrial biotechnology', 'architectural restoration adaptive reuse', 'technologies industrial', 'health biotechnology', 'bioengineering', 'biomass industrial', 'towards highervalue', 'materials science', 'biopolymer', 'carbon footprint', 'sectoral change', 'machine automation', 'astrobiology', 'plant industrial', 'sustainable energy', 'industrial engineering', 'product liability', 'composite materials', 'bioengineering technologies', 'ecosystem', 'chemicals biobased', 'metabolic engineering', 'self-driving cars', 'europe joint', 'synthetic biology', 'materials biobased', 'european studies', 'biotech innovation', 'joint undertaking', 'stepbiotech horizonjucbeiaflag', 'bioengineering applications', 'dependency criteria', 'cognitive processes', 'supply logistics', 'biofuels biobased', 'material based design', 'products circular', 'bioderived bulk', 'fit', 'bioremediation', 'bioenergy', 'biochemistry', 'manufacturing systems', 'undertaking biobased', 'retrofitting biorefineries', 'products products', 'novel materials', 'biocatalysis fermentation', 'secondary biomass', 'processes relying', 'plastics biofuels', 'logistics biorefinery', 'sustainability stepbiotech', 'horizonjucbeiaflag horizonjucbe', 'adaptation', 'biobased materials', 'hybrid', 'biomass sustainability', 'biobased bioderived', 'power conversion', 'fine chemicals', 'moral values', 'biobased plastics', 'mechanical engineering materials']</t>
         </is>
       </c>
     </row>
@@ -3976,7 +3976,7 @@
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>['kelp mariculture', 'production planning', 'local food', 'fisheries biobased', 'chemical engineering', 'biotechnology innovation', 'ecology', 'material feedstock', 'fit', 'plants products', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'biomolecular research', 'bioengineering applications', 'engineering', 'bioprocessing', 'biodefense', 'nutritional biotechnology', 'bulk fine', 'horizonjucbe aquaculture', 'applications cultivation', 'electronics manufacturing', 'system design', 'oceanography', 'green technologies', 'freshwater kelp', 'enzymology', 'astrophysics', 'eco-design', 'aquaculture fisheries', 'marketing product brand management', 'biodegradable polymers', 'products environment', 'marine technology', 'materials biobased', 'aquafarming benthic', 'biobased products', 'medical biotechnology', 'deep ecology', 'biobased materials', 'smart systems', 'ethnography', 'biobased europe', 'biomaterials', 'aquaculture aquafarming', 'biotechnological applications', 'social media innovation', 'macroalgae systems', 'production systems', 'robotic collaboration', 'technology fashion products', 'biotech innovation', 'products manufactured', 'bioenergy', 'circular biobased', 'mechanical engineering materials', 'biotech startups', 'mechanical engineering production', 'biopolymer', 'bioengineering', 'using biological', 'dynamical systems', 'optimised production', 'systems engineering', 'petroleum engineering', 'distribution agreements', 'feedstock biobased', 'addedvalue applications', 'biotechnology', 'systems innovative', 'joint undertaking', 'systems circular', 'benthic freshwater', 'sustainability', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'materials chemical', 'environmental engineering', 'change innovation.', 'mobile applications', 'biotechnology companies', 'dynamic systems', 'marine ecosystem', 'products products', 'biochemistry', 'water resources engineering', 'mariculture seaweed', 'biomedical', 'biological material', 'materials science', 'seaweed stepbiotech', 'biobased bioderived', 'biological agents', 'composite materials', 'software', 'innovative addedvalue', 'plastics biofuels', 'novel materials', 'biotech industry', 'renewable materials', 'logistics optimization', 'biobased plastics', 'pharmaceutical industry', 'aquaculture interactions', 'horizonjucbeia horizonjucbe', 'system dynamics', 'cultivation optimised', 'biological systems', 'growth development', 'estuaries rivers (wave', 'undertaking algaculture', 'manufacturing systems', 'product liability', 'manufactured using', 'technology', 'toxicology', 'biodegradable materials', 'law sea', 'bioderived bulk', 'biofuels biobased', 'sustainable macroalgae', 'algaculture aquaculture', 'engineering plants', 'health biotechnology', 'stepbiotech horizonjucbeia', 'seas', 'contract law', 'african culture', 'european integration', 'food heritage', 'fine chemicals', 'fisheries aquaculture', 'environment fisheries', 'values', 'systems theory', 'bioreactors', 'material based design', 'sustainable consumption']</t>
+          <t>['robotic collaboration', 'food heritage', 'marketing product brand management', 'medical biotechnology', 'biological agents', 'biological material', 'law sea', 'toxicology', 'nutritional biotechnology', 'change innovation.', 'stepbiotech horizonjucbeia', 'systems theory', 'sustainable consumption', 'fisheries aquaculture', 'environment fisheries', 'biobased europe', 'biobased products', 'fisheries biobased', 'products environment', 'production planning', 'ecology', 'biodegradable polymers', 'feedstock biobased', 'ethnography', 'biotech industry', 'optimised production', 'values', 'estuaries rivers (wave', 'systems engineering', 'aquaculture fisheries', 'mobile applications', 'materials chemical', 'smart systems', 'biotech startups', 'chemical engineering', 'seas', 'biodefense', 'biodegradable materials', 'horizonjucbeia horizonjucbe', 'bulk fine', 'oceanography', 'mariculture seaweed', 'benthic freshwater', 'quality', 'bioreactors', 'european integration', 'contract law', 'biological systems', 'logistics optimization', 'enzymology', 'astrophysics', 'biomaterials', 'circular biobased', 'technology fashion products', 'growth development', 'pharmaceutical industry', 'plants products', 'biotechnology innovation', 'local food', 'electronics manufacturing', 'software', 'material feedstock', 'biomolecular research', 'distribution agreements', 'system design', 'bioderived novel', 'technology', 'european union', 'using biological', 'biotechnological applications', 'system dynamics', 'biotechnology companies', 'biomedical', 'products manufactured', 'engineering', 'black hole physics', 'applications cultivation', 'algaculture aquaculture', 'sustainability', 'dynamical systems', 'marine ecosystem', 'bioprocessing', 'engineering plants', 'freshwater kelp', 'green technologies', 'manufactured using', 'biotechnology', 'environmental engineering', 'kelp mariculture', 'systems innovative', 'seaweed stepbiotech', 'social media innovation', 'health biotechnology', 'bioengineering', 'materials science', 'biopolymer', 'deep ecology', 'water resources engineering', 'astrobiology', 'systems circular', 'product liability', 'horizonjucbe aquaculture', 'composite materials', 'chemicals biobased', 'europe joint', 'materials biobased', 'european studies', 'biotech innovation', 'innovative addedvalue', 'joint undertaking', 'macroalgae systems', 'bioengineering applications', 'marine technology', 'cultivation optimised', 'mechanical engineering production', 'addedvalue applications', 'biofuels biobased', 'material based design', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'products products', 'novel materials', 'petroleum engineering', 'sustainable macroalgae', 'plastics biofuels', 'african culture', 'aquaculture interactions', 'biobased materials', 'eco-design', 'biobased bioderived', 'renewable materials', 'fine chemicals', 'biobased plastics', 'aquafarming benthic', 'dynamic systems', 'aquaculture aquafarming', 'mechanical engineering materials', 'undertaking algaculture', 'production systems']</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>['composition', 'space maintenance', 'drink processing', 'local food', 'alternative sources', 'processing nutrition', 'protein engineering', 'chemical engineering', 'ecology', 'materials bioprocessing', 'material feedstock', 'insect livestock', 'fit', 'european union', 'europe joint', 'additives food', 'european studies', 'quality', 'black hole physics', 'food waste', 'biocatalysis fermentation', 'biomolecular research', 'bioengineering applications', 'machine automation', 'bioprocessing', 'biodefense', 'nutritional biotechnology', 'scalingup nutritional', 'bulk fine', 'drive process', 'amino acid', 'fishmeal hydrolysate', 'electronics manufacturing', 'local cuisines turkey', 'multi-agent systems', 'astrophysics', 'planetary science', 'marketing product brand management', 'biodegradable polymers', 'cognitive processes', 'materials biobased', 'nutritional supplements', 'biobased products', 'medical nutrition therapy diseases', 'medical biotechnology', 'biobased materials', 'biobased europe', 'self-driving cars', 'therapeutic proteins', 'biomaterials', 'research methods', 'feedstuff fishmeal', 'robotic collaboration', 'metabolic engineering', 'bioinformatics', 'biotech innovation', 'technology fashion products', 'meal nourishment', 'products manufactured', 'protein biochemistry', 'bioenergy', 'undertaking amino', 'food chemistry', 'hydropower', 'circular biobased', 'mechanical engineering materials', 'biopolymer', 'biotech startups', 'social influence', 'alternative media', 'bioengineering', 'functional foods', 'using biological', 'livestock meal', 'turkish cuisine', 'fermentation feed', 'distribution agreements', 'feedstock biobased', 'feed additives', 'biotechnology', 'joint undertaking', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'robotic consulting', 'water purification', 'dependency criteria', 'alternative organizations', 'industrial engineering', 'processes relying', 'products products', 'biochemistry', 'industrial processes', 'hydrolysate insect', 'process biocatalysis', 'water resources engineering', 'biomedical', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'composite materials', 'relying biological', 'seasonal agricultural work', 'biocompability', 'plastics biofuels', 'novel materials', 'biotech industry', 'logistics optimization', 'biobased plastics', 'pharmaceutical industry', 'horizonjucbeia horizonjucbe', 'poultry stepbiotech', 'industrial design', 'nutrition dietetics', 'biological systems', 'bioprocessing technologies', 'estuaries rivers (wave', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'clinical nutrition', 'toxicology', 'biodegradable materials', 'bioderived bulk', 'diet feedstuff', 'agents drive', 'proteins alternative', 'biofuels biobased', 'nourishment poultry', 'sports nutrition', 'bioengineering technologies', 'health biotechnology', 'sources circular', 'stepbiotech horizonjucbeia', 'technologies industrial', 'contract law', 'european integration', 'horizonjucbe biobased', 'food drink', 'food heritage', 'nutritional proteins', 'fine chemicals', 'ottoman period food beverage enterprises', 'bioreactors', 'material based design', 'cognitive processes work', 'acid diet']</t>
+          <t>['bioprocessing technologies', 'industrial processes', 'robotic collaboration', 'food heritage', 'turkish cuisine', 'water purification', 'acid diet', 'biocompability', 'biological agents', 'medical biotechnology', 'marketing product brand management', 'relying biological', 'biological material', 'bioinformatics', 'drive process', 'toxicology', 'nutritional biotechnology', 'livestock meal', 'horizonjucbe biobased', 'alternative sources', 'stepbiotech horizonjucbeia', 'biobased europe', 'biobased products', 'medical nutrition therapy diseases', 'agents drive', 'ecology', 'biodegradable polymers', 'feedstock biobased', 'ottoman period food beverage enterprises', 'biotech industry', 'estuaries rivers (wave', 'social influence', 'nutrition dietetics', 'composition', 'space maintenance', 'undertaking amino', 'multi-agent systems', 'sources circular', 'biotech startups', 'chemical engineering', 'biodefense', 'biodegradable materials', 'horizonjucbeia horizonjucbe', 'feed additives', 'nutritional proteins', 'bulk fine', 'materials bioprocessing', 'quality', 'food chemistry', 'planetary science', 'bioreactors', 'european integration', 'contract law', 'scalingup nutritional', 'biological systems', 'logistics optimization', 'astrophysics', 'biomaterials', 'circular biobased', 'robotic consulting', 'technology fashion products', 'pharmaceutical industry', 'local food', 'processing nutrition', 'electronics manufacturing', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'european union', 'using biological', 'biomedical', 'products manufactured', 'insect livestock', 'seasonal agricultural work', 'black hole physics', 'protein engineering', 'process biocatalysis', 'functional foods', 'industrial design', 'bioprocessing', 'research methods', 'amino acid', 'manufactured using', 'cognitive processes work', 'biotechnology', 'food waste', 'fermentation feed', 'technologies industrial', 'health biotechnology', 'food drink', 'bioengineering', 'materials science', 'biopolymer', 'machine automation', 'water resources engineering', 'astrobiology', 'additives food', 'product liability', 'industrial engineering', 'composite materials', 'bioengineering technologies', 'chemicals biobased', 'sports nutrition', 'metabolic engineering', 'nutritional supplements', 'self-driving cars', 'hydropower', 'europe joint', 'proteins alternative', 'alternative organizations', 'local cuisines turkey', 'materials biobased', 'nourishment poultry', 'european studies', 'biotech innovation', 'meal nourishment', 'alternative media', 'joint undertaking', 'bioengineering applications', 'dependency criteria', 'diet feedstuff', 'cognitive processes', 'feedstuff fishmeal', 'biofuels biobased', 'material based design', 'clinical nutrition', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'products products', 'novel materials', 'biocatalysis fermentation', 'processes relying', 'therapeutic proteins', 'plastics biofuels', 'hydrolysate insect', 'biobased materials', 'biobased bioderived', 'fine chemicals', 'drink processing', 'biobased plastics', 'fishmeal hydrolysate', 'protein biochemistry', 'poultry stepbiotech', 'mechanical engineering materials']</t>
         </is>
       </c>
     </row>
@@ -4050,7 +4050,7 @@
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>['production planning', 'clothe clothing', 'chemicals textiles', 'chemical engineering', 'yarn stepbiotech', 'sustainable fashion', 'material feedstock', 'dyes colours', 'dyeing fashion', 'fit', 'plants products', 'european union', 'europe joint', 'european studies', 'patient safety', 'quality', 'black hole physics', 'synthetic biology', 'biomolecular research', 'engineering', 'biodefense', 'nutritional biotechnology', 'bulk fine', 'products textile', 'electronics manufacturing', 'green technologies', 'astrophysics', 'colours fibres', 'fashion buying', 'biosecurity', 'technical textiles', 'marketing product brand management', 'biodegradable polymers', 'yarn', 'materials biobased', 'biobased products', 'medical biotechnology', 'biobased materials', 'biobased europe', 'textile history', 'biomaterials', 'production circular', 'synthetic dyes', 'textiles production', 'fibre yarn', 'conventional chemicals', 'clothing dyeing', 'robotic collaboration', 'fashion fiber', 'technology fashion products', 'bioinformatics', 'biotech innovation', 'products manufactured', 'solutions replace', 'bioenergy', 'food chemistry', 'circular biobased', 'knitting weaving technologies', 'mechanical engineering materials', 'biotech startups', 'mechanical engineering production', 'biopolymer', 'bioengineering', 'using biological', 'textiles including', 'plants textiles', 'rewriting', 'including synthetic', 'petroleum engineering', 'distribution agreements', 'biobased solutions', 'feedstock biobased', 'employee safety', 'biotechnology', 'joint undertaking', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'materials chemical', 'environmental engineering', 'biotechnology companies', 'products products', 'biochemistry', 'replace hazardous', 'biomedical', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'composite materials', '3d garment simulation', 'fiber fibre', 'plastics biofuels', 'novel materials', 'biotech industry', 'renewable materials', 'bioengineering solutions', 'logistics optimization', 'biobased plastics', 'pharmaceutical industry', 'robotic solutions', 'horizonjucbeia horizonjucbe', 'biological systems', 'toxicology', 'manufacturing systems', 'product liability', 'manufactured using', 'occupational health safety', 'technology', 'biodegradable materials', 'bioderived bulk', 'photopolymerization', 'textile art', 'biofuels biobased', 'hazardous conventional', 'fiber art', 'undertaking clothe', 'adaptation', 'engineering plants', 'textile plants', 'health biotechnology', 'stepbiotech horizonjucbeia', 'contract law', 'european integration', 'horizonjucbe biobased', 'fine chemicals', 'optical fibers', 'bioreactors', 'material based design', 'ssbd biobased']</t>
+          <t>['robotic collaboration', 'plants textiles', 'dyes colours', 'biological agents', 'medical biotechnology', 'marketing product brand management', 'production circular', 'biological material', 'bioinformatics', 'toxicology', 'nutritional biotechnology', 'rewriting', 'horizonjucbe biobased', 'stepbiotech horizonjucbeia', 'robotic solutions', 'undertaking clothe', 'yarn', 'biobased europe', 'biobased products', 'production planning', 'hazardous conventional', 'biodegradable polymers', 'colours fibres', 'feedstock biobased', 'biotech industry', 'textiles including', 'bioengineering solutions', 'textiles production', 'materials chemical', 'biotech startups', 'chemical engineering', 'biodefense', 'biodegradable materials', 'horizonjucbeia horizonjucbe', 'ssbd biobased', 'bulk fine', 'sustainable fashion', 'food chemistry', 'quality', 'bioreactors', 'european integration', 'contract law', 'dyeing fashion', 'biological systems', 'fashion buying', 'logistics optimization', 'products textile', 'biobased solutions', 'clothing dyeing', 'astrophysics', 'biomaterials', 'circular biobased', 'biosecurity', 'technology fashion products', 'pharmaceutical industry', 'plants products', 'electronics manufacturing', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'patient safety', 'european union', 'using biological', 'biotechnology companies', 'biomedical', 'products manufactured', 'employee safety', 'engineering', 'textile plants', 'black hole physics', 'yarn stepbiotech', 'photopolymerization', 'chemicals textiles', 'solutions replace', 'textile art', 'engineering plants', 'green technologies', '3d garment simulation', 'fashion fiber', 'manufactured using', 'biotechnology', 'environmental engineering', 'textile history', 'health biotechnology', 'bioengineering', 'materials science', 'biopolymer', 'occupational health safety', 'astrobiology', 'including synthetic', 'product liability', 'composite materials', 'fiber fibre', 'chemicals biobased', 'conventional chemicals', 'synthetic dyes', 'europe joint', 'replace hazardous', 'synthetic biology', 'materials biobased', 'european studies', 'biotech innovation', 'joint undertaking', 'fiber art', 'mechanical engineering production', 'biofuels biobased', 'material based design', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'optical fibers', 'products products', 'novel materials', 'knitting weaving technologies', 'petroleum engineering', 'plastics biofuels', 'clothe clothing', 'adaptation', 'biobased materials', 'biobased bioderived', 'technical textiles', 'renewable materials', 'fibre yarn', 'fine chemicals', 'biobased plastics', 'mechanical engineering materials']</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4087,7 @@
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>['production planning', 'biotechnology research', 'soil health', 'biobased biodegradable', 'chemical engineering', 'farmers fertilisation', 'material feedstock', 'soil biology', 'fit', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'biomolecular research', 'bioengineering applications', 'biodefense', 'nutritional biotechnology', 'products reduce', 'bulk fine', 'delivery systems', 'systems fertilising', 'biobased fertilisers', 'electronics manufacturing', 'plastics farmers', 'green technologies', 'marketing product brand management', 'biodegradable polymers', 'microplastics soil', 'related crop', 'materials biobased', 'biobased products', 'medical biotechnology', 'biology biobased', 'biobased materials', 'biobased europe', 'biomaterials', 'air pollution control', 'mechanical equipment', 'biotechnological applications', 'freight transportation', 'robotic collaboration', 'technology fashion products', 'biotech innovation', 'horizonjucbe agriculture', 'plasticity', 'delivery system', 'products manufactured', 'geology', 'health horizonjucberia', 'crop production', 'community health', 'bioenergy', 'system biodegradable', 'polymers biobased', 'circular biobased', 'biomedical research', 'public health', 'mechanical engineering materials', 'molecular biology', 'biopolymer', 'biotech startups', 'health circular', 'bioengineering', 'fertiliser application', 'fertilisation fertiliser', 'using biological', 'carbon reduction', 'drug delivery', 'applied macro', 'biology cultivation', 'production soil', 'distribution agreements', 'plant biology', 'feedstock biobased', 'materials fertilisation', 'promote soil', 'bioremediation', 'biotechnology', 'joint undertaking', 'undertaking agriculture', 'fertilisers biodegradable', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'controlled drug delivery systems', 'environmental economics', 'applied plant', 'global health', 'mobile applications', 'products products', 'biochemistry', 'biodegradable plastics', 'precision agriculture', 'biomedical', 'biological material', 'pollution promote', 'materials science', 'agriculture related', 'biological agents', 'biobased bioderived', '(integrative) system biology', 'biotechnology commercialization', 'biodegradable delivery', 'soil architecture', 'poor soil characterization', 'sustainable agriculture', 'health informatics', 'composite materials', 'concordat', 'software', 'seasonal agricultural work', 'plastics biofuels', 'novel materials', 'biotech industry', 'logistics optimization', 'fertilising products', 'biobased plastics', 'space debris', 'pharmaceutical industry', 'biological systems', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'toxicology', 'biodegradable materials', 'land reclamation', 'bioderived bulk', 'reduce microplastics', 'biofuels biobased', 'africa health', 'fertilisation microplastics', 'tissue engineering', 'cell biology', 'contract law', 'european integration', 'reproductive technologies', 'microplastics pollution', 'horizonjucberia horizonjucbe', 'agriculture biobased', 'fine chemicals', 'application equipment', 'cultivation applied', 'bioreactors', 'environmental policy', 'material based design']</t>
+          <t>['robotic collaboration', 'space debris', 'health horizonjucberia', 'health circular', 'horizonjucbe agriculture', 'marketing product brand management', 'medical biotechnology', 'biological agents', 'biological material', 'toxicology', 'nutritional biotechnology', 'application equipment', '(integrative) system biology', 'land reclamation', 'fertilisers biodegradable', 'cultivation applied', 'system biodegradable', 'biobased europe', 'fertilisation microplastics', 'agriculture related', 'biobased products', 'related crop', 'delivery systems', 'sustainable agriculture', 'plant biology', 'production planning', 'biodegradable polymers', 'biobased fertilisers', 'feedstock biobased', 'biotech industry', 'carbon reduction', 'geology', 'concordat', 'mobile applications', 'biotech startups', 'chemical engineering', 'production soil', 'plasticity', 'biodefense', 'biodegradable materials', 'microplastics soil', 'applied macro', 'bulk fine', 'polymers biobased', 'quality', 'bioreactors', 'european integration', 'biodegradable delivery', 'contract law', 'biological systems', 'logistics optimization', 'systems fertilising', 'promote soil', 'controlled drug delivery systems', 'horizonjucberia horizonjucbe', 'biomaterials', 'circular biobased', 'technology fashion products', 'pharmaceutical industry', 'electronics manufacturing', 'software', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'european union', 'using biological', 'biotechnological applications', 'biodegradable plastics', 'biomedical', 'products manufactured', 'seasonal agricultural work', 'black hole physics', 'biomedical research', 'products reduce', 'reproductive technologies', 'air pollution control', 'pollution promote', 'crop production', 'farmers fertilisation', 'green technologies', 'manufactured using', 'reduce microplastics', 'molecular biology', 'biotechnology', 'delivery system', 'freight transportation', 'health informatics', 'soil health', 'bioengineering', 'soil architecture', 'fertilisation fertiliser', 'materials science', 'biopolymer', 'fertiliser application', 'environmental economics', 'astrobiology', 'poor soil characterization', 'agriculture biobased', 'product liability', 'composite materials', 'chemicals biobased', 'biology cultivation', 'global health', 'europe joint', 'fertilising products', 'materials biobased', 'european studies', 'biotech innovation', 'public health', 'drug delivery', 'joint undertaking', 'bioengineering applications', 'microplastics pollution', 'biofuels biobased', 'cell biology', 'material based design', 'community health', 'bioderived bulk', 'fit', 'bioremediation', 'bioenergy', 'biochemistry', 'manufacturing systems', 'products products', 'novel materials', 'mechanical equipment', 'soil biology', 'plastics biofuels', 'biobased biodegradable', 'environmental policy', 'africa health', 'biobased materials', 'applied plant', 'biology biobased', 'undertaking agriculture', 'biobased bioderived', 'fine chemicals', 'biotechnology research', 'biobased plastics', 'tissue engineering', 'precision agriculture', 'mechanical engineering materials', 'plastics farmers', 'biotechnology commercialization', 'materials fertilisation']</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>['space maintenance', 'biotechnology research', 'chemical engineering', 'materials bioprocessing', 'material feedstock', 'microbiology', 'fit', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'biocatalysis fermentation', 'biomolecular research', 'bioengineering applications', 'machine automation', 'bioprocessing', 'biodefense', 'nutritional biotechnology', 'bulk fine', 'drive process', 'electronics manufacturing', 'multi-agent systems', 'astrophysics', 'horizonjucbe applied', 'marketing product brand management', 'biodegradable polymers', 'cognitive processes', 'materials biobased', 'biobased products', 'medical biotechnology', 'applied microbiology', 'microtechnology', 'biobased materials', 'biotech biobased', 'biobased europe', 'microbiology biobased', 'biomaterials', 'applied biotechnology', 'self-driving cars', 'biotechnological applications', 'microorganism stepbiotech', 'robust control', 'fermentation industrial', 'physical processes coasts', 'robotic collaboration', 'metabolic engineering', 'biomedical applications', 'technology fashion products', 'microorganism microorganism', 'biotech innovation', 'nonmedical bioreactors', 'products manufactured', 'bioenergy', 'processes circular', 'circular biobased', 'mechanical engineering materials', 'biotech startups', 'mechanical engineering processes', 'hydraulic engineering', 'biopolymer', 'bioengineering', 'using biological', 'applied macro', 'distribution agreements', 'continuous biotech', 'bioreactors applied', 'feedstock biobased', 'costeffective robust', 'undertaking bioreactor', 'biotechnology', 'joint undertaking', 'biobased processes', 'cae methodology development', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'robotic consulting', 'water purification', 'dependency criteria', 'biomedical sciences technologies', 'hydraulics', 'membrane microorganism', 'dynamic systems', 'industrial engineering', 'processes relying', 'products products', 'biochemistry', 'industrial processes', 'process biocatalysis', 'biomedical', 'biological material', 'materials science', 'biological agents', 'biobased bioderived', 'composite materials', 'relying biological', 'biocompability', 'plastics biofuels', 'novel materials', 'biotech industry', 'flow membrane', 'logistics optimization', 'industrial biotechnology', 'biobased plastics', 'pharmaceutical industry', 'horizonjucbeia horizonjucbe', 'industrial design', 'biological systems', 'bioreactor fermentation', 'bioprocessing technologies', 'manufacturing systems', 'technology', 'robotic safety', 'manufactured using', 'product liability', 'toxicology', 'biodegradable materials', 'bioderived bulk', 'agents drive', 'biofuels biobased', 'fermentation flow', 'bioengineering technologies', 'health biotechnology', 'biotechnology nonmedical', 'stepbiotech horizonjucbeia', 'technologies industrial', 'contract law', 'european integration', 'fine chemicals', 'sensitivity analysis', 'bioreactors', 'material based design', 'cognitive processes work', 'robust continuous']</t>
+          <t>['bioprocessing technologies', 'industrial processes', 'robotic collaboration', 'water purification', 'biocompability', 'biological agents', 'medical biotechnology', 'marketing product brand management', 'relying biological', 'biological material', 'drive process', 'toxicology', 'nutritional biotechnology', 'robust continuous', 'fermentation industrial', 'stepbiotech horizonjucbeia', 'robust control', 'microorganism stepbiotech', 'applied biotechnology', 'flow membrane', 'biobased europe', 'biobased products', 'bioreactor fermentation', 'agents drive', 'biodegradable polymers', 'feedstock biobased', 'biotech industry', 'biomedical applications', 'space maintenance', 'mechanical engineering processes', 'multi-agent systems', 'bioreactors applied', 'biotech startups', 'chemical engineering', 'microbiology biobased', 'biodefense', 'biodegradable materials', 'horizonjucbeia horizonjucbe', 'applied macro', 'applied microbiology', 'bulk fine', 'materials bioprocessing', 'undertaking bioreactor', 'biomedical sciences technologies', 'quality', 'bioreactors', 'european integration', 'biobased processes', 'contract law', 'biological systems', 'logistics optimization', 'microtechnology', 'astrophysics', 'biomaterials', 'circular biobased', 'robotic consulting', 'technology fashion products', 'nonmedical bioreactors', 'pharmaceutical industry', 'robotic safety', 'electronics manufacturing', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'european union', 'using biological', 'biotechnological applications', 'biomedical', 'products manufactured', 'black hole physics', 'process biocatalysis', 'sensitivity analysis', 'industrial design', 'bioprocessing', 'horizonjucbe applied', 'physical processes coasts', 'cae methodology development', 'manufactured using', 'cognitive processes work', 'biotechnology', 'industrial biotechnology', 'technologies industrial', 'health biotechnology', 'bioengineering', 'hydraulics', 'materials science', 'biopolymer', 'machine automation', 'astrobiology', 'costeffective robust', 'fermentation flow', 'product liability', 'microbiology', 'composite materials', 'bioengineering technologies', 'industrial engineering', 'chemicals biobased', 'continuous biotech', 'metabolic engineering', 'biotechnology nonmedical', 'self-driving cars', 'europe joint', 'european studies', 'materials biobased', 'biotech innovation', 'joint undertaking', 'bioengineering applications', 'dependency criteria', 'cognitive processes', 'biofuels biobased', 'hydraulic engineering', 'material based design', 'bioderived bulk', 'fit', 'bioenergy', 'biochemistry', 'manufacturing systems', 'products products', 'novel materials', 'biocatalysis fermentation', 'processes relying', 'plastics biofuels', 'biobased materials', 'microorganism microorganism', 'membrane microorganism', 'biotech biobased', 'processes circular', 'biobased bioderived', 'fine chemicals', 'biotechnology research', 'biobased plastics', 'dynamic systems', 'mechanical engineering materials']</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>['polymers plastics', 'new market', 'biopolymer biopolymer', 'labor market', 'chemical engineering', 'chemistry polymers', 'cellulose chitin', 'material feedstock', 'robotic applications', 'fit', 'european union', 'europe joint', 'european studies', 'quality', 'black hole physics', 'biomolecular research', 'biodefense', 'applications mathematical physics', 'nutritional biotechnology', 'biobased polymerscopolymers', 'mechanical engineering applications', 'bulk fine', 'geopolymers', 'electronics manufacturing', 'cell culture', 'enzymology', 'astrophysics', 'horizonjucbe applied', 'biosecurity', 'new media', 'technical textiles', 'biodegradable polymers', 'marketing product brand management', 'yarn', 'materials biobased', 'composites', 'biobased products', 'medical biotechnology', 'biobased materials', 'undertaking biopolymer', 'biobased europe', 'biomaterials', 'mechanical components', 'starch sugar', 'applied industrial', 'robotic collaboration', 'technology fashion products', 'biotech innovation', 'materials engineering', 'plasticity', 'products manufactured', 'bioenergy', 'food chemistry', 'circular biobased', 'industrial data', 'mechanical engineering materials', 'biotech startups', 'biopolymer', 'bioengineering', 'using biological', 'polymer chemistry', 'polymerscopolymers unlocking', 'applied macro', 'etc polymer', 'distribution agreements', 'feedstock biobased', 'polymer materials engineering behaviors civil engineering', 'biotechnology', 'joint undertaking', 'cae methodology development', 'chemicals biobased', 'astrobiology', 'bioderived novel', 'steel', 'market applications', 'change innovation.', 'industrial engineering', 'products products', 'biochemistry', 'biomaterials metals', 'market policies', 'biomedical', 'biological material', 'biopolymer cellulose', 'new ways working', 'materials science', 'industrial chemistry', 'biological agents', 'biobased bioderived', 'composite materials', 'plastics biofuels', 'novel materials', 'metals ceramics', 'biotech industry', 'chitin fiber', 'fiber starch', 'logistics optimization', 'biobased plastics', 'pharmaceutical industry', 'horizonjucbeia horizonjucbe', 'lactose intolerance', 'industrial design', 'chemistry biobased', 'biological systems', 'manufacturing systems', 'technology', 'product liability', 'manufactured using', 'toxicology', 'biodegradable materials', 'bioderived bulk', 'engineering biomaterials', 'digital marketing', 'photopolymerization', 'biofuels biobased', 'sugar stepbiotech', 'fiber art', 'applications circular', 'corporate marketing', 'materials materials', 'health biotechnology', 'ferroelectric materials', 'stepbiotech horizonjucbeia', 'composites etc', 'contract law', 'european integration', 'polymers composites', 'fine chemicals', 'pulp', 'optical fibers', 'ceramics polymers', 'bioreactors', 'material based design', 'ssbd biobased', 'unlocking new']</t>
+          <t>['robotic collaboration', 'digital marketing', 'applications circular', 'polymer chemistry', 'marketing product brand management', 'medical biotechnology', 'materials materials', 'biological agents', 'mechanical engineering applications', 'biological material', 'geopolymers', 'toxicology', 'nutritional biotechnology', 'change innovation.', 'starch sugar', 'chemistry polymers', 'unlocking new', 'stepbiotech horizonjucbeia', 'market applications', 'yarn', 'ceramics polymers', 'biobased europe', 'biobased products', 'metals ceramics', 'steel', 'industrial chemistry', 'undertaking biopolymer', 'biodegradable polymers', 'feedstock biobased', 'biotech industry', 'fiber starch', 'chemistry biobased', 'biotech startups', 'chemical engineering', 'plasticity', 'biodefense', 'biodegradable materials', 'horizonjucbeia horizonjucbe', 'applied macro', 'ssbd biobased', 'bulk fine', 'etc polymer', 'quality', 'food chemistry', 'bioreactors', 'european integration', 'contract law', 'biological systems', 'logistics optimization', 'polymers plastics', 'enzymology', 'astrophysics', 'biomaterials', 'circular biobased', 'biosecurity', 'technology fashion products', 'pulp', 'pharmaceutical industry', 'electronics manufacturing', 'material feedstock', 'biomolecular research', 'distribution agreements', 'technology', 'bioderived novel', 'european union', 'using biological', 'biomedical', 'products manufactured', 'cellulose chitin', 'black hole physics', 'market policies', 'industrial design', 'engineering biomaterials', 'applied industrial', 'photopolymerization', 'horizonjucbe applied', 'industrial data', 'cae methodology development', 'manufactured using', 'biotechnology', 'polymer materials engineering behaviors civil engineering', 'composites etc', 'health biotechnology', 'bioengineering', 'materials science', 'biopolymer biopolymer', 'biopolymer', 'astrobiology', 'labor market', 'corporate marketing', 'materials engineering', 'industrial engineering', 'product liability', 'composite materials', 'chemicals biobased', 'polymerscopolymers unlocking', 'new market', 'europe joint', 'european studies', 'materials biobased', 'chitin fiber', 'biotech innovation', 'new media', 'biomaterials metals', 'joint undertaking', 'robotic applications', 'fiber art', 'biofuels biobased', 'material based design', 'polymers composites', 'new ways working', 'bioderived bulk', 'cell culture', 'fit', 'ferroelectric materials', 'bioenergy', 'biochemistry', 'manufacturing systems', 'optical fibers', 'products products', 'novel materials', 'biobased polymerscopolymers', 'composites', 'plastics biofuels', 'biobased materials', 'applications mathematical physics', 'biobased bioderived', 'technical textiles', 'fine chemicals', 'biobased plastics', 'mechanical components', 'sugar stepbiotech', 'mechanical engineering materials', 'biopolymer cellulose', 'lactose intolerance']</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>['interest representation', 'development economics', 'hinfinity control', 'magnetic levitation', 'power supplies', 'development linear', 'planning design', 'biotechnology innovation', 'proposals configuration', 'european union', 'human development', 'robotic validation', 'maglevderived system', 'eu law', 'black hole physics', 'validation horizonerjufa', 'magnetic semiconductors', 'child development', 'electromagnetism', 'transport engineering', 'design management', 'sustainable technology', 'system design', 'technological development', 'power supply', 'motor maglev', 'architecture', 'call proposals', 'innovation power', 'design development', 'electronic testing', 'development maglevderived', 'mechanical equipment', 'design education', 'social media innovation', 'freight transportation', 'combustion engines', 'teleworking', 'maglev maglevderived', 'biotech innovation', 'transportation engineering', 'disruptive innovation', 'green consensus', 'system testing', 'design thinking', 'railway sustainable', 'horizonerjufa horizonjuer', 'history ottoman railways', 'system magnetic', 'eurail ju', 'testing validation', 'urban communication', 'sustainability', 'change innovation.', 'railguided system', 'linear motor', 'architectural design', 'electromechanical systems', 'magnetic mems', 'transmission lines', 'software design', 'ju call', 'mechatronics', 'concordat', 'transportation planning', 'automated testing', 'economic development', 'configuration design', 'highways railways infrastructure design construction', 'system dynamics', 'play', 'sustainable transport', 'growth development', 'robotic testing', 'technology', 'levitation railguided', 'maglevderived systems', 'power systems', 'space validation', 'aerospace structures', 'motor development', 'supply railway', 'vote', 'systems eurail', 'power electronics', 'horizonjuer disruptive']</t>
+          <t>['sustainable technology', 'development linear', 'sustainable transport', 'robotic validation', 'play', 'magnetic semiconductors', 'economic development', 'electronic testing', 'transportation planning', 'horizonerjufa horizonjuer', 'development economics', 'change innovation.', 'systems eurail', 'child development', 'history ottoman railways', 'urban communication', 'automated testing', 'electromechanical systems', 'development maglevderived', 'horizonjuer disruptive', 'testing validation', 'robotic testing', 'mechatronics', 'concordat', 'design development', 'eu law', 'combustion engines', 'magnetic mems', 'interest representation', 'magnetic levitation', 'ju call', 'design thinking', 'disruptive innovation', 'design education', 'transmission lines', 'hinfinity control', 'power supplies', 'railguided system', 'technological development', 'architecture', 'growth development', 'biotechnology innovation', 'space validation', 'levitation railguided', 'technology', 'system design', 'european union', 'system dynamics', 'power systems', 'black hole physics', 'maglevderived systems', 'sustainability', 'vote', 'motor maglev', 'configuration design', 'linear motor', 'innovation power', 'freight transportation', 'social media innovation', 'human development', 'system testing', 'maglev maglevderived', 'proposals configuration', 'green consensus', 'eurail ju', 'motor development', 'design management', 'biotech innovation', 'maglevderived system', 'software design', 'power electronics', 'aerospace structures', 'supply railway', 'railway sustainable', 'power supply', 'highways railways infrastructure design construction', 'mechanical equipment', 'electromagnetism', 'teleworking', 'transportation engineering', 'validation horizonerjufa', 'transport engineering', 'system magnetic', 'call proposals', 'planning design', 'architectural design']</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>['braincomputer interface', 'manufacturing systems', 'ai ai', 'thermofluids', 'hpcai tpc', 'therapeutic proteins', 'collaboration hpc', 'memory', 'factories hpcai', 'international relations', 'intelligence high', 'hpcai eurohpc', 'international collaboration', 'european union', 'performance studies', 'robotic support', 'space collaboration', 'ai factories', 'intelligence decision', 'robotic collaboration', 'VLSI design', 'black hole physics', 'artifical intelligence', 'mechanical engineering support', 'computing international', 'performance based design', 'decision theory', 'high performance', 'cyber intelligence', 'consortium horizonjueurohpcinco', 'variable structure control', 'international organizations', 'performance computing', 'eurohpc international', 'collaboration ai', 'hpc hpcai', 'parameter consortium', 'blockchain', 'parametric modeling', 'tpc trillion', 'horizonjueurohpcinco horizonjueurohpcinco', 'cooperation ai', 'trillion parameter', 'artificial intelligence', 'industrial data', 'cad/cam technologies', 'factories collaboration', 'european education area', 'performance', 'system on chip', 'biopolymer', 'international cooperation', 'computer aided drug design', 'global collaboration', 'internationalization', 'decision support', 'mentalization', 'computer graphics', 'international development', 'inflation', 'values', 'decision analysis', 'support artificial', 'optimization algorithms', 'data-driven decision making', 'horizonjueurohpcinco artificial', 'robotic solutions', 'industrial design']</t>
+          <t>['eurohpc international', 'computing international', 'international relations', 'robotic collaboration', 'black hole physics', 'performance computing', 'blockchain', 'industrial design', 'cad/cam technologies', 'high performance', 'collaboration ai', 'memory', 'computer aided drug design', 'industrial data', 'decision theory', 'trillion parameter', 'data-driven decision making', 'global collaboration', 'tpc trillion', 'artifical intelligence', 'performance', 'factories hpcai', 'international organizations', 'collaboration hpc', 'thermofluids', 'consortium horizonjueurohpcinco', 'hpcai eurohpc', 'robotic solutions', 'manufacturing systems', 'parameter consortium', 'decision analysis', 'horizonjueurohpcinco artificial', 'artificial intelligence', 'mechanical engineering support', 'mentalization', 'international development', 'therapeutic proteins', 'hpc hpcai', 'decision support', 'variable structure control', 'horizonjueurohpcinco horizonjueurohpcinco', 'optimization algorithms', 'performance based design', 'intelligence high', 'biopolymer', 'hpcai tpc', 'system on chip', 'robotic support', 'computer graphics', 'ai factories', 'space collaboration', 'international collaboration', 'inflation', 'ai ai', 'braincomputer interface', 'cyber intelligence', 'international cooperation', 'parametric modeling', 'intelligence decision', 'factories collaboration', 'values', 'european education area', 'european union', 'performance studies', 'internationalization', 'VLSI design', 'support artificial', 'cooperation ai']</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>['interest representation', 'excellence centres', 'growth development', 'ai excellence', 'trust service provider', 'radicalisation', 'robotic innovation', 'expanding european', 'quality management system', 'green finance', 'mechanical equipment', 'biotechnology innovation', 'octis enfield', 'lighthouse ria', 'innovation schemes', 'european network', 'proposals octis', 'network ai', 'green ai', 'city', 'urban communication', 'modernism', 'aesthetics place', 'architectural geometry.', 'ai lighthouse', 'european union', 'mechanical', 'european studies', 'management organization', 'change innovation.', 'second call', 'teleworking', 'centres expanding', 'aerospace engineering', 'biotech innovation', 'cyber intelligence', 'enfield european', 'growth', 'european ai', 'european integration', 'heritage tourism', 'deviance', 'european lighthouse', 'europeanization', 'green consensus', 'ai innovation', 'artificial intelligence', 'accreditation', 'film', 'trust law', 'artificial intelligence research', 'ria innovation', 'european education area', 'trust services', 'architecture', 'lighthouse manifest', 'coastal structures', 'green technologies', 'manifest trustworthy', 'evaluation', 'schemes second', 'architectural geometry computing', 'call proposals', 'trustworthy green']</t>
+          <t>['biotech innovation', 'trust service provider', 'evaluation', 'network ai', 'european network', 'robotic innovation', 'trust services', 'trust law', 'deviance', 'green ai', 'green technologies', 'european ai', 'film', 'second call', 'interest representation', 'europeanization', 'expanding european', 'ai lighthouse', 'change innovation.', 'trustworthy green', 'european integration', 'city', 'artificial intelligence', 'mechanical equipment', 'artificial intelligence research', 'accreditation', 'innovation schemes', 'urban communication', 'quality management system', 'aerospace engineering', 'ai excellence', 'heritage tourism', 'lighthouse ria', 'schemes second', 'teleworking', 'enfield european', 'radicalisation', 'architecture', 'centres expanding', 'growth', 'lighthouse manifest', 'growth development', 'aesthetics place', 'cyber intelligence', 'coastal structures', 'biotechnology innovation', 'architectural geometry computing', 'modernism', 'octis enfield', 'ai innovation', 'excellence centres', 'management organization', 'green consensus', 'call proposals', 'manifest trustworthy', 'european education area', 'european union', 'architectural geometry.', 'ria innovation', 'green finance', 'european studies', 'proposals octis', 'european lighthouse', 'mechanical']</t>
         </is>
       </c>
     </row>
@@ -4309,7 +4309,7 @@
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>['tide', 'performance arts', 'contribution creative', 'water arts', 'deep ecology', 'space services', 'landscapes art', 'ocean energy', 'transforming inspiring', 'inspiring aquatic', 'law sea', 'arts transforming', 'arts contribution', 'urban communication', 'ecology', 'mission ocean', 'ocean waters', 'revolutionary changes world', 'mediterranean sea', 'telemedicine', 'waters mediterranean', 'performing arts', 'adaptation', 'lighthouse call', 'teleworking', 'ocean water', 'creative sectors', 'traditional mediterranean architecture', 'sectors mission', 'seas', 'creativity', 'creative industry', 'aquatic landscapes', 'art culture', 'call tidal', 'creative labor', 'space exploration', 'cultural industries creative economy', 'oceanography', 'coastal structures', 'art sustainability', 'art sciences', 'cultural landscapes', 'visual arts', 'tidal arts', 'sea lighthouse']</t>
+          <t>['space exploration', 'water arts', 'call tidal', 'revolutionary changes world', 'lighthouse call', 'seas', 'cultural landscapes', 'arts transforming', 'ocean energy', 'oceanography', 'inspiring aquatic', 'cultural industries creative economy', 'law sea', 'telemedicine', 'transforming inspiring', 'mediterranean sea', 'ocean water', 'visual arts', 'art sustainability', 'urban communication', 'traditional mediterranean architecture', 'contribution creative', 'landscapes art', 'waters mediterranean', 'art sciences', 'adaptation', 'mission ocean', 'ocean waters', 'teleworking', 'deep ecology', 'aquatic landscapes', 'coastal structures', 'performance arts', 'art culture', 'ecology', 'tide', 'tidal arts', 'performing arts', 'creative industry', 'space services', 'creativity', 'arts contribution', 'creative sectors', 'sea lighthouse', 'creative labor', 'sectors mission']</t>
         </is>
       </c>
     </row>
@@ -4346,7 +4346,7 @@
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>['tide', 'performance arts', 'estuaries rivers (wave', 'contribution creative', 'water arts', 'deep ecology', 'space services', 'landscapes art', 'ocean energy', 'transforming inspiring', 'inspiring aquatic', 'law sea', 'arts transforming', 'arts contribution', 'urban communication', 'baltic north', 'ecology', 'mission ocean', 'ocean waters', 'revolutionary changes world', 'telemedicine', 'performing arts', 'north sea', 'lighthouse call', 'adaptation', 'teleworking', 'ocean water', 'creative sectors', 'waters baltic', 'sectors mission', 'seas', 'creativity', 'creative industry', 'russia', 'aquatic landscapes', 'art culture', 'call tidal', 'creative labor', 'space exploration', 'balkans', 'cultural industries creative economy', 'oceanography', 'coastal structures', 'art sustainability', 'art sciences', 'cultural landscapes', 'visual arts', 'tidal arts', 'sea lighthouse']</t>
+          <t>['space exploration', 'water arts', 'call tidal', 'revolutionary changes world', 'lighthouse call', 'seas', 'baltic north', 'cultural landscapes', 'arts transforming', 'ocean energy', 'north sea', 'oceanography', 'inspiring aquatic', 'cultural industries creative economy', 'law sea', 'telemedicine', 'transforming inspiring', 'ocean water', 'visual arts', 'art sustainability', 'urban communication', 'balkans', 'contribution creative', 'landscapes art', 'art sciences', 'adaptation', 'mission ocean', 'ocean waters', 'teleworking', 'deep ecology', 'waters baltic', 'aquatic landscapes', 'coastal structures', 'performance arts', 'art culture', 'ecology', 'tide', 'tidal arts', 'performing arts', 'creative industry', 'estuaries rivers (wave', 'space services', 'russia', 'creativity', 'arts contribution', 'creative sectors', 'sea lighthouse', 'creative labor', 'sectors mission']</t>
         </is>
       </c>
     </row>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>['blue sustainability', 'literacy school', 'educational psychology', 'estuaries rivers (wave', 'higher education', 'student school', 'environmental sustainability', 'ecosystem services', 'community development', 'media literacy', 'right education', 'ocean energy', 'agents change', 'ecology', 'sustainability', 'physical activity motivation', 'physical activity', 'shore empower', 'protection human rights sea', 'maritime security', 'ecosystem', 'irregular maritime migration', 'change innovation.', 'empower students', 'child studies', 'ocean water', 'promotion education', 'activities promotion', 'marine ecosystem', 'educational technologies', 'protection marine', 'seas', 'youth studies', 'water resources engineering', 'education policy', 'school communities', 'rewarding', 'sailing towards', 'marine freshwater', 'community studies', 'biological agents', 'ecosystems sailing', 'hydropower', 'school activities', 'freshwater ecosystems', 'towards ocean', 'marine law', 'sustainability protection', 'school books', 'oceanography', 'preschool education', 'coastal structures', 'education blue', 'sociology of education', 'multi-agent systems', 'robotic education', 'students agents', 'communities shore', 'maritime delimitation', 'water literacy', 'education']</t>
+          <t>['school communities', 'sociology of education', 'sustainability', 'educational technologies', 'seas', 'marine ecosystem', 'biological agents', 'literacy school', 'agents change', 'higher education', 'activities promotion', 'rewarding', 'robotic education', 'right education', 'ocean energy', 'environmental sustainability', 'oceanography', 'ecosystems sailing', 'educational psychology', 'change innovation.', 'promotion education', 'ocean water', 'marine law', 'sailing towards', 'physical activity', 'communities shore', 'community studies', 'community development', 'physical activity motivation', 'protection marine', 'maritime security', 'water literacy', 'school activities', 'protection human rights sea', 'water resources engineering', 'multi-agent systems', 'student school', 'education blue', 'towards ocean', 'students agents', 'coastal structures', 'empower students', 'education', 'ecology', 'preschool education', 'blue sustainability', 'school books', 'sustainability protection', 'ecosystem', 'irregular maritime migration', 'marine freshwater', 'child studies', 'estuaries rivers (wave', 'hydropower', 'freshwater ecosystems', 'shore empower', 'maritime delimitation', 'education policy', 'media literacy', 'ecosystem services', 'youth studies']</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="G108" t="inlineStr">
         <is>
-          <t>['social capital', 'hinfinity control', 'open eic', 'technology business', 'market commercial', 'horizoneictransitionopen deep', 'deep ecology', 'technology', 'labor market', 'electronic commerce', 'critical mapping', 'biotechnology innovation', 'eic technology', 'healthcare technology', 'transition horizoneictransitionopen', 'business market', 'service marketing', 'open data', 'cosmology', 'patient satisfaction', 'capital markets law', 'patient capital', 'patient safety', 'change innovation.', 'black hole physics', 'robotic technology', 'information technology', 'corporate marketing', 'transition open', 'open banking', 'animation', 'innovation technology', 'electronic devices', 'research innovation', 'horizoneictransitionopen horizoneictransitionopen', 'technology eic', 'deep tech', 'space exploration', 'capital research', 'eic transition', 'electronic signature', 'technology society', 'research performance', 'deep neural network', 'advertising', 'tech patient', 'deep learning']</t>
+          <t>['patient capital', 'horizoneictransitionopen horizoneictransitionopen', 'space exploration', 'technology eic', 'transition horizoneictransitionopen', 'business market', 'research performance', 'capital markets law', 'critical mapping', 'deep neural network', 'tech patient', 'horizoneictransitionopen deep', 'deep tech', 'technology business', 'animation', 'cosmology', 'social capital', 'electronic devices', 'open eic', 'change innovation.', 'technology society', 'patient satisfaction', 'robotic technology', 'electronic commerce', 'transition open', 'service marketing', 'hinfinity control', 'capital research', 'deep ecology', 'innovation technology', 'deep learning', 'labor market', 'eic technology', 'corporate marketing', 'biotechnology innovation', 'advertising', 'healthcare technology', 'electronic signature', 'research innovation', 'market commercial', 'open data', 'technology', 'eic transition', 'patient safety', 'open banking', 'information technology', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -4457,7 +4457,7 @@
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>['short film', 'production planning', 'nonwood products', 'small medium enterprises', 'nd smurf', 'penology', 'ecosystem services', 'manufacturing systems', 'deep ecology', 'environmental sustainability', 'community development', 'call small', 'land reclamation', 'global value chains', 'property law', 'small forests', 'ecology', 'sustainability', 'moral values', 'forestbased value', 'organisations sustainable', 'chains small', 'sustainable production', 'fit', 'steel', 'open data', 'ecosystem', 'open call', 'software development', 'management organization', 'decision tree', 'forest owners', 'properties development', 'teleworking', 'organisation theory', 'alternative organizations', 'technology fashion products', 'mechanical properties', 'management models', 'growth', 'optimising sustainable', 'development new', 'sustainable management', 'open banking', 'blockchain', 'new ways working', 'production wood', 'products small', 'owners organisations', 'model evaluation', 'forest properties', 'sustainable technology', 'chains nd', 'new forestbased', 'sustainable energy', 'mechanical engineering production', 'pulp', 'biopolymer', 'models theory', 'wood nonwood', 'small forest', 'smurf open', 'values', 'convergans clubs', 'value chains', 'models value', 'form', 'business model studies']</t>
+          <t>['sustainable technology', 'penology', 'blockchain', 'business model studies', 'sustainability', 'development new', 'mechanical properties', 'nd smurf', 'property law', 'forest properties', 'owners organisations', 'environmental sustainability', 'small forest', 'mechanical engineering production', 'organisations sustainable', 'small medium enterprises', 'new ways working', 'open call', 'fit', 'models theory', 'manufacturing systems', 'land reclamation', 'community development', 'form', 'smurf open', 'chains nd', 'properties development', 'call small', 'short film', 'value chains', 'biopolymer', 'teleworking', 'global value chains', 'production wood', 'sustainable management', 'deep ecology', 'new forestbased', 'technology fashion products', 'steel', 'growth', 'chains small', 'forestbased value', 'wood nonwood', 'production planning', 'forest owners', 'pulp', 'ecology', 'sustainable energy', 'moral values', 'nonwood products', 'organisation theory', 'software development', 'sustainable production', 'ecosystem', 'optimising sustainable', 'products small', 'values', 'open data', 'management organization', 'model evaluation', 'management models', 'small forests', 'decision tree', 'models value', 'open banking', 'alternative organizations', 'convergans clubs', 'ecosystem services']</t>
         </is>
       </c>
     </row>
@@ -4494,7 +4494,7 @@
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>['solutions streamline', 'media studies', 'thermal engineering', 'attachment', 'renewable energy', 'space integration', 'mobilization', 'transgenic organisms', 'space solutions', 'local food', 'thermofluids', 'inclusion', 'political activism', 'positive energy', 'renewable energy systems', 'solutions positive', 'energy storage', 'interoperable solutions', 'local excess', 'molecular evolution', 'positive clinical psychology', 'documentary', 'open data', 'thermal engineering systems', 'open call', 'energy', 'performance studies', 'computational heat transfer', 'local renewables', 'child studies', 'quality', 'call demonstrators', 'd esign education', 'teleworking', 'renewables local', 'heat sources', 'ped evolution', 'supporters', 'medical devices', 'energy districts', 'hydraulics', 'better integration', 'education urban space / traffic)', 'crosssectoral integration', 'integration local', 'evolution crosssectoral', 'open banking', 'mechanical engineering integration', 'piping systems', 'genetic engineering', 'including better', 'peds including', 'computer aided engineering', 'electronic payment services', 'pedvolution open', 'dark energy', 'performance', 'streamline ped', 'hydraulic engineering', 'evolutionary computing', 'public administration', 'photovoltaics', 'sources pedvolution', 'activist public relations', 'renewable materials', 'multi-agent systems', 'over urbanization', 'districts peds', 'bioengineering solutions', 'peds interoperable', 'excess heat', 'energy policy', 'robotic solutions', 'demonstrators positive', 'education']</t>
+          <t>['renewables local', 'solutions streamline', 'sources pedvolution', 'supporters', 'computer aided engineering', 'activist public relations', 'electronic payment services', 'thermal engineering systems', 'attachment', 'over urbanization', 'thermal engineering', 'photovoltaics', 'interoperable solutions', 'genetic engineering', 'including better', 'peds including', 'local renewables', 'medical devices', 'political activism', 'hydraulic engineering', 'evolution crosssectoral', 'performance', 'molecular evolution', 'thermofluids', 'd esign education', 'excess heat', 'quality', 'open call', 'space integration', 'renewable energy', 'inclusion', 'energy policy', 'robotic solutions', 'piping systems', 'renewable energy systems', 'dark energy', 'space solutions', 'better integration', 'solutions positive', 'mobilization', 'evolutionary computing', 'hydraulics', 'teleworking', 'districts peds', 'pedvolution open', 'peds interoperable', 'documentary', 'call demonstrators', 'media studies', 'integration local', 'mechanical engineering integration', 'energy districts', 'local excess', 'education', 'transgenic organisms', 'crosssectoral integration', 'renewable materials', 'education urban space / traffic)', 'local food', 'heat sources', 'ped evolution', 'computational heat transfer', 'child studies', 'public administration', 'positive clinical psychology', 'open data', 'energy storage', 'bioengineering solutions', 'performance studies', 'positive energy', 'open banking', 'multi-agent systems', 'demonstrators positive', 'energy', 'streamline ped']</t>
         </is>
       </c>
     </row>
@@ -4531,7 +4531,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>['programme mvp', 'strategic communication', 'presentation', 'global studies', 'startups automotive', 'disadvantaged groups', 'crosscultural management', 'entrepreneurship', 'automotive fintech', 'fintech crosskic', 'd esign education', 'mvp startups', 'eit crosskic', 'mechanical engineering automation', 'sports marketing', 'qualitative research', 'competitive strategies', 'community studies', 'strategic outreach', 'globalization', 'd esign management', 'software design', 'strategic management', 'concordat', 'biotech startups', 'software', 'industrial automation', 'banking', 'global collaboration', 'crosskic strategic', 'biotech industry', 'mechanical engineering', 'crosskic global', 'mechanical engineering technology', 'outreach qscale', 'quantum computing', 'strategy', 'qscale programme', 'mechanical engineering manufacturing', 'global outreach']</t>
+          <t>['crosskic global', 'strategic management', 'mechanical engineering manufacturing', 'software design', 'qscale programme', 'strategic communication', 'biotech startups', 'crosscultural management', 'crosskic strategic', 'programme mvp', 'mechanical engineering technology', 'quantum computing', 'global collaboration', 'd esign education', 'mechanical engineering', 'd esign management', 'community studies', 'globalization', 'strategy', 'disadvantaged groups', 'qualitative research', 'mechanical engineering automation', 'sports marketing', 'presentation', 'global studies', 'global outreach', 'entrepreneurship', 'eit crosskic', 'outreach qscale', 'automotive fintech', 'competitive strategies', 'strategic outreach', 'software', 'fintech crosskic', 'banking', 'biotech industry', 'industrial automation', 'concordat', 'mvp startups', 'startups automotive']</t>
         </is>
       </c>
     </row>
@@ -4568,7 +4568,7 @@
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>['play', 'composites', 'aircraft systems', 'internet governance', 'ia ngi', 'f fediversity', 'africa', 'digital humanities', 'digital culture', 'generation internet', 'african education', 'internet things', 'aviation', 'children', 'open data', 'open call', 'internet of things', 'teleworking', 'd esign education', 'digital media children', 'pilots next', 'open banking', 'fediversity open', 'vote', 'social media', 'lgbti', 'internet ia', 'nursing education', 'call f', 'ngi fediversity', 'educational buildings', 'aviation management', 'demographic change', 'next generation', 'ngo']</t>
+          <t>['play', 'fediversity open', 'africa', 'vote', 'ngi fediversity', 'f fediversity', 'aircraft systems', 'aviation', 'd esign education', 'open call', 'social media', 'internet things', 'pilots next', 'demographic change', 'composites', 'african education', 'internet ia', 'teleworking', 'digital culture', 'nursing education', 'ia ngi', 'call f', 'lgbti', 'generation internet', 'digital humanities', 'next generation', 'aviation management', 'internet of things', 'open data', 'educational buildings', 'open banking', 'internet governance', 'digital media children', 'ngo', 'children']</t>
         </is>
       </c>
     </row>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="G113" t="inlineStr">
         <is>
-          <t>['ria ngi', 'fund z', 'digital craft', 'growth development', 'zero emission', 'internet governance', 'digital culture', 'internet commons', 'fund ria', 'zero commons', 'green finance', 'spina bifida', 'zero emissions', 'generation internet', 'grow internet', 'ngi zero', 'children', 'aging', 'z create', 'commons fund', 'internet of things', 'digital media children', 'mature grow', 'growth', 'internet fund', 'international finance', 'coalition politics', 'lgbti', 'social media', 'electronic payment services', 'crowdfunding', 'developmental needs', 'macro', 'create mature', 'form', 'demographic change', 'next generation', 'ngo']</t>
+          <t>['electronic payment services', 'zero commons', 'developmental needs', 'macro', 'ngi zero', 'crowdfunding', 'zero emission', 'z create', 'social media', 'fund ria', 'form', 'fund z', 'spina bifida', 'zero emissions', 'mature grow', 'internet fund', 'commons fund', 'demographic change', 'aging', 'digital culture', 'international finance', 'growth development', 'growth', 'lgbti', 'generation internet', 'ria ngi', 'digital craft', 'next generation', 'grow internet', 'internet of things', 'coalition politics', 'create mature', 'internet commons', 'green finance', 'internet governance', 'digital media children', 'ngo', 'children']</t>
         </is>
       </c>
     </row>
@@ -4642,7 +4642,7 @@
       </c>
       <c r="G114" t="inlineStr">
         <is>
-          <t>['eu missions', 'hinfinity control', 'medical research', 'civil society', 'television studies', 'researchers night', 'urban society', 'civil servants legislation.', 'horizonmscacitizens horizonmscacitizens', 'higher education', 'ecosystem services', 'space research', 'sustainable eco', 'urban ecology', 'global studies', 'climate change', 'citizenship', 'society climate', 'universitycivil society relations', 'sustainability', 'climate', 'eco ecosystem', 'schools msca', 'ecosystem', 'european union', 'horizonmscacitizens sustainable', 'european studies', 'researchers schools', 'child studies', 'msca citizens', 'space collaboration', 'black hole physics', 'urban design', 'eu law', 'society', 'night researchers', 'youth studies', 'european integration', 'ecosystem urban', 'community studies', 'citizens horizonmscacitizens', 'european researchers', 'research academia', 'biomedical research', 'change eu', 'missions research', 'dark energy', 'sustainable energy', 'sustainable cities', 'research performance', 'astrophysics', 'artificial ecosystems', 'audience research', 'sustainable consumption', 'education']</t>
+          <t>['society', 'european researchers', 'biomedical research', 'black hole physics', 'sustainability', 'researchers night', 'change eu', 'research performance', 'night researchers', 'horizonmscacitizens horizonmscacitizens', 'urban society', 'higher education', 'eu law', 'schools msca', 'researchers schools', 'universitycivil society relations', 'urban ecology', 'horizonmscacitizens sustainable', 'citizens horizonmscacitizens', 'european integration', 'community studies', 'civil servants legislation.', 'climate', 'dark energy', 'sustainable cities', 'sustainable consumption', 'urban design', 'hinfinity control', 'research academia', 'television studies', 'msca citizens', 'citizenship', 'artificial ecosystems', 'sustainable eco', 'astrophysics', 'global studies', 'eu missions', 'space collaboration', 'society climate', 'education', 'civil society', 'sustainable energy', 'climate change', 'eco ecosystem', 'ecosystem urban', 'ecosystem', 'child studies', 'european union', 'medical research', 'missions research', 'audience research', 'space research', 'european studies', 'ecosystem services', 'youth studies']</t>
         </is>
       </c>
     </row>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>['hydrogen microplastics', 'mechanical devices', 'production planning', 'biology synthetic', 'carbon footprint', 'recycling renewable', 'challenges challenges', 'critical mapping', 'anthropology', 'chemical engineering', 'utilization climate', 'desalination brines', 'climate adaptation', 'microbiology', 'chemicals hydrogen', 'critical raw', 'food waste', 'challenges pathfinderchallenges', 'synthetic biology', 'pathfinder challenges', 'alternative dispute resolution', 'plastic waste', 'conflict resolution', 'polymers waste', 'competitive strategies', 'electromagnetism', 'computational design', 'water wastetovalue', 'circular production', 'optoelectronic devices', 'production renewable', 'nonbiologic origin', 'aviation management', 'optimization algorithms', 'algorithm optimization', 'biodegradable polymers', 'economy', 'composites', 'medical biotechnology', 'solar energy', 'renewable energy', 'fuels synthetic', 'biomaterials', 'devices horizoneicpathfinderchallenges', 'aviation fuels', 'critical thinking', 'electrical engineering', 'aviation', 'fuels nonbiologic', 'computational material', 'combustion engines', 'metabolic engineering', 'plasticity', 'pathfinderchallenges bioremediation', 'geology', 'electrochemistry fossilfree', 'bioenergy', 'food chemistry', 'electronic devices', 'hydropower', 'waste management', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'mechanical engineering materials', 'biopolymer', 'mechanical engineering production', 'bioengineering', 'optoelectronics', 'photovoltaics', 'pathfinder pathfinder', 'carbon reduction', 'materials desalination', 'microplastics photocatalysis', 'material science', 'learning difficulties', 'waste water', 'petroleum engineering', 'robotics', 'computational theory', 'challenges circular', 'bioremediation', 'polymer materials engineering behaviors civil engineering', 'biotechnology', 'devices circular', 'raw materials', 'renewable energy systems', 'climate change', 'sustainability', 'astrobiology', 'water purification', 'solar solar', 'renewable fuels', 'brines electricity', 'biosimilars', 'fossilfree chemicals', 'fuels renewable', 'change innovation.', 'medical devices', 'biochemistry', 'water resources engineering', 'metaheuristic approaches', 'materials science', 'capture utilization', 'composite materials', 'renewable materials', 'photocatalysis plastic', 'waste valorization', 'origin solar', 'sustainable aviation', 'strategy', 'recycling technologies', 'carbon tax', 'bioremediation bottomup', 'eic pathfinder', 'solar reforming', 'data acquisition', 'manufacturing systems', 'bottomup synthetic', 'toxicology', 'critical theory', 'biodegradable materials', 'synthetic polymers', 'sustainable development', 'valorization waste', 'photopolymerization', 'change mitigation', 'metaheuristic algorithms', 'climate', 'chemicals materials', 'renewable energy engineering', 'carbon capture', 'science critical', 'electricity electrochemistry', 'energy renewable', 'wastetovalue devices', 'materials eic', 'algorithm design', 'space coordination', 'fuels chemicals', 'economy pathfinder', 'biology carbon', 'environmental science', 'material design behavior', 'mitigation computational', 'circular economy', 'computational physics', 'space exploration', 'computational studies', 'reforming sustainable', 'hydrogen energy', 'waste recycling', 'economics', 'material based design', 'sharing economy']</t>
+          <t>['conflict resolution', 'water purification', 'chemicals materials', 'capture utilization', 'waste management', 'medical biotechnology', 'electrical engineering', 'chemicals hydrogen', 'medical devices', 'renewable fuels', 'renewable energy engineering', 'toxicology', 'aviation', 'change innovation.', 'reforming sustainable', 'synthetic polymers', 'computational design', 'fuels chemicals', 'photocatalysis plastic', 'sharing economy', 'material design behavior', 'recycling renewable', 'computational physics', 'brines electricity', 'learning difficulties', 'economy', 'circular economy', 'robotics', 'devices circular', 'carbon capture', 'carbon tax', 'solar reforming', 'production planning', 'biodegradable polymers', 'alternative dispute resolution', 'metaheuristic approaches', 'carbon reduction', 'geology', 'biology carbon', 'biosimilars', 'solar energy', 'aviation fuels', 'polymers waste', 'water wastetovalue', 'waste valorization', 'origin solar', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'chemical engineering', 'plasticity', 'recycling technologies', 'climate adaptation', 'biodegradable materials', 'combustion engines', 'electronic devices', 'food chemistry', 'renewable energy', 'microplastics photocatalysis', 'renewable energy systems', 'sustainable development', 'climate', 'bottomup synthetic', 'fuels synthetic', 'eic pathfinder', 'computational studies', 'energy renewable', 'economy pathfinder', 'biomaterials', 'optoelectronic devices', 'algorithm design', 'climate change', 'challenges pathfinderchallenges', 'competitive strategies', 'fossilfree chemicals', 'nonbiologic origin', 'raw materials', 'mechanical devices', 'devices horizoneicpathfinderchallenges', 'mitigation computational', 'electrochemistry fossilfree', 'optoelectronics', 'computational material', 'economics', 'challenges circular', 'sustainability', 'space coordination', 'photovoltaics', 'photopolymerization', 'hydrogen energy', 'data acquisition', 'challenges challenges', 'anthropology', 'algorithm optimization', 'science critical', 'plastic waste', 'biology synthetic', 'biotechnology', 'polymer materials engineering behaviors civil engineering', 'change mitigation', 'food waste', 'sustainable aviation', 'strategy', 'bioengineering', 'materials science', 'desalination brines', 'biopolymer', 'pathfinderchallenges bioremediation', 'carbon footprint', 'water resources engineering', 'astrobiology', 'waste water', 'critical theory', 'materials eic', 'composite materials', 'microbiology', 'aviation management', 'metabolic engineering', 'hydropower', 'synthetic biology', 'pathfinder pathfinder', 'metaheuristic algorithms', 'space exploration', 'critical raw', 'circular production', 'materials desalination', 'critical mapping', 'electricity electrochemistry', 'fuels renewable', 'utilization climate', 'mechanical engineering production', 'material based design', 'hydrogen microplastics', 'bioremediation', 'bioenergy', 'biochemistry', 'manufacturing systems', 'petroleum engineering', 'electromagnetism', 'composites', 'fuels nonbiologic', 'optimization algorithms', 'production renewable', 'computational theory', 'solar solar', 'renewable materials', 'material science', 'waste recycling', 'pathfinder challenges', 'wastetovalue devices', 'valorization waste', 'bioremediation bottomup', 'mechanical engineering materials', 'critical thinking', 'environmental science']</t>
         </is>
       </c>
     </row>
@@ -4716,7 +4716,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>['space infrastructure', 'mechanical devices', 'field robotics', 'architectural geometry.', 'collaborative tasks', 'productivity autonomous', 'mechanical engineering robotics', 'challenges ai', 'challenges pathfinderchallenges', 'autonomy building', 'pathfinder challenges', 'ai automation', 'machine automation', 'education urban space / traffic)', 'road engineering', 'robotics housing', 'construction management', 'detector rd', 'cognitive processes work', 'service robotics', 'multi-agent systems', 'construction environments', 'automation autonomy', 'eco-design', 'optimization algorithms', 'architecture', 'algorithm optimization', 'blocks challenges', 'towards autonomous', 'collaborative field', 'tasks dynamic', 'building information modeling', 'modular nrmm', 'housing infrastructure', 'mechanical equipment', 'dynamic unstructured', 'flexible work management', 'robotics service', 'robotic engineering', 'robotic technology', 'robotic collaboration', 'recommendation systems', 'highway equipment', 'robot collectives', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'smart infrastructure', 'structural engineering', 'collectives construction', 'new buildins historical environments', 'global collaboration', 'nrmm non', 'autonomous robot', 'educational buildings', 'dynamical systems', 'pathfinder pathfinder', 'ngo', 'automation', 'structural engineering design', 'nuclear fusion', 'delivering collaborative', 'zero emission', 'robotics', 'mechanical engineering collaboration', 'environments eic', 'productivity', 'social constructionism', 'equipment pathfinder', 'environmental engineering', 'building building', 'road mobile', 'space collaboration', 'mobile applications', 'dynamic systems', 'tunnel engineering', 'dynamic', 'energy efficiency', 'machinery highway', 'pathfinderchallenges productivity', 'industrial robotics', 'blockchain', 'metaheuristic approaches', 'non road', 'artificial intelligence', 'evolutionary computing', 'robotics design', 'collective identities', 'collective bargaining models', 'transportation planning', 'construction robotics', 'artificial ecosystems', 'autonomous collectives', 'robotic services', 'eic pathfinder', 'building blocks', 'mobilization', ' housing studies', 'unstructured construction', 'metaheuristic algorithms', 'challenges collaborative', 'autonomy development', 'group dynamics', 'algorithm design', 'space coordination', 'mobile machinery', 'collectives delivering', 'infrastructure modular', 'contra', 'space exploration', 'modulators', 'robotic deployment', 'robotics swarm', 'swarm horizoneicpathfinderchallenges']</t>
+          <t>['challenges ai', 'robotic collaboration', 'robotic engineering', 'robotics service', 'robotics swarm', 'global collaboration', 'transportation planning', 'group dynamics', 'dynamic unstructured', 'pathfinderchallenges productivity', 'robotic services', 'ai automation', 'evolutionary computing', 'artificial ecosystems', 'robotics', 'construction management', 'equipment pathfinder', 'autonomous robot', 'recommendation systems', 'collective identities', 'building information modeling', 'robotic deployment', 'metaheuristic approaches', 'road mobile', 'social constructionism', 'educational buildings', 'multi-agent systems', 'ngo', 'mobile applications', ' housing studies', 'tunnel engineering', 'building blocks', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'robotics design', 'autonomous collectives', 'autonomy building', 'industrial robotics', 'contra', 'artificial intelligence', 'eic pathfinder', 'mobile machinery', 'swarm horizoneicpathfinderchallenges', 'service robotics', 'mechanical engineering collaboration', 'construction environments', 'architecture', 'space collaboration', 'building building', 'flexible work management', 'algorithm design', 'robotics housing', 'challenges pathfinderchallenges', 'nrmm non', 'unstructured construction', 'mechanical devices', 'towards autonomous', 'space coordination', 'dynamical systems', 'machinery highway', 'highway equipment', 'mechanical engineering robotics', 'modulators', 'algorithm optimization', 'smart infrastructure', 'housing infrastructure', 'zero emission', 'cognitive processes work', 'environmental engineering', 'detector rd', 'tasks dynamic', 'robotic technology', 'mobilization', 'challenges collaborative', 'robot collectives', 'machine automation', 'environments eic', 'structural engineering design', 'nuclear fusion', 'education urban space / traffic)', 'road engineering', 'space infrastructure', 'automation', 'blocks challenges', 'architectural geometry.', 'energy efficiency', 'pathfinder pathfinder', 'collectives delivering', 'metaheuristic algorithms', 'space exploration', 'blockchain', 'modular nrmm', 'automation autonomy', 'collaborative tasks', 'collective bargaining models', 'infrastructure modular', 'new buildins historical environments', 'productivity', 'productivity autonomous', 'mechanical equipment', 'collectives construction', 'collaborative field', 'optimization algorithms', 'autonomy development', 'non road', 'eco-design', 'structural engineering', 'construction robotics', 'delivering collaborative', 'pathfinder challenges', 'dynamic systems', 'field robotics', 'dynamic']</t>
         </is>
       </c>
     </row>
@@ -4753,7 +4753,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>['tumor growth', 'medical diagnosis', 'eic pathfinder', 'data horizoneicpathfinderchallenges', 'medical research', 'learning difficulties', 'nursing image', 'data acquisition', 'medical data analytics', 'graphic representation', 'robotics', 'data collection', 'revolutionize medical', 'challenges challenges', 'cancer eic', 'challenges pathfinder', 'healthcare technology', 'clinical applications', 'medical history', 'metaheuristic algorithms', 'generative algorithms', 'cancer biochemistry', 'pathfinderchallenges cancer', 'health diagnostics', 'data wrangling', 'challenges pathfinderchallenges', 'medical devices', 'pathfinder challenges', 'tumor biomarkers', 'algorithm design', 'space coordination', 'medical data', 'competitive strategies', 'generativeai based', 'metaheuristic approaches', 'generativeai medical', 'biological agents', 'based agents', 'agents revolutionize', 'unsupervised learning', 'artificial intelligence', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'medical imaging', 'space exploration', 'health informatics', 'tumor development', 'breast cancer', 'treatment cancer', 'diagnosis treatment', 'multi-agent systems', 'clinical diagnostics', 'optimization algorithms', 'artificial ecosystems', 'strategy', 'pathfinder pathfinder', 'cancer generativeai', 'algorithm optimization']</t>
+          <t>['medical history', 'metaheuristic algorithms', 'space exploration', 'generativeai medical', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'space coordination', 'cancer generativeai', 'biological agents', 'medical devices', 'tumor biomarkers', 'data wrangling', 'data acquisition', 'challenges challenges', 'algorithm optimization', 'medical diagnosis', 'health informatics', 'diagnosis treatment', 'artificial intelligence', 'data collection', 'eic pathfinder', 'strategy', 'health diagnostics', 'agents revolutionize', 'cancer eic', 'artificial ecosystems', 'optimization algorithms', 'learning difficulties', 'unsupervised learning', 'tumor growth', 'robotics', 'nursing image', 'data horizoneicpathfinderchallenges', 'challenges pathfinder', 'algorithm design', 'based agents', 'pathfinderchallenges cancer', 'revolutionize medical', 'medical data', 'challenges pathfinderchallenges', 'healthcare technology', 'clinical applications', 'treatment cancer', 'generative algorithms', 'metaheuristic approaches', 'competitive strategies', 'tumor development', 'pathfinder challenges', 'clinical diagnostics', 'medical imaging', 'medical research', 'generativeai based', 'cancer biochemistry', 'medical data analytics', 'multi-agent systems', 'graphic representation', 'pathfinder pathfinder', 'breast cancer']</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>['pathfinderchallenges biomanufacturing', 'eic pathfinder', 'deep ecology', 'robotics', 'biomanufacturing eic', 'biotechnology', 'biotechnological applications', 'challenges pathfinder', 'climate adaptation', 'metaheuristic algorithms', 'plantbased horizoneicpathfinderchallenges', 'ecological resilience', 'bioengineering technologies', 'challenges pathfinderchallenges', 'crops plantbased', 'pathfinder challenges', 'algorithm design', 'space coordination', 'biotechnological research', 'precision agriculture', 'metaheuristic approaches', 'biomanufacturing plantbased', 'plantbased biomanufacturing', 'sustainable agriculture', 'resilient crops', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'space exploration', 'climate resilient', 'seasonal agricultural work', 'bioengineering', 'biotech industry', 'resilience', 'optimization algorithms', 'bioengineering solutions', 'artificial ecosystems', 'pathfinder pathfinder', 'biotech climate', 'algorithm optimization']</t>
+          <t>['metaheuristic algorithms', 'biomanufacturing eic', 'space exploration', 'seasonal agricultural work', 'horizoneicpathfinderchallenges horizoneicpathfinderchallenges', 'space coordination', 'biomanufacturing plantbased', 'plantbased horizoneicpathfinderchallenges', 'climate adaptation', 'biotech climate', 'algorithm optimization', 'biotechnology', 'eic pathfinder', 'bioengineering', 'optimization algorithms', 'artificial ecosystems', 'plantbased biomanufacturing', 'deep ecology', 'robotics', 'sustainable agriculture', 'ecological resilience', 'challenges pathfinder', 'algorithm design', 'metaheuristic approaches', 'resilient crops', 'challenges pathfinderchallenges', 'biotech industry', 'bioengineering technologies', 'pathfinderchallenges biomanufacturing', 'climate resilient', 'crops plantbased', 'biotechnological research', 'pathfinder challenges', 'precision agriculture', 'bioengineering solutions', 'biotechnological applications', 'resilience', 'pathfinder pathfinder']</t>
         </is>
       </c>
     </row>
@@ -4827,7 +4827,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>['new media (technologies)', 'galactic astronomy', 'fellowships horizonwideratalents', 'technology', 'robotic innovation', 'digital humanities', 'biotechnology innovation', 'universitycivil society relations', 'astrobiology', 'fellowships era', 'philosophy social sciences', 'change innovation.', 'black hole physics', 'widening countries', 'international organizations', 'innovation technology', 'horizonwideratalents horizonwideratalents', 'globalization', 'space support', 'therapeutic alliance', 'global collaboration', 'era fellowships', 'ri innovation', 'international development', 'technology widening', 'boundary layer)', 'horizonwideratalents ri']</t>
+          <t>['fellowships horizonwideratalents', 'robotic innovation', 'ri innovation', 'philosophy social sciences', 'fellowships era', 'global collaboration', 'horizonwideratalents ri', 'universitycivil society relations', 'international organizations', 'technology widening', 'change innovation.', 'horizonwideratalents horizonwideratalents', 'new media (technologies)', 'space support', 'globalization', 'international development', 'therapeutic alliance', 'widening countries', 'innovation technology', 'astrobiology', 'galactic astronomy', 'biotechnology innovation', 'digital humanities', 'boundary layer)', 'technology', 'era fellowships', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>['storytelling', 'aircraft systems', 'internet governance', 'ngi taler', 'ia ngi', 'libre electronic', 'electronic commerce', 'africa', 'digital culture', 'freedom association', 'generation internet', 'energy storage', 'internet things', 'aviation', 'children', 'open data', 'open call', 'anonymous libre', 'internet of things', 'taxable anonymous', 'teleworking', 'digital media children', 'pilots next', 'tax law', 'taler open', 'open banking', 'electronic reserves', 'digital electronics', 'social media', 'lgbti', 'electronic devices', 'internet ia', 'tax laws', 'mythology', 'privacy', 'aviation management', 'call taxable', 'demographic change', 'taxation', 'next generation', 'ngo', 'electronic circuits']</t>
+          <t>['electronic circuits', 'africa', 'ngi taler', 'digital electronics', 'anonymous libre', 'taxation', 'electronic devices', 'taler open', 'aircraft systems', 'aviation', 'privacy', 'open call', 'social media', 'storytelling', 'internet things', 'pilots next', 'electronic commerce', 'demographic change', 'electronic reserves', 'internet ia', 'teleworking', 'digital culture', 'taxable anonymous', 'tax law', 'libre electronic', 'tax laws', 'ia ngi', 'lgbti', 'generation internet', 'freedom association', 'next generation', 'aviation management', 'internet of things', 'open data', 'mythology', 'energy storage', 'open banking', 'internet governance', 'digital media children', 'ngo', 'children', 'call taxable']</t>
         </is>
       </c>
     </row>
@@ -4901,7 +4901,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>['hinfinity control', 'transnational adaptations', 'horizonmscapf phd', 'higher education', 'communication consultancy', 'robotic innovation', 'digital humanities', 'fellowships msca', 'social media innovation', 'interdisciplinary mobility', 'clinical psychology', 'msca postdoctoral', 'space collaboration', 'space consulting', 'postdoctoral ri', 'change innovation.', 'ri interdisciplinary', 'education urban space / traffic)', 'sociology.', 'intersectional inequalities', 'fellowships horizonmscapf', 'community studies', 'accreditation', 'sponsorship management', 'therapeutic alliance', 'horizonmscapf horizonmscapf', 'postdoc postdoctoral', 'transportation planning', 'mobility innovation', 'postdoctoral fellowships', 'phd doctoral', 'einstein finsler metrics', 'doctoral postdoc']</t>
+          <t>['msca postdoctoral', 'robotic innovation', 'communication consultancy', 'phd doctoral', 'clinical psychology', 'higher education', 'horizonmscapf horizonmscapf', 'space consulting', 'transportation planning', 'einstein finsler metrics', 'change innovation.', 'horizonmscapf phd', 'community studies', 'mobility innovation', 'accreditation', 'social media innovation', 'therapeutic alliance', 'hinfinity control', 'intersectional inequalities', 'doctoral postdoc', 'space collaboration', 'postdoctoral ri', 'interdisciplinary mobility', 'fellowships horizonmscapf', 'digital humanities', 'transnational adaptations', 'fellowships msca', 'education urban space / traffic)', 'postdoc postdoctoral', 'postdoctoral fellowships', 'ri interdisciplinary', 'sponsorship management', 'sociology.']</t>
         </is>
       </c>
     </row>
@@ -4938,7 +4938,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>['engineering systems', 'security services', 'g smart', 'systems engineering', 'space communication', 'data security', 'horizonjusnsstreamb horizonjusns', 'trust service provider', 'smart systems', 'space services', 'mechanical engineering communication', 'cyber security', 'cybersecurity', 'astrobiology', 'social services', 'horizonjusns g', 'networks services', 'communication systems', 'black hole physics', 'artifical intelligence', 'services sns', 'network analysis', 'communication', 'smart city', 'cyber intelligence', 'smart networks', 'horizonjusns communication', 'security security', 'communication engineering', 'sensor networks', 'systems telecommunications', 'digital services', 'smart infrastructure', 'concordat', 'smart security', 'services horizonjusns', 'digital systems', 'dark matter', 'sns horizonjusnsstreamb', 'mechanical engineering systems', 'electronic communications systems']</t>
+          <t>['trust service provider', 'networks services', 'cyber security', 'smart systems', 'horizonjusns g', 'communication engineering', 'smart networks', 'communication systems', 'artifical intelligence', 'smart infrastructure', 'sensor networks', 'smart security', 'mechanical engineering communication', 'space communication', 'engineering systems', 'electronic communications systems', 'horizonjusnsstreamb horizonjusns', 'cybersecurity', 'communication', 'sns horizonjusnsstreamb', 'social services', 'astrobiology', 'mechanical engineering systems', 'security services', 'services horizonjusns', 'cyber intelligence', 'horizonjusns communication', 'security security', 'digital services', 'network analysis', 'systems engineering', 'data security', 'space services', 'smart city', 'concordat', 'systems telecommunications', 'digital systems', 'dark matter', 'services sns', 'g smart', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -4975,7 +4975,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>['iot device', 'engineering systems', 'g smart', 'systems engineering', 'space communication', 'technology', 'horizonjusnsstreamb horizonjusns', 'trust service provider', 'smart systems', 'space services', 'embedded technologies', 'mechanical engineering communication', 'internet things', 'astrobiology', 'social services', 'horizonjusns g', 'networks services', 'internet of things', 'communication systems', 'black hole physics', 'artifical intelligence', 'services sns', 'network analysis', 'communication', 'smart city', 'cyber intelligence', 'smart networks', 'horizonjusns communication', 'communication engineering', 'space exploration technologies', 'sensor networks', 'electronic devices', 'systems telecommunications', 'digital services', 'smart infrastructure', 'device technologies', 'concordat', 'green technologies', 'digital systems', 'dark matter', 'sns horizonjusnsstreamb', 'mechanical engineering systems', 'advanced iot', 'technologies horizonjusns', 'electronic communications systems']</t>
+          <t>['trust service provider', 'networks services', 'smart systems', 'horizonjusns g', 'communication engineering', 'smart networks', 'green technologies', 'communication systems', 'smart infrastructure', 'artifical intelligence', 'sensor networks', 'electronic devices', 'mechanical engineering communication', 'space communication', 'internet things', 'space exploration technologies', 'engineering systems', 'electronic communications systems', 'horizonjusnsstreamb horizonjusns', 'technologies horizonjusns', 'iot device', 'communication', 'sns horizonjusnsstreamb', 'social services', 'astrobiology', 'mechanical engineering systems', 'cyber intelligence', 'horizonjusns communication', 'advanced iot', 'device technologies', 'internet of things', 'digital services', 'network analysis', 'technology', 'smart city', 'space services', 'concordat', 'systems engineering', 'systems telecommunications', 'digital systems', 'embedded technologies', 'dark matter', 'services sns', 'g smart', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -5012,7 +5012,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>['engineering systems', 'g smart', 'systems engineering', 'space communication', 'horizonjusnsstreamb horizonjusns', 'trust service provider', 'smart systems', 'space services', 'mechanical engineering communication', 'alternative dispute resolution - reconciliation', 'astrobiology', 'social services', 'horizonjusns g', 'networks services', 'communication systems', 'black hole physics', 'artifical intelligence', 'services sns', 'network analysis', 'unification german principalities under prussian leadership emergence germany on historical stage', 'communication', 'smart city', 'cyber intelligence', 'smart networks', 'horizonjusns communication', 'conflict resolution', 'g ntntn', 'theory restoration', 'communication engineering', 'sensor networks', 'reputation', 'ntntn unificationintegration', 'systems telecommunications', 'unificationintegration horizonjusns', 'smart infrastructure', 'digital services', 'concordat', 'digital systems', 'dark matter', 'sns horizonjusnsstreamb', 'mechanical engineering systems', 'electronic communications systems', 'current', 'neural network']</t>
+          <t>['conflict resolution', 'trust service provider', 'networks services', 'smart systems', 'horizonjusns g', 'communication engineering', 'alternative dispute resolution - reconciliation', 'smart networks', 'communication systems', 'artifical intelligence', 'smart infrastructure', 'reputation', 'sensor networks', 'unificationintegration horizonjusns', 'mechanical engineering communication', 'space communication', 'engineering systems', 'theory restoration', 'electronic communications systems', 'horizonjusnsstreamb horizonjusns', 'current', 'communication', 'sns horizonjusnsstreamb', 'g ntntn', 'social services', 'ntntn unificationintegration', 'astrobiology', 'mechanical engineering systems', 'cyber intelligence', 'horizonjusns communication', 'unification german principalities under prussian leadership emergence germany on historical stage', 'digital services', 'network analysis', 'neural network', 'systems engineering', 'smart city', 'space services', 'concordat', 'digital systems', 'systems telecommunications', 'dark matter', 'services sns', 'g smart', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -5049,7 +5049,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>['engineering systems', 'microelectromechanical systems', 'g smart', 'composites', 'space communication', 'systems engineering', 'horizonjusnsstreamb horizonjusns', 'trust service provider', 'smart systems', 'space services', 'ui/ux', 'mechanical engineering communication', 'astrobiology', 'social services', 'module fem', 'steel', 'horizonjusns g', 'microelectronic frontend', 'networks services', 'communication systems', 'black hole physics', 'artifical intelligence', 'services sns', 'network analysis', 'communication', 'smart city', 'cyber intelligence', 'fem horizonjusns', 'smart networks', 'horizonjusns communication', 'magnetic mems', 'homicide femicide', 'communication engineering', 'sensor networks', 'frontend module', 'software design', 'systems telecommunications', 'digital services', 'smart infrastructure', 'concordat', 'software', 'digital systems', 'dark matter', 'sns horizonjusnsstreamb', 'mechanical engineering systems', 'modulators', 'electronic communications systems', 'microelectronics', 'mems']</t>
+          <t>['trust service provider', 'networks services', 'software design', 'smart systems', 'microelectronic frontend', 'horizonjusns g', 'communication engineering', 'smart networks', 'communication systems', 'modulators', 'magnetic mems', 'artifical intelligence', 'smart infrastructure', 'sensor networks', 'mechanical engineering communication', 'space communication', 'engineering systems', 'electronic communications systems', 'module fem', 'horizonjusnsstreamb horizonjusns', 'composites', 'communication', 'sns horizonjusnsstreamb', 'social services', 'astrobiology', 'mechanical engineering systems', 'steel', 'frontend module', 'cyber intelligence', 'horizonjusns communication', 'mems', 'fem horizonjusns', 'ui/ux', 'software', 'digital services', 'network analysis', 'microelectronics', 'homicide femicide', 'microelectromechanical systems', 'smart city', 'space services', 'concordat', 'systems engineering', 'systems telecommunications', 'digital systems', 'dark matter', 'services sns', 'g smart', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -5086,7 +5086,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>['hinfinity control', 'engineering systems', 'g smart', 'systems engineering', 'space communication', 'horizonjusnsstreamc horizonjusns', 'space services', 'policy implementation', 'inclusion', 'smart systems', 'service provision', 'provision enablers', 'trust service provider', 'g telco', 'mechanical engineering communication', 'cloud-based systems', 'business capabilities', 'cloud service', 'cloud storage', 'astrobiology', 'social services', 'disabled care)', 'service marketing', 'telemedicine', 'horizonjusns g', 'networks services', 'communication systems', 'teleworking', 'black hole physics', 'services sns', 'artifical intelligence', 'network analysis', 'communication', 'smart city', 'enablers horizonjusns', 'cyber intelligence', 'smart networks', 'horizonjusns communication', 'communication engineering', 'sensor networks', 'systems telecommunications', 'space support', 'smart infrastructure', 'digital services', 'cloud computing', 'concordat', 'sns horizonjusnsstreamc', 'digital systems', 'dark matter', 'mechanical engineering systems', 'telco cloud', 'teleoperation', 'electronic communications systems']</t>
+          <t>['trust service provider', 'networks services', 'sns horizonjusnsstreamc', 'cloud-based systems', 'smart systems', 'telco cloud', 'horizonjusns g', 'communication engineering', 'smart networks', 'communication systems', 'service provision', 'g telco', 'provision enablers', 'artifical intelligence', 'smart infrastructure', 'sensor networks', 'telemedicine', 'mechanical engineering communication', 'inclusion', 'space communication', 'space support', 'cloud storage', 'engineering systems', 'cloud computing', 'electronic communications systems', 'service marketing', 'hinfinity control', 'cloud service', 'communication', 'disabled care)', 'teleworking', 'teleoperation', 'social services', 'astrobiology', 'horizonjusnsstreamc horizonjusns', 'mechanical engineering systems', 'policy implementation', 'cyber intelligence', 'horizonjusns communication', 'business capabilities', 'digital services', 'network analysis', 'systems engineering', 'space services', 'smart city', 'concordat', 'digital systems', 'systems telecommunications', 'dark matter', 'enablers horizonjusns', 'services sns', 'g smart', 'black hole physics']</t>
         </is>
       </c>
     </row>
@@ -5123,7 +5123,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>['engineering systems', 'g smart', 'systems engineering', 'space communication', 'technology', 'horizonjusnsstreamb horizonjusns', 'trust service provider', 'smart systems', 'space services', 'mechanical engineering communication', 'astrobiology', 'social services', 'horizonjusns g', 'networks services', 'communication systems', 'black hole physics', 'artifical intelligence', 'services sns', 'network analysis', 'systems technologies', 'communication', 'smart city', 'cyber intelligence', 'architectural design', 'smart networks', 'horizonjusns communication', 'communication engineering', 'space exploration technologies', 'sensor networks', 'systems telecommunications', 'digital services', 'architectures systems', 'smart infrastructure', 'concordat', 'digital systems', 'green technologies', 'dark matter', 'sns horizonjusnsstreamb', 'mechanical engineering systems', 'electronic communications systems', 'technologies horizonjusns', 'architecture', 'advanced architectures']</t>
+          <t>['architectures systems', 'black hole physics', 'trust service provider', 'networks services', 'smart systems', 'advanced architectures', 'horizonjusns g', 'communication engineering', 'smart networks', 'green technologies', 'communication systems', 'artifical intelligence', 'smart infrastructure', 'sensor networks', 'mechanical engineering communication', 'space communication', 'space exploration technologies', 'engineering systems', 'electronic communications systems', 'horizonjusnsstreamb horizonjusns', 'technologies horizonjusns', 'communication', 'sns horizonjusnsstreamb', 'social services', 'astrobiology', 'architecture', 'mechanical engineering systems', 'cyber intelligence', 'horizonjusns communication', 'digital services', 'network analysis', 'systems technologies', 'systems engineering', 'digital systems', 'technology', 'smart city', 'space services', 'systems telecommunications', 'concordat', 'dark matter', 'services sns', 'g smart', 'architectural design']</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>['engineering systems', 'g smart', 'networks future', 'neural network architecture', 'space communication', 'systems engineering', 'horizonjusnsstreamb horizonjusns', 'trust service provider', 'smart systems', 'space services', 'optical network', 'optical access', 'rocket propulsion', 'mechanical engineering communication', 'architecture g', 'endodontics', 'psychological networks', 'returns education', 'astrobiology', 'social services', 'higher speed', 'horizonjusns g', 'networks services', 'communication systems', 'network analysis', 'black hole physics', 'services sns', 'artifical intelligence', 'endtoend packet', 'communication', 'smart city', 'cyber intelligence', 'architectural design', 'smart networks', 'horizonjusns communication', 'airport access', 'access networks', 'optical mems', 'communication engineering', 'future endtoend', 'sensor networks', 'systems telecommunications', 'digital services', 'smart infrastructure', 'performance', 'concordat', 'speed optical', 'physics', 'packet optical', 'optical fibers', 'optoelectronics', 'network architecture', 'digital systems', 'g horizonjusns', 'sns horizonjusnsstreamb', 'communication protocols', 'dark matter', 'mechanical engineering systems', 'electronic communications systems', 'architecture', ' future work', 'drug delivery']</t>
+          <t>['black hole physics', 'trust service provider', 'networks future', 'networks services', 'access networks', 'drug delivery', 'smart systems', 'neural network architecture', 'architecture g', 'horizonjusns g', 'communication engineering', 'airport access', 'dark matter', 'smart networks', 'communication protocols', 'physics', 'communication systems', 'speed optical', 'artifical intelligence', 'packet optical', 'sensor networks', 'smart infrastructure', 'performance', 'mechanical engineering communication', 'space communication', 'higher speed', 'engineering systems', 'optical fibers', 'rocket propulsion', 'g horizonjusns', 'electronic communications systems', 'horizonjusnsstreamb horizonjusns', 'communication', 'sns horizonjusnsstreamb', 'optical mems', 'psychological networks', 'social services', 'optical network', 'astrobiology', 'architecture', 'mechanical engineering systems', 'optical access', 'cyber intelligence', 'horizonjusns communication', 'endtoend packet', 'returns education', 'endodontics', 'future endtoend', 'digital services', 'network analysis', 'systems engineering', 'smart city', 'concordat', 'space services', 'digital systems', 'systems telecommunications', 'network architecture', 'optoelectronics', ' future work', 'services sns', 'g smart', 'architectural design']</t>
         </is>
       </c>
     </row>
@@ -5197,7 +5197,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>['hinfinity control', 'engineering systems', 'g smart', 'composites', 'space communication', 'systems engineering', 'horizonjusnsstreamb horizonjusns', 'signal processing', 'space services', 'standardisation followuppocs', 'trust service provider', 'wireless sensors', 'communication technologies', 'mechanical engineering communication', 'processing standardisation', 'social media standards tools', 'technologies signal', 'smart netwroks', 'netwroks services', 'astrobiology', 'social services', 'service marketing', 'horizonjusns g', 'followuppocs horizonjusns', 'communication systems', 'black hole physics', 'artifical intelligence', 'services sns', 'communication', 'wireless communication', 'smart city', 'cyber intelligence', 'data preprocessing', 'horizonjusns communication', 'smart grids', 'communication engineering', 'green consensus', 'systems telecommunications', 'wireless technology', 'digitization', 'robotic standards', 'smart infrastructure', 'digital services', 'concordat', 'digital systems', 'dark matter', 'sns horizonjusnsstreamb', 'mechanical engineering systems', 'digital communication', 'electronic communications systems', 'data transformation']</t>
+          <t>['black hole physics', 'trust service provider', 'signal processing', 'horizonjusns g', 'communication engineering', 'wireless technology', 'standardisation followuppocs', 'smart grids', 'artifical intelligence', 'smart infrastructure', 'social media standards tools', 'mechanical engineering communication', 'space communication', 'data transformation', 'engineering systems', 'electronic communications systems', 'horizonjusnsstreamb horizonjusns', 'service marketing', 'hinfinity control', 'composites', 'communication', 'sns horizonjusnsstreamb', 'social services', 'astrobiology', 'digital communication', 'mechanical engineering systems', 'cyber intelligence', 'horizonjusns communication', 'robotic standards', 'technologies signal', 'netwroks services', 'processing standardisation', 'followuppocs horizonjusns', 'digitization', 'green consensus', 'digital services', 'systems engineering', 'smart netwroks', 'smart city', 'data preprocessing', 'space services', 'systems telecommunications', 'concordat', 'digital systems', 'dark matter', 'wireless sensors', 'communication technologies', 'services sns', 'g smart', 'communication systems', 'wireless communication']</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>['robotic services', 'engineering systems', 'g smart', 'systems engineering', 'space communication', 'horizonjusnsstreamb horizonjusns', 'trust service provider', 'space services', 'smart systems', 'reliability', 'mechanical engineering communication', 'services operation', 'astrobiology', 'social services', 'service marketing', 'horizonjusns g', 'networks services', 'communication systems', 'black hole physics', 'artifical intelligence', 'services sns', 'network analysis', 'communication', 'smart city', 'cyber intelligence', 'smart networks', 'horizonjusns communication', 'communication engineering', 'operation horizonjusns', 'sensor networks', 'systems telecommunications', 'digital services', 'smart infrastructure', 'reliable services', 'trust services', 'concordat', 'digital systems', 'dark matter', 'sns horizonjusnsstreamb', 'mechanical engineering systems', 'electronic communications systems']</t>
+          <t>['trust service provider', 'networks services', 'trust services', 'smart systems', 'horizonjusns g', 'communication engineering', 'smart networks', 'communication systems', 'artifical intelligence', 'smart infrastructure', 'sensor networks', 'mechanical engineering communication', 'space communication', 'engineering systems', 'reliable services', 'services operation', 'electronic communications systems', 'robotic services', 'horizonjusnsstreamb horizonjusns', 'service marketing', 'operation horizonjusns', 'communication', 'sns horizonjusnsstreamb', 'social services', 'astrobiology', 'mechanical engineering systems', 'cyber intelligence', 'horizonjusns communication', 'digital services', 'network analysis', 'systems engineering', 'space services', 'reliability', 'smart city', 'concordat', 'systems telecommunications', 'digital systems', 'dark matter', 'services sns', 'g smart', 'black hole physics']</t>
         </is>
       </c>
     </row>

</xml_diff>